<commit_message>
Perbarui struktur organisasi (2026-09-01T06:17:46.749Z)
</commit_message>
<xml_diff>
--- a/data/struktur-organisasi.xlsx
+++ b/data/struktur-organisasi.xlsx
@@ -63909,7 +63909,7 @@
     </row>
     <row r="1669">
       <c r="A1669" t="str">
-        <v>Kmti9yukcofxe</v>
+        <v>Kmti9zgfv26p3</v>
       </c>
       <c r="B1669" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -63947,7 +63947,7 @@
     </row>
     <row r="1670">
       <c r="A1670" t="str">
-        <v>Kmti9yukcfsz7</v>
+        <v>Kmti9zgfvwyrb</v>
       </c>
       <c r="B1670" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -63985,7 +63985,7 @@
     </row>
     <row r="1671">
       <c r="A1671" t="str">
-        <v>Kmti9yukcf9iq</v>
+        <v>Kmti9zgfvtx00</v>
       </c>
       <c r="B1671" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -64023,7 +64023,7 @@
     </row>
     <row r="1672">
       <c r="A1672" t="str">
-        <v>Kmti9yukc58uh</v>
+        <v>Kmti9zgfv4cbb</v>
       </c>
       <c r="B1672" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -64061,7 +64061,7 @@
     </row>
     <row r="1673">
       <c r="A1673" t="str">
-        <v>Kmti9yukcfnao</v>
+        <v>Kmti9zgfv0cd5</v>
       </c>
       <c r="B1673" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -64099,7 +64099,7 @@
     </row>
     <row r="1674">
       <c r="A1674" t="str">
-        <v>Kmti9yukc81rb</v>
+        <v>Kmti9zgfv45ja</v>
       </c>
       <c r="B1674" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64137,7 +64137,7 @@
     </row>
     <row r="1675">
       <c r="A1675" t="str">
-        <v>Kmti9yukcmk5n</v>
+        <v>Kmti9zgfv5dbr</v>
       </c>
       <c r="B1675" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64175,7 +64175,7 @@
     </row>
     <row r="1676">
       <c r="A1676" t="str">
-        <v>Kmti9yukctkgi</v>
+        <v>Kmti9zgfvpxse</v>
       </c>
       <c r="B1676" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -64251,7 +64251,7 @@
     </row>
     <row r="1678">
       <c r="A1678" t="str">
-        <v>Kmti9yukcp0hn</v>
+        <v>Kmti9zgfvuuv7</v>
       </c>
       <c r="B1678" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -64289,7 +64289,7 @@
     </row>
     <row r="1679">
       <c r="A1679" t="str">
-        <v>Kmti9yukcj4fo</v>
+        <v>Kmti9zgfvlrdk</v>
       </c>
       <c r="B1679" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -64327,7 +64327,7 @@
     </row>
     <row r="1680">
       <c r="A1680" t="str">
-        <v>Kmti9yukc4zuf</v>
+        <v>Kmti9zgfvbsli</v>
       </c>
       <c r="B1680" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -64365,7 +64365,7 @@
     </row>
     <row r="1681">
       <c r="A1681" t="str">
-        <v>Kmti9yukczuqw</v>
+        <v>Kmti9zgfv70po</v>
       </c>
       <c r="B1681" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -64403,7 +64403,7 @@
     </row>
     <row r="1682">
       <c r="A1682" t="str">
-        <v>Kmti9yukc8u3w</v>
+        <v>Kmti9zgfveogu</v>
       </c>
       <c r="B1682" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -64441,7 +64441,7 @@
     </row>
     <row r="1683">
       <c r="A1683" t="str">
-        <v>Kmti9yukckfny</v>
+        <v>Kmti9zgfvmgxf</v>
       </c>
       <c r="B1683" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64479,7 +64479,7 @@
     </row>
     <row r="1684">
       <c r="A1684" t="str">
-        <v>Kmti9yukcwern</v>
+        <v>Kmti9zgfvknli</v>
       </c>
       <c r="B1684" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64517,7 +64517,7 @@
     </row>
     <row r="1685">
       <c r="A1685" t="str">
-        <v>Kmti9yukck28r</v>
+        <v>Kmti9zgfvprvh</v>
       </c>
       <c r="B1685" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -64593,7 +64593,7 @@
     </row>
     <row r="1687">
       <c r="A1687" t="str">
-        <v>Kmti9yukcd9l6</v>
+        <v>Kmti9zgfvbb3w</v>
       </c>
       <c r="B1687" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -64631,7 +64631,7 @@
     </row>
     <row r="1688">
       <c r="A1688" t="str">
-        <v>Kmti9yukcrw7k</v>
+        <v>Kmti9zgfvdowe</v>
       </c>
       <c r="B1688" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -64669,7 +64669,7 @@
     </row>
     <row r="1689">
       <c r="A1689" t="str">
-        <v>Kmti9yukc9eg8</v>
+        <v>Kmti9zgfvapml</v>
       </c>
       <c r="B1689" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -64707,7 +64707,7 @@
     </row>
     <row r="1690">
       <c r="A1690" t="str">
-        <v>Kmti9yukckemr</v>
+        <v>Kmti9zgfv6noy</v>
       </c>
       <c r="B1690" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -64745,7 +64745,7 @@
     </row>
     <row r="1691">
       <c r="A1691" t="str">
-        <v>Kmti9yukcky8f</v>
+        <v>Kmti9zgfvsrt3</v>
       </c>
       <c r="B1691" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -64783,7 +64783,7 @@
     </row>
     <row r="1692">
       <c r="A1692" t="str">
-        <v>Kmti9yukc38w9</v>
+        <v>Kmti9zgfv7snw</v>
       </c>
       <c r="B1692" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64821,7 +64821,7 @@
     </row>
     <row r="1693">
       <c r="A1693" t="str">
-        <v>Kmti9yukcyfpi</v>
+        <v>Kmti9zgfvijxf</v>
       </c>
       <c r="B1693" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64859,7 +64859,7 @@
     </row>
     <row r="1694">
       <c r="A1694" t="str">
-        <v>Kmti9yukcourn</v>
+        <v>Kmti9zgfvq82j</v>
       </c>
       <c r="B1694" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -64897,7 +64897,7 @@
     </row>
     <row r="1695">
       <c r="A1695" t="str">
-        <v>Kmti9yukcl2av</v>
+        <v>Kmti9zgfvy2bj</v>
       </c>
       <c r="B1695" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64935,7 +64935,7 @@
     </row>
     <row r="1696">
       <c r="A1696" t="str">
-        <v>Kmti9yukczj03</v>
+        <v>Kmti9zgfv3xh5</v>
       </c>
       <c r="B1696" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64973,7 +64973,7 @@
     </row>
     <row r="1697">
       <c r="A1697" t="str">
-        <v>Kmti9yukc6j0x</v>
+        <v>Kmti9zgfv676s</v>
       </c>
       <c r="B1697" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -65087,7 +65087,7 @@
     </row>
     <row r="1700">
       <c r="A1700" t="str">
-        <v>Kmti9yukc1hrv</v>
+        <v>Kmti9zgfv4f31</v>
       </c>
       <c r="B1700" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -65125,7 +65125,7 @@
     </row>
     <row r="1701">
       <c r="A1701" t="str">
-        <v>Kmti9yukc74ou</v>
+        <v>Kmti9zgfvaki2</v>
       </c>
       <c r="B1701" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -65163,7 +65163,7 @@
     </row>
     <row r="1702">
       <c r="A1702" t="str">
-        <v>Kmti9yukcqe1f</v>
+        <v>Kmti9zgfvljfh</v>
       </c>
       <c r="B1702" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -65201,7 +65201,7 @@
     </row>
     <row r="1703">
       <c r="A1703" t="str">
-        <v>Kmti9yukc1ni9</v>
+        <v>Kmti9zgfvbm7i</v>
       </c>
       <c r="B1703" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -65239,7 +65239,7 @@
     </row>
     <row r="1704">
       <c r="A1704" t="str">
-        <v>Kmti9yukcau4s</v>
+        <v>Kmti9zgfvw9hy</v>
       </c>
       <c r="B1704" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -65277,7 +65277,7 @@
     </row>
     <row r="1705">
       <c r="A1705" t="str">
-        <v>Kmti9yukcz88u</v>
+        <v>Kmti9zgfv2qcb</v>
       </c>
       <c r="B1705" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -65315,7 +65315,7 @@
     </row>
     <row r="1706">
       <c r="A1706" t="str">
-        <v>Kmti9yukctog3</v>
+        <v>Kmti9zgfvd8mh</v>
       </c>
       <c r="B1706" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -65353,7 +65353,7 @@
     </row>
     <row r="1707">
       <c r="A1707" t="str">
-        <v>Kmti9yukc0jz8</v>
+        <v>Kmti9zgfvc9si</v>
       </c>
       <c r="B1707" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -65391,7 +65391,7 @@
     </row>
     <row r="1708">
       <c r="A1708" t="str">
-        <v>Kmti9yukc8mjr</v>
+        <v>Kmti9zgfvawm4</v>
       </c>
       <c r="B1708" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -65429,7 +65429,7 @@
     </row>
     <row r="1709">
       <c r="A1709" t="str">
-        <v>Kmti9yukc0x73</v>
+        <v>Kmti9zgfvu4kv</v>
       </c>
       <c r="B1709" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -65505,7 +65505,7 @@
     </row>
     <row r="1711">
       <c r="A1711" t="str">
-        <v>Kmti9yukchmug</v>
+        <v>Kmti9zgfvn91l</v>
       </c>
       <c r="B1711" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -65543,7 +65543,7 @@
     </row>
     <row r="1712">
       <c r="A1712" t="str">
-        <v>Kmti9yukce7ib</v>
+        <v>Kmti9zgfvy7ll</v>
       </c>
       <c r="B1712" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -65581,7 +65581,7 @@
     </row>
     <row r="1713">
       <c r="A1713" t="str">
-        <v>Kmti9yukcwch7</v>
+        <v>Kmti9zgfv3bkw</v>
       </c>
       <c r="B1713" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -65619,7 +65619,7 @@
     </row>
     <row r="1714">
       <c r="A1714" t="str">
-        <v>Kmti9yukd5n45</v>
+        <v>Kmti9zgfvk58c</v>
       </c>
       <c r="B1714" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -65657,7 +65657,7 @@
     </row>
     <row r="1715">
       <c r="A1715" t="str">
-        <v>Kmti9yukdbjt6</v>
+        <v>Kmti9zgfvg5e1</v>
       </c>
       <c r="B1715" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -65695,7 +65695,7 @@
     </row>
     <row r="1716">
       <c r="A1716" t="str">
-        <v>Kmti9yukd8bkx</v>
+        <v>Kmti9zgfvk469</v>
       </c>
       <c r="B1716" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -65733,7 +65733,7 @@
     </row>
     <row r="1717">
       <c r="A1717" t="str">
-        <v>Kmti9yukdr5rn</v>
+        <v>Kmti9zgfwkwkh</v>
       </c>
       <c r="B1717" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -65771,7 +65771,7 @@
     </row>
     <row r="1718">
       <c r="A1718" t="str">
-        <v>Kmti9yukd68w6</v>
+        <v>Kmti9zgfwsx0u</v>
       </c>
       <c r="B1718" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -65847,7 +65847,7 @@
     </row>
     <row r="1720">
       <c r="A1720" t="str">
-        <v>Kmti9yukdttf6</v>
+        <v>Kmti9zgfwr6bz</v>
       </c>
       <c r="B1720" t="str">
         <v>Penata Layanan Operasional</v>
@@ -65885,7 +65885,7 @@
     </row>
     <row r="1721">
       <c r="A1721" t="str">
-        <v>Kmti9yukdsgax</v>
+        <v>Kmti9zgfwgsxa</v>
       </c>
       <c r="B1721" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -65923,7 +65923,7 @@
     </row>
     <row r="1722">
       <c r="A1722" t="str">
-        <v>Kmti9yukd1eo1</v>
+        <v>Kmti9zgfw4dul</v>
       </c>
       <c r="B1722" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -65961,7 +65961,7 @@
     </row>
     <row r="1723">
       <c r="A1723" t="str">
-        <v>Kmti9yukdbiv0</v>
+        <v>Kmti9zgfwowkd</v>
       </c>
       <c r="B1723" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -65999,7 +65999,7 @@
     </row>
     <row r="1724">
       <c r="A1724" t="str">
-        <v>Kmti9yukdtdrn</v>
+        <v>Kmti9zgfwsb26</v>
       </c>
       <c r="B1724" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -66037,7 +66037,7 @@
     </row>
     <row r="1725">
       <c r="A1725" t="str">
-        <v>Kmti9yukd3t41</v>
+        <v>Kmti9zgfwaza4</v>
       </c>
       <c r="B1725" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -66075,7 +66075,7 @@
     </row>
     <row r="1726">
       <c r="A1726" t="str">
-        <v>Kmti9yukd5ff9</v>
+        <v>Kmti9zgfwure0</v>
       </c>
       <c r="B1726" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -66113,7 +66113,7 @@
     </row>
     <row r="1727">
       <c r="A1727" t="str">
-        <v>Kmti9yukd5ywk</v>
+        <v>Kmti9zgfwsb5n</v>
       </c>
       <c r="B1727" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -66189,7 +66189,7 @@
     </row>
     <row r="1729">
       <c r="A1729" t="str">
-        <v>Kmti9yukd1qen</v>
+        <v>Kmti9zgfw36rk</v>
       </c>
       <c r="B1729" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -66227,7 +66227,7 @@
     </row>
     <row r="1730">
       <c r="A1730" t="str">
-        <v>Kmti9yukdt9eg</v>
+        <v>Kmti9zgfw3xp6</v>
       </c>
       <c r="B1730" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -66265,7 +66265,7 @@
     </row>
     <row r="1731">
       <c r="A1731" t="str">
-        <v>Kmti9yukdd73v</v>
+        <v>Kmti9zgfwfvik</v>
       </c>
       <c r="B1731" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -66303,7 +66303,7 @@
     </row>
     <row r="1732">
       <c r="A1732" t="str">
-        <v>Kmti9yukdmgrp</v>
+        <v>Kmti9zgfw4593</v>
       </c>
       <c r="B1732" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -66341,7 +66341,7 @@
     </row>
     <row r="1733">
       <c r="A1733" t="str">
-        <v>Kmti9yukd38cl</v>
+        <v>Kmti9zgfw4kki</v>
       </c>
       <c r="B1733" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -66379,7 +66379,7 @@
     </row>
     <row r="1734">
       <c r="A1734" t="str">
-        <v>Kmti9yukd6vj8</v>
+        <v>Kmti9zgfw72q9</v>
       </c>
       <c r="B1734" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -66417,7 +66417,7 @@
     </row>
     <row r="1735">
       <c r="A1735" t="str">
-        <v>Kmti9yukdcc39</v>
+        <v>Kmti9zgfw0hmg</v>
       </c>
       <c r="B1735" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -66455,7 +66455,7 @@
     </row>
     <row r="1736">
       <c r="A1736" t="str">
-        <v>Kmti9yukd2qa4</v>
+        <v>Kmti9zgfw9jf7</v>
       </c>
       <c r="B1736" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -66493,7 +66493,7 @@
     </row>
     <row r="1737">
       <c r="A1737" t="str">
-        <v>Kmti9yukdn227</v>
+        <v>Kmti9zgfw4y3j</v>
       </c>
       <c r="B1737" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -66531,7 +66531,7 @@
     </row>
     <row r="1738">
       <c r="A1738" t="str">
-        <v>Kmti9yukdtavb</v>
+        <v>Kmti9zgfwto78</v>
       </c>
       <c r="B1738" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -66569,7 +66569,7 @@
     </row>
     <row r="1739">
       <c r="A1739" t="str">
-        <v>Kmti9yukd06ri</v>
+        <v>Kmti9zgfw6xgk</v>
       </c>
       <c r="B1739" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -66607,7 +66607,7 @@
     </row>
     <row r="1740">
       <c r="A1740" t="str">
-        <v>Kmti9yukd69i6</v>
+        <v>Kmti9zgfw57jm</v>
       </c>
       <c r="B1740" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -66645,7 +66645,7 @@
     </row>
     <row r="1741">
       <c r="A1741" t="str">
-        <v>Kmti9yukdfab6</v>
+        <v>Kmti9zgfwlksp</v>
       </c>
       <c r="B1741" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -66683,7 +66683,7 @@
     </row>
     <row r="1742">
       <c r="A1742" t="str">
-        <v>Kmti9yukdmc22</v>
+        <v>Kmti9zgfwiets</v>
       </c>
       <c r="B1742" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -66721,7 +66721,7 @@
     </row>
     <row r="1743">
       <c r="A1743" t="str">
-        <v>Kmti9yukdamse</v>
+        <v>Kmti9zgfwmd71</v>
       </c>
       <c r="B1743" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -66835,7 +66835,7 @@
     </row>
     <row r="1746">
       <c r="A1746" t="str">
-        <v>Kmti9yukduryf</v>
+        <v>Kmti9zgfwph3s</v>
       </c>
       <c r="B1746" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -66873,7 +66873,7 @@
     </row>
     <row r="1747">
       <c r="A1747" t="str">
-        <v>Kmti9yukdo9fp</v>
+        <v>Kmti9zgfwkppc</v>
       </c>
       <c r="B1747" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -66911,7 +66911,7 @@
     </row>
     <row r="1748">
       <c r="A1748" t="str">
-        <v>Kmti9yukdl6ik</v>
+        <v>Kmti9zgfw0cxv</v>
       </c>
       <c r="B1748" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -66949,7 +66949,7 @@
     </row>
     <row r="1749" xml:space="preserve">
       <c r="A1749" t="str">
-        <v>Kmti9yukdfnw9</v>
+        <v>Kmti9zgfw6ykh</v>
       </c>
       <c r="B1749" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -66988,7 +66988,7 @@
     </row>
     <row r="1750">
       <c r="A1750" t="str">
-        <v>Kmti9yukdhnmb</v>
+        <v>Kmti9zgfwrkt3</v>
       </c>
       <c r="B1750" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -67064,7 +67064,7 @@
     </row>
     <row r="1752">
       <c r="A1752" t="str">
-        <v>Kmti9yukdnord</v>
+        <v>Kmti9zgfw2txy</v>
       </c>
       <c r="B1752" t="str">
         <v>Penata Layanan Operasional</v>
@@ -67102,7 +67102,7 @@
     </row>
     <row r="1753">
       <c r="A1753" t="str">
-        <v>Kmti9yukdayap</v>
+        <v>Kmti9zgfw3olu</v>
       </c>
       <c r="B1753" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -67140,7 +67140,7 @@
     </row>
     <row r="1754">
       <c r="A1754" t="str">
-        <v>Kmti9yukdzmt5</v>
+        <v>Kmti9zgfwyrgw</v>
       </c>
       <c r="B1754" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -67178,7 +67178,7 @@
     </row>
     <row r="1755" xml:space="preserve">
       <c r="A1755" t="str">
-        <v>Kmti9yukdt06d</v>
+        <v>Kmti9zgfw5xjt</v>
       </c>
       <c r="B1755" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -67217,7 +67217,7 @@
     </row>
     <row r="1756" xml:space="preserve">
       <c r="A1756" t="str">
-        <v>Kmti9yukd7zza</v>
+        <v>Kmti9zgfwukt5</v>
       </c>
       <c r="B1756" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -67256,7 +67256,7 @@
     </row>
     <row r="1757">
       <c r="A1757" t="str">
-        <v>Kmti9yukdua60</v>
+        <v>Kmti9zgfwffgf</v>
       </c>
       <c r="B1757" t="str">
         <v>Pranata Keuangan APBN Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -67294,7 +67294,7 @@
     </row>
     <row r="1758" xml:space="preserve">
       <c r="A1758" t="str">
-        <v>Kmti9yukd6m0x</v>
+        <v>Kmti9zgfwfrt0</v>
       </c>
       <c r="B1758" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Mahir/_x000d_
@@ -67333,7 +67333,7 @@
     </row>
     <row r="1759" xml:space="preserve">
       <c r="A1759" t="str">
-        <v>Kmti9yukdhaia</v>
+        <v>Kmti9zgfwqx35</v>
       </c>
       <c r="B1759" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Terampil/_x000d_
@@ -67410,7 +67410,7 @@
     </row>
     <row r="1761">
       <c r="A1761" t="str">
-        <v>Kmti9yukdotfj</v>
+        <v>Kmti9zgfwp79t</v>
       </c>
       <c r="B1761" t="str">
         <v>Penata Layanan Operasional</v>
@@ -67448,7 +67448,7 @@
     </row>
     <row r="1762">
       <c r="A1762" t="str">
-        <v>Kmti9yukdqwgc</v>
+        <v>Kmti9zgfw5w0d</v>
       </c>
       <c r="B1762" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -67486,7 +67486,7 @@
     </row>
     <row r="1763">
       <c r="A1763" t="str">
-        <v>Kmti9yukd9fk0</v>
+        <v>Kmti9zgfwwc7b</v>
       </c>
       <c r="B1763" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -67524,7 +67524,7 @@
     </row>
     <row r="1764" xml:space="preserve">
       <c r="A1764" t="str">
-        <v>Kmti9yukd876c</v>
+        <v>Kmti9zgfwgmis</v>
       </c>
       <c r="B1764" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -67563,7 +67563,7 @@
     </row>
     <row r="1765" xml:space="preserve">
       <c r="A1765" t="str">
-        <v>Kmti9yukdhsac</v>
+        <v>Kmti9zgfwqfcn</v>
       </c>
       <c r="B1765" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -67602,7 +67602,7 @@
     </row>
     <row r="1766">
       <c r="A1766" t="str">
-        <v>Kmti9yukdd1hm</v>
+        <v>Kmti9zgfw8fwd</v>
       </c>
       <c r="B1766" t="str">
         <v>Pranata Keuangan APBN Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -67640,7 +67640,7 @@
     </row>
     <row r="1767" xml:space="preserve">
       <c r="A1767" t="str">
-        <v>Kmti9yukdfk38</v>
+        <v>Kmti9zgfw3a03</v>
       </c>
       <c r="B1767" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Mahir/_x000d_
@@ -67679,7 +67679,7 @@
     </row>
     <row r="1768" xml:space="preserve">
       <c r="A1768" t="str">
-        <v>Kmti9yukdeysi</v>
+        <v>Kmti9zgfwnd9w</v>
       </c>
       <c r="B1768" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Terampil/_x000d_
@@ -67718,7 +67718,7 @@
     </row>
     <row r="1769">
       <c r="A1769" t="str">
-        <v>Kmti9yukd6dko</v>
+        <v>Kmti9zgfwg7p6</v>
       </c>
       <c r="B1769" t="str">
         <v>Analis Anggaran Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -67756,7 +67756,7 @@
     </row>
     <row r="1770">
       <c r="A1770" t="str">
-        <v>Kmti9yukdrkj3</v>
+        <v>Kmti9zgfwlxww</v>
       </c>
       <c r="B1770" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -67794,7 +67794,7 @@
     </row>
     <row r="1771">
       <c r="A1771" t="str">
-        <v>Kmti9yukdg2zo</v>
+        <v>Kmti9zgfweso7</v>
       </c>
       <c r="B1771" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Madya/Pengawas Keuangan Negara Ahli Madya</v>
@@ -67832,7 +67832,7 @@
     </row>
     <row r="1772">
       <c r="A1772" t="str">
-        <v>Kmti9yukd5qt2</v>
+        <v>Kmti9zgfwya1b</v>
       </c>
       <c r="B1772" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Muda/Pengawas Keuangan Negara Ahli Ahli Muda</v>
@@ -67870,7 +67870,7 @@
     </row>
     <row r="1773">
       <c r="A1773" t="str">
-        <v>Kmti9yukdb432</v>
+        <v>Kmti9zgfwol0w</v>
       </c>
       <c r="B1773" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Pertama/Pengawas Keuangan Negara Ahli Pertama</v>
@@ -67908,7 +67908,7 @@
     </row>
     <row r="1774">
       <c r="A1774" t="str">
-        <v>Kmti9yukdvcur</v>
+        <v>Kmti9zgfw4mzw</v>
       </c>
       <c r="B1774" t="str">
         <v>Pranata Keuangan APBN Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -67946,7 +67946,7 @@
     </row>
     <row r="1775">
       <c r="A1775" t="str">
-        <v>Kmti9yukdzk8r</v>
+        <v>Kmti9zgfwb5sn</v>
       </c>
       <c r="B1775" t="str">
         <v>Pranata Keuangan APBN Mahir/Pengawas Keuangan Negara Mahir</v>
@@ -67984,7 +67984,7 @@
     </row>
     <row r="1776">
       <c r="A1776" t="str">
-        <v>Kmti9yukdjzl7</v>
+        <v>Kmti9zgfw42g7</v>
       </c>
       <c r="B1776" t="str">
         <v>Pranata Keuangan APBN Terampil/Pengawas Keuangan Negara Terampil</v>
@@ -68098,7 +68098,7 @@
     </row>
     <row r="1779">
       <c r="A1779" t="str">
-        <v>Kmti9yukd2pmd</v>
+        <v>Kmti9zgfwgvaq</v>
       </c>
       <c r="B1779" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68136,7 +68136,7 @@
     </row>
     <row r="1780">
       <c r="A1780" t="str">
-        <v>Kmti9yukdptus</v>
+        <v>Kmti9zgfw117s</v>
       </c>
       <c r="B1780" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -68174,7 +68174,7 @@
     </row>
     <row r="1781">
       <c r="A1781" t="str">
-        <v>Kmti9yukd1j09</v>
+        <v>Kmti9zgfwc6hl</v>
       </c>
       <c r="B1781" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -68250,7 +68250,7 @@
     </row>
     <row r="1783">
       <c r="A1783" t="str">
-        <v>Kmti9yukdir23</v>
+        <v>Kmti9zgfwprkg</v>
       </c>
       <c r="B1783" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68288,7 +68288,7 @@
     </row>
     <row r="1784">
       <c r="A1784" t="str">
-        <v>Kmti9yukd7ymh</v>
+        <v>Kmti9zgfwlhys</v>
       </c>
       <c r="B1784" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -68326,7 +68326,7 @@
     </row>
     <row r="1785">
       <c r="A1785" t="str">
-        <v>Kmti9yukd1zh1</v>
+        <v>Kmti9zgfwkuna</v>
       </c>
       <c r="B1785" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -68364,7 +68364,7 @@
     </row>
     <row r="1786">
       <c r="A1786" t="str">
-        <v>Kmti9yukdbv0k</v>
+        <v>Kmti9zgfwluh2</v>
       </c>
       <c r="B1786" t="str">
         <v>Penata Keprotokolan*</v>
@@ -68402,7 +68402,7 @@
     </row>
     <row r="1787">
       <c r="A1787" t="str">
-        <v>Kmti9yukd9si1</v>
+        <v>Kmti9zgfwg7ii</v>
       </c>
       <c r="B1787" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -68440,7 +68440,7 @@
     </row>
     <row r="1788">
       <c r="A1788" t="str">
-        <v>Kmti9yukdlwj5</v>
+        <v>Kmti9zgfwzqqc</v>
       </c>
       <c r="B1788" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -68478,7 +68478,7 @@
     </row>
     <row r="1789">
       <c r="A1789" t="str">
-        <v>Kmti9yukd70ag</v>
+        <v>Kmti9zgfwg8vo</v>
       </c>
       <c r="B1789" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -68516,7 +68516,7 @@
     </row>
     <row r="1790">
       <c r="A1790" t="str">
-        <v>Kmti9yukd5w8m</v>
+        <v>Kmti9zgfw6kia</v>
       </c>
       <c r="B1790" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -68592,7 +68592,7 @@
     </row>
     <row r="1792">
       <c r="A1792" t="str">
-        <v>Kmti9yukd0wrn</v>
+        <v>Kmti9zgfwvs7f</v>
       </c>
       <c r="B1792" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68630,7 +68630,7 @@
     </row>
     <row r="1793">
       <c r="A1793" t="str">
-        <v>Kmti9yukdqmsb</v>
+        <v>Kmti9zgfwinbd</v>
       </c>
       <c r="B1793" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -68668,7 +68668,7 @@
     </row>
     <row r="1794">
       <c r="A1794" t="str">
-        <v>Kmti9yukd0sfv</v>
+        <v>Kmti9zgfwi2a5</v>
       </c>
       <c r="B1794" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -68706,7 +68706,7 @@
     </row>
     <row r="1795">
       <c r="A1795" t="str">
-        <v>Kmti9yukdmve6</v>
+        <v>Kmti9zgfw1s7e</v>
       </c>
       <c r="B1795" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -68744,7 +68744,7 @@
     </row>
     <row r="1796">
       <c r="A1796" t="str">
-        <v>Kmti9yukdl7jm</v>
+        <v>Kmti9zgfwtdxj</v>
       </c>
       <c r="B1796" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -68782,7 +68782,7 @@
     </row>
     <row r="1797">
       <c r="A1797" t="str">
-        <v>Kmti9yukde0xl</v>
+        <v>Kmti9zgfw2ch2</v>
       </c>
       <c r="B1797" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -68820,7 +68820,7 @@
     </row>
     <row r="1798">
       <c r="A1798" t="str">
-        <v>Kmti9yukds4g5</v>
+        <v>Kmti9zgfwp942</v>
       </c>
       <c r="B1798" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -68858,7 +68858,7 @@
     </row>
     <row r="1799">
       <c r="A1799" t="str">
-        <v>Kmti9yukd2c9l</v>
+        <v>Kmti9zgfw2ttx</v>
       </c>
       <c r="B1799" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -68934,7 +68934,7 @@
     </row>
     <row r="1801">
       <c r="A1801" t="str">
-        <v>Kmti9yukdbfr5</v>
+        <v>Kmti9zgfw74gb</v>
       </c>
       <c r="B1801" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68972,7 +68972,7 @@
     </row>
     <row r="1802">
       <c r="A1802" t="str">
-        <v>Kmti9yukdtwzc</v>
+        <v>Kmti9zgfwbjjg</v>
       </c>
       <c r="B1802" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -69010,7 +69010,7 @@
     </row>
     <row r="1803">
       <c r="A1803" t="str">
-        <v>Kmti9yukdtwi5</v>
+        <v>Kmti9zgfwrqwo</v>
       </c>
       <c r="B1803" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -69048,7 +69048,7 @@
     </row>
     <row r="1804">
       <c r="A1804" t="str">
-        <v>Kmti9yukdgvp4</v>
+        <v>Kmti9zgfwhexu</v>
       </c>
       <c r="B1804" t="str">
         <v>Penata Keprotokolan*</v>
@@ -69086,7 +69086,7 @@
     </row>
     <row r="1805">
       <c r="A1805" t="str">
-        <v>Kmti9yukdntuz</v>
+        <v>Kmti9zgfwdna0</v>
       </c>
       <c r="B1805" t="str">
         <v>Arsiparis Ahli Muda</v>
@@ -69124,7 +69124,7 @@
     </row>
     <row r="1806">
       <c r="A1806" t="str">
-        <v>Kmti9yukdtlp0</v>
+        <v>Kmti9zgfwxez5</v>
       </c>
       <c r="B1806" t="str">
         <v>Arsiparis Ahli Pertama</v>
@@ -69162,7 +69162,7 @@
     </row>
     <row r="1807">
       <c r="A1807" t="str">
-        <v>Kmti9yukd7iki</v>
+        <v>Kmti9zgfwy5z6</v>
       </c>
       <c r="B1807" t="str">
         <v>Arsiparis Penyelia</v>
@@ -69200,7 +69200,7 @@
     </row>
     <row r="1808">
       <c r="A1808" t="str">
-        <v>Kmti9yukd7j9j</v>
+        <v>Kmti9zgfw5cy1</v>
       </c>
       <c r="B1808" t="str">
         <v>Arsiparis Mahir</v>
@@ -69238,7 +69238,7 @@
     </row>
     <row r="1809">
       <c r="A1809" t="str">
-        <v>Kmti9yukdsrua</v>
+        <v>Kmti9zgfweff0</v>
       </c>
       <c r="B1809" t="str">
         <v>Arsiparis Terampil</v>
@@ -69276,7 +69276,7 @@
     </row>
     <row r="1810">
       <c r="A1810" t="str">
-        <v>Kmti9yukdu6x7</v>
+        <v>Kmti9zgfwfxcr</v>
       </c>
       <c r="B1810" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -69314,7 +69314,7 @@
     </row>
     <row r="1811">
       <c r="A1811" t="str">
-        <v>Kmti9yukdxuwv</v>
+        <v>Kmti9zgfwj2pm</v>
       </c>
       <c r="B1811" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -69352,7 +69352,7 @@
     </row>
     <row r="1812">
       <c r="A1812" t="str">
-        <v>Kmti9yukdb1tw</v>
+        <v>Kmti9zgfwe8ra</v>
       </c>
       <c r="B1812" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -69390,7 +69390,7 @@
     </row>
     <row r="1813">
       <c r="A1813" t="str">
-        <v>Kmti9yukddvq3</v>
+        <v>Kmti9zgfwaj0c</v>
       </c>
       <c r="B1813" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -69428,7 +69428,7 @@
     </row>
     <row r="1814">
       <c r="A1814" t="str">
-        <v>Kmti9yukdz3ei</v>
+        <v>Kmti9zgfwvo49</v>
       </c>
       <c r="B1814" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -69542,7 +69542,7 @@
     </row>
     <row r="1817">
       <c r="A1817" t="str">
-        <v>Kmti9yukdoadn</v>
+        <v>Kmti9zgfwjqwo</v>
       </c>
       <c r="B1817" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -69580,7 +69580,7 @@
     </row>
     <row r="1818">
       <c r="A1818" t="str">
-        <v>Kmti9yukdaz20</v>
+        <v>Kmti9zgfwem78</v>
       </c>
       <c r="B1818" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -69618,7 +69618,7 @@
     </row>
     <row r="1819">
       <c r="A1819" t="str">
-        <v>Kmti9yukdcd45</v>
+        <v>Kmti9zgfw48hj</v>
       </c>
       <c r="B1819" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -69656,7 +69656,7 @@
     </row>
     <row r="1820">
       <c r="A1820" t="str">
-        <v>Kmti9yukd2xjx</v>
+        <v>Kmti9zgfwyiy6</v>
       </c>
       <c r="B1820" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -69694,7 +69694,7 @@
     </row>
     <row r="1821">
       <c r="A1821" t="str">
-        <v>Kmti9yukdvgf1</v>
+        <v>Kmti9zgfw4rmo</v>
       </c>
       <c r="B1821" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -69732,7 +69732,7 @@
     </row>
     <row r="1822">
       <c r="A1822" t="str">
-        <v>Kmti9yukdz9ez</v>
+        <v>Kmti9zgfwsdmd</v>
       </c>
       <c r="B1822" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -69808,7 +69808,7 @@
     </row>
     <row r="1824">
       <c r="A1824" t="str">
-        <v>Kmti9yukdkg0u</v>
+        <v>Kmti9zgfwhaic</v>
       </c>
       <c r="B1824" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -69846,7 +69846,7 @@
     </row>
     <row r="1825">
       <c r="A1825" t="str">
-        <v>Kmti9yukdiopv</v>
+        <v>Kmti9zgfwz66l</v>
       </c>
       <c r="B1825" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -69884,7 +69884,7 @@
     </row>
     <row r="1826">
       <c r="A1826" t="str">
-        <v>Kmti9yukdum1c</v>
+        <v>Kmti9zgfw2y2o</v>
       </c>
       <c r="B1826" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -69922,7 +69922,7 @@
     </row>
     <row r="1827">
       <c r="A1827" t="str">
-        <v>Kmti9yukd8o94</v>
+        <v>Kmti9zgfwldzg</v>
       </c>
       <c r="B1827" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -69960,7 +69960,7 @@
     </row>
     <row r="1828">
       <c r="A1828" t="str">
-        <v>Kmti9yukdqu4z</v>
+        <v>Kmti9zgfwln2m</v>
       </c>
       <c r="B1828" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -69998,7 +69998,7 @@
     </row>
     <row r="1829">
       <c r="A1829" t="str">
-        <v>Kmti9yukdefhz</v>
+        <v>Kmti9zgfw4fjz</v>
       </c>
       <c r="B1829" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -70036,7 +70036,7 @@
     </row>
     <row r="1830">
       <c r="A1830" t="str">
-        <v>Kmti9yukd7cn7</v>
+        <v>Kmti9zgfwrcj7</v>
       </c>
       <c r="B1830" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -70112,7 +70112,7 @@
     </row>
     <row r="1832">
       <c r="A1832" t="str">
-        <v>Kmti9yukdf082</v>
+        <v>Kmti9zgfwwsyh</v>
       </c>
       <c r="B1832" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -70150,7 +70150,7 @@
     </row>
     <row r="1833">
       <c r="A1833" t="str">
-        <v>Kmti9yukdnr6u</v>
+        <v>Kmti9zgfwtkvi</v>
       </c>
       <c r="B1833" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -70188,7 +70188,7 @@
     </row>
     <row r="1834">
       <c r="A1834" t="str">
-        <v>Kmti9yukd1kb5</v>
+        <v>Kmti9zgfwv418</v>
       </c>
       <c r="B1834" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -70226,7 +70226,7 @@
     </row>
     <row r="1835">
       <c r="A1835" t="str">
-        <v>Kmti9yukdva2t</v>
+        <v>Kmti9zgfw5nyi</v>
       </c>
       <c r="B1835" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -70264,7 +70264,7 @@
     </row>
     <row r="1836">
       <c r="A1836" t="str">
-        <v>Kmti9yukdytm7</v>
+        <v>Kmti9zgfw36v4</v>
       </c>
       <c r="B1836" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -70302,7 +70302,7 @@
     </row>
     <row r="1837">
       <c r="A1837" t="str">
-        <v>Kmti9yukdbeo2</v>
+        <v>Kmti9zgfwrhj9</v>
       </c>
       <c r="B1837" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -70340,7 +70340,7 @@
     </row>
     <row r="1838">
       <c r="A1838" t="str">
-        <v>Kmti9yukdb3wl</v>
+        <v>Kmti9zgfw9p5y</v>
       </c>
       <c r="B1838" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -70378,7 +70378,7 @@
     </row>
     <row r="1839">
       <c r="A1839" t="str">
-        <v>Kmti9yukd4qwr</v>
+        <v>Kmti9zgfw7yh8</v>
       </c>
       <c r="B1839" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -70416,7 +70416,7 @@
     </row>
     <row r="1840">
       <c r="A1840" t="str">
-        <v>Kmti9yukdjmm3</v>
+        <v>Kmti9zgfwytqd</v>
       </c>
       <c r="B1840" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -70454,7 +70454,7 @@
     </row>
     <row r="1841">
       <c r="A1841" t="str">
-        <v>Kmti9yukdpbgy</v>
+        <v>Kmti9zgfwidk1</v>
       </c>
       <c r="B1841" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -70492,7 +70492,7 @@
     </row>
     <row r="1842">
       <c r="A1842" t="str">
-        <v>Kmti9yukdv0ch</v>
+        <v>Kmti9zgfw5qi3</v>
       </c>
       <c r="B1842" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -70568,7 +70568,7 @@
     </row>
     <row r="1844">
       <c r="A1844" t="str">
-        <v>Kmti9yukdhmjh</v>
+        <v>Kmti9zgfw7bm4</v>
       </c>
       <c r="B1844" t="str">
         <v>Penata Layanan Operasional</v>
@@ -70606,7 +70606,7 @@
     </row>
     <row r="1845">
       <c r="A1845" t="str">
-        <v>Kmti9yukdgast</v>
+        <v>Kmti9zgfwsvbt</v>
       </c>
       <c r="B1845" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -70644,7 +70644,7 @@
     </row>
     <row r="1846">
       <c r="A1846" t="str">
-        <v>Kmti9yukd50io</v>
+        <v>Kmti9zgfwg9f7</v>
       </c>
       <c r="B1846" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -70682,7 +70682,7 @@
     </row>
     <row r="1847">
       <c r="A1847" t="str">
-        <v>Kmti9yukdovi3</v>
+        <v>Kmti9zgfwwt6t</v>
       </c>
       <c r="B1847" t="str">
         <v>Pranata Humas Ahli Muda</v>
@@ -70720,7 +70720,7 @@
     </row>
     <row r="1848">
       <c r="A1848" t="str">
-        <v>Kmti9yukdvidh</v>
+        <v>Kmti9zgfwv7iq</v>
       </c>
       <c r="B1848" t="str">
         <v>Pranata Humas Ahli Pertama</v>
@@ -70758,7 +70758,7 @@
     </row>
     <row r="1849">
       <c r="A1849" t="str">
-        <v>Kmti9yukdf8oe</v>
+        <v>Kmti9zgfwdkza</v>
       </c>
       <c r="B1849" t="str">
         <v>Pranata Humas Penyelia</v>
@@ -70796,7 +70796,7 @@
     </row>
     <row r="1850">
       <c r="A1850" t="str">
-        <v>Kmti9yukdw37h</v>
+        <v>Kmti9zgfwko74</v>
       </c>
       <c r="B1850" t="str">
         <v>Pranata Humas Mahir</v>
@@ -70834,7 +70834,7 @@
     </row>
     <row r="1851">
       <c r="A1851" t="str">
-        <v>Kmti9yukdmias</v>
+        <v>Kmti9zgfwifm5</v>
       </c>
       <c r="B1851" t="str">
         <v>Pranata Humas Terampil</v>
@@ -70872,7 +70872,7 @@
     </row>
     <row r="1852">
       <c r="A1852" t="str">
-        <v>Kmti9yukdc4qm</v>
+        <v>Kmti9zgfw8us7</v>
       </c>
       <c r="B1852" t="str">
         <v>Pustakawan Ahli Muda</v>
@@ -70910,7 +70910,7 @@
     </row>
     <row r="1853">
       <c r="A1853" t="str">
-        <v>Kmti9yukdo9vl</v>
+        <v>Kmti9zgfwbumm</v>
       </c>
       <c r="B1853" t="str">
         <v>Pustakawan Ahli Pertama</v>
@@ -70948,7 +70948,7 @@
     </row>
     <row r="1854">
       <c r="A1854" t="str">
-        <v>Kmti9yukdoge2</v>
+        <v>Kmti9zgfw2iij</v>
       </c>
       <c r="B1854" t="str">
         <v>Pustakawan Penyelia</v>
@@ -70986,7 +70986,7 @@
     </row>
     <row r="1855">
       <c r="A1855" t="str">
-        <v>Kmti9yukdodqd</v>
+        <v>Kmti9zgfwyyps</v>
       </c>
       <c r="B1855" t="str">
         <v>Pustakawan Mahir</v>
@@ -71024,7 +71024,7 @@
     </row>
     <row r="1856">
       <c r="A1856" t="str">
-        <v>Kmti9yukdzku7</v>
+        <v>Kmti9zgfwjo3x</v>
       </c>
       <c r="B1856" t="str">
         <v>Pustakawan Terampil</v>
@@ -71138,7 +71138,7 @@
     </row>
     <row r="1859">
       <c r="A1859" t="str">
-        <v>Kmti9yukdf6us</v>
+        <v>Kmti9zgfw0xyq</v>
       </c>
       <c r="B1859" t="str">
         <v>Penata Layanan Operasional</v>
@@ -71176,7 +71176,7 @@
     </row>
     <row r="1860">
       <c r="A1860" t="str">
-        <v>Kmti9yukdzqya</v>
+        <v>Kmti9zgfwe6ho</v>
       </c>
       <c r="B1860" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71214,7 +71214,7 @@
     </row>
     <row r="1861">
       <c r="A1861" t="str">
-        <v>Kmti9yukd1tea</v>
+        <v>Kmti9zgfwfgw6</v>
       </c>
       <c r="B1861" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71252,7 +71252,7 @@
     </row>
     <row r="1862">
       <c r="A1862" t="str">
-        <v>Kmti9yukdnev6</v>
+        <v>Kmti9zgfwla25</v>
       </c>
       <c r="B1862" t="str">
         <v>Penata Keprotokolan*</v>
@@ -71366,7 +71366,7 @@
     </row>
     <row r="1865">
       <c r="A1865" t="str">
-        <v>Kmti9yukd9qe0</v>
+        <v>Kmti9zgfw2nin</v>
       </c>
       <c r="B1865" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -71404,7 +71404,7 @@
     </row>
     <row r="1866">
       <c r="A1866" t="str">
-        <v>Kmti9yukdk4nc</v>
+        <v>Kmti9zgfw7zit</v>
       </c>
       <c r="B1866" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71442,7 +71442,7 @@
     </row>
     <row r="1867">
       <c r="A1867" t="str">
-        <v>Kmti9yukdr0g3</v>
+        <v>Kmti9zgfwii39</v>
       </c>
       <c r="B1867" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71518,7 +71518,7 @@
     </row>
     <row r="1869">
       <c r="A1869" t="str">
-        <v>Kmti9yukd9fw7</v>
+        <v>Kmti9zgfwzuwq</v>
       </c>
       <c r="B1869" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -71556,7 +71556,7 @@
     </row>
     <row r="1870">
       <c r="A1870" t="str">
-        <v>Kmti9yukdij1c</v>
+        <v>Kmti9zgfwlnqc</v>
       </c>
       <c r="B1870" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71594,7 +71594,7 @@
     </row>
     <row r="1871">
       <c r="A1871" t="str">
-        <v>Kmti9yukd56qp</v>
+        <v>Kmti9zgfwp5sv</v>
       </c>
       <c r="B1871" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71632,7 +71632,7 @@
     </row>
     <row r="1872" xml:space="preserve">
       <c r="A1872" t="str">
-        <v>Kmti9yukdplf0</v>
+        <v>Kmti9zgfw0ds4</v>
       </c>
       <c r="B1872" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -71671,7 +71671,7 @@
     </row>
     <row r="1873" xml:space="preserve">
       <c r="A1873" t="str">
-        <v>Kmti9yukd35hi</v>
+        <v>Kmti9zgfwa6fc</v>
       </c>
       <c r="B1873" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -71710,7 +71710,7 @@
     </row>
     <row r="1874" xml:space="preserve">
       <c r="A1874" t="str">
-        <v>Kmti9yukd9mox</v>
+        <v>Kmti9zgfwajv1</v>
       </c>
       <c r="B1874" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -71749,7 +71749,7 @@
     </row>
     <row r="1875" xml:space="preserve">
       <c r="A1875" t="str">
-        <v>Kmti9yukd8gtj</v>
+        <v>Kmti9zgfwc10z</v>
       </c>
       <c r="B1875" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -71864,7 +71864,7 @@
     </row>
     <row r="1878">
       <c r="A1878" t="str">
-        <v>Kmti9yukd6ugj</v>
+        <v>Kmti9zgfwygzd</v>
       </c>
       <c r="B1878" t="str">
         <v>Penata Layanan Operasional</v>
@@ -71902,7 +71902,7 @@
     </row>
     <row r="1879">
       <c r="A1879" t="str">
-        <v>Kmti9yukdywdj</v>
+        <v>Kmti9zgfwoltt</v>
       </c>
       <c r="B1879" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71940,7 +71940,7 @@
     </row>
     <row r="1880">
       <c r="A1880" t="str">
-        <v>Kmti9yukdkt2q</v>
+        <v>Kmti9zgfwqkai</v>
       </c>
       <c r="B1880" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71978,7 +71978,7 @@
     </row>
     <row r="1881">
       <c r="A1881" t="str">
-        <v>Kmti9yukd37kp</v>
+        <v>Kmti9zgfwypfl</v>
       </c>
       <c r="B1881" t="str">
         <v>Penata Keprotokolan*</v>
@@ -72092,7 +72092,7 @@
     </row>
     <row r="1884">
       <c r="A1884" t="str">
-        <v>Kmti9yukdr0na</v>
+        <v>Kmti9zgfwhczd</v>
       </c>
       <c r="B1884" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -72130,7 +72130,7 @@
     </row>
     <row r="1885">
       <c r="A1885" t="str">
-        <v>Kmti9yukdj2f6</v>
+        <v>Kmti9zgfw7qoi</v>
       </c>
       <c r="B1885" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72168,7 +72168,7 @@
     </row>
     <row r="1886">
       <c r="A1886" t="str">
-        <v>Kmti9yukdhk60</v>
+        <v>Kmti9zgfwb0ne</v>
       </c>
       <c r="B1886" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72244,7 +72244,7 @@
     </row>
     <row r="1888">
       <c r="A1888" t="str">
-        <v>Kmti9yukddrak</v>
+        <v>Kmti9zgfwonwb</v>
       </c>
       <c r="B1888" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -72282,7 +72282,7 @@
     </row>
     <row r="1889">
       <c r="A1889" t="str">
-        <v>Kmti9yukdsik3</v>
+        <v>Kmti9zgfwmcx1</v>
       </c>
       <c r="B1889" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72320,7 +72320,7 @@
     </row>
     <row r="1890">
       <c r="A1890" t="str">
-        <v>Kmti9yukd4q3k</v>
+        <v>Kmti9zgfwvgey</v>
       </c>
       <c r="B1890" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72358,7 +72358,7 @@
     </row>
     <row r="1891" xml:space="preserve">
       <c r="A1891" t="str">
-        <v>Kmti9yukdbrn8</v>
+        <v>Kmti9zgfwhsjl</v>
       </c>
       <c r="B1891" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -72397,7 +72397,7 @@
     </row>
     <row r="1892" xml:space="preserve">
       <c r="A1892" t="str">
-        <v>Kmti9yukd5h1h</v>
+        <v>Kmti9zgfwz45u</v>
       </c>
       <c r="B1892" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -72436,7 +72436,7 @@
     </row>
     <row r="1893" xml:space="preserve">
       <c r="A1893" t="str">
-        <v>Kmti9yukddzuq</v>
+        <v>Kmti9zgfwkdjf</v>
       </c>
       <c r="B1893" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -72475,7 +72475,7 @@
     </row>
     <row r="1894" xml:space="preserve">
       <c r="A1894" t="str">
-        <v>Kmti9yukdu7z7</v>
+        <v>Kmti9zgfwqky1</v>
       </c>
       <c r="B1894" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -72590,7 +72590,7 @@
     </row>
     <row r="1897">
       <c r="A1897" t="str">
-        <v>Kmti9yukdxyx2</v>
+        <v>Kmti9zgfwdg9m</v>
       </c>
       <c r="B1897" t="str">
         <v>Penata Layanan Operasional</v>
@@ -72628,7 +72628,7 @@
     </row>
     <row r="1898">
       <c r="A1898" t="str">
-        <v>Kmti9yukdjqee</v>
+        <v>Kmti9zgfw93o7</v>
       </c>
       <c r="B1898" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72666,7 +72666,7 @@
     </row>
     <row r="1899">
       <c r="A1899" t="str">
-        <v>Kmti9yukdad06</v>
+        <v>Kmti9zgfw3rvs</v>
       </c>
       <c r="B1899" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72704,7 +72704,7 @@
     </row>
     <row r="1900">
       <c r="A1900" t="str">
-        <v>Kmti9yukdgzir</v>
+        <v>Kmti9zgfwaiyz</v>
       </c>
       <c r="B1900" t="str">
         <v>Penata Keprotokolan*</v>
@@ -72818,7 +72818,7 @@
     </row>
     <row r="1903">
       <c r="A1903" t="str">
-        <v>Kmti9yukdip56</v>
+        <v>Kmti9zgfwqae2</v>
       </c>
       <c r="B1903" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -72856,7 +72856,7 @@
     </row>
     <row r="1904">
       <c r="A1904" t="str">
-        <v>Kmti9yukdlmdu</v>
+        <v>Kmti9zgfwd4z6</v>
       </c>
       <c r="B1904" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72894,7 +72894,7 @@
     </row>
     <row r="1905">
       <c r="A1905" t="str">
-        <v>Kmti9yukdf555</v>
+        <v>Kmti9zgfw2ujl</v>
       </c>
       <c r="B1905" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72970,7 +72970,7 @@
     </row>
     <row r="1907">
       <c r="A1907" t="str">
-        <v>Kmti9yukd7sdf</v>
+        <v>Kmti9zgfw9m04</v>
       </c>
       <c r="B1907" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -73008,7 +73008,7 @@
     </row>
     <row r="1908">
       <c r="A1908" t="str">
-        <v>Kmti9yukd4w3j</v>
+        <v>Kmti9zgfwx768</v>
       </c>
       <c r="B1908" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73046,7 +73046,7 @@
     </row>
     <row r="1909">
       <c r="A1909" t="str">
-        <v>Kmti9yukdyngy</v>
+        <v>Kmti9zgfwvkwj</v>
       </c>
       <c r="B1909" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73084,7 +73084,7 @@
     </row>
     <row r="1910" xml:space="preserve">
       <c r="A1910" t="str">
-        <v>Kmti9yukdftgs</v>
+        <v>Kmti9zgfw6b8v</v>
       </c>
       <c r="B1910" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -73123,7 +73123,7 @@
     </row>
     <row r="1911" xml:space="preserve">
       <c r="A1911" t="str">
-        <v>Kmti9yukdka1c</v>
+        <v>Kmti9zgfwsy1c</v>
       </c>
       <c r="B1911" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -73162,7 +73162,7 @@
     </row>
     <row r="1912" xml:space="preserve">
       <c r="A1912" t="str">
-        <v>Kmti9yukdlgby</v>
+        <v>Kmti9zgfw5kvp</v>
       </c>
       <c r="B1912" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -73201,7 +73201,7 @@
     </row>
     <row r="1913" xml:space="preserve">
       <c r="A1913" t="str">
-        <v>Kmti9yukd65sw</v>
+        <v>Kmti9zgfwz84e</v>
       </c>
       <c r="B1913" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -73316,7 +73316,7 @@
     </row>
     <row r="1916">
       <c r="A1916" t="str">
-        <v>Kmti9yukd3yfq</v>
+        <v>Kmti9zgfwbw3m</v>
       </c>
       <c r="B1916" t="str">
         <v>Penata Layanan Operasional</v>
@@ -73354,7 +73354,7 @@
     </row>
     <row r="1917">
       <c r="A1917" t="str">
-        <v>Kmti9yukd8265</v>
+        <v>Kmti9zgfwkfny</v>
       </c>
       <c r="B1917" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73392,7 +73392,7 @@
     </row>
     <row r="1918">
       <c r="A1918" t="str">
-        <v>Kmti9yukd8vm2</v>
+        <v>Kmti9zgfwcyo6</v>
       </c>
       <c r="B1918" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73430,7 +73430,7 @@
     </row>
     <row r="1919">
       <c r="A1919" t="str">
-        <v>Kmti9yukdf5ep</v>
+        <v>Kmti9zgfw0tnz</v>
       </c>
       <c r="B1919" t="str">
         <v>Penata Keprotokolan*</v>
@@ -73544,7 +73544,7 @@
     </row>
     <row r="1922">
       <c r="A1922" t="str">
-        <v>Kmti9yukdbq33</v>
+        <v>Kmti9zgfwltys</v>
       </c>
       <c r="B1922" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -73582,7 +73582,7 @@
     </row>
     <row r="1923">
       <c r="A1923" t="str">
-        <v>Kmti9yukd63dr</v>
+        <v>Kmti9zgfwlv3o</v>
       </c>
       <c r="B1923" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73620,7 +73620,7 @@
     </row>
     <row r="1924">
       <c r="A1924" t="str">
-        <v>Kmti9yukdzfru</v>
+        <v>Kmti9zgfwjioh</v>
       </c>
       <c r="B1924" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73696,7 +73696,7 @@
     </row>
     <row r="1926">
       <c r="A1926" t="str">
-        <v>Kmti9yukddm3x</v>
+        <v>Kmti9zgfw06pe</v>
       </c>
       <c r="B1926" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -73734,7 +73734,7 @@
     </row>
     <row r="1927">
       <c r="A1927" t="str">
-        <v>Kmti9yukd21x6</v>
+        <v>Kmti9zgfwuj6q</v>
       </c>
       <c r="B1927" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73772,7 +73772,7 @@
     </row>
     <row r="1928">
       <c r="A1928" t="str">
-        <v>Kmti9yukd353p</v>
+        <v>Kmti9zgfw033o</v>
       </c>
       <c r="B1928" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73810,7 +73810,7 @@
     </row>
     <row r="1929" xml:space="preserve">
       <c r="A1929" t="str">
-        <v>Kmti9yukdcr1w</v>
+        <v>Kmti9zgfwjjey</v>
       </c>
       <c r="B1929" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -73849,7 +73849,7 @@
     </row>
     <row r="1930" xml:space="preserve">
       <c r="A1930" t="str">
-        <v>Kmti9yukd9gxi</v>
+        <v>Kmti9zgfwnnpn</v>
       </c>
       <c r="B1930" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -73888,7 +73888,7 @@
     </row>
     <row r="1931" xml:space="preserve">
       <c r="A1931" t="str">
-        <v>Kmti9yukdv3kv</v>
+        <v>Kmti9zgfw6gap</v>
       </c>
       <c r="B1931" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -73927,7 +73927,7 @@
     </row>
     <row r="1932" xml:space="preserve">
       <c r="A1932" t="str">
-        <v>Kmti9yukddphs</v>
+        <v>Kmti9zgfwoabt</v>
       </c>
       <c r="B1932" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -73966,7 +73966,7 @@
     </row>
     <row r="1933" xml:space="preserve">
       <c r="A1933" t="str">
-        <v>Kmti9yukdf4zn</v>
+        <v>Kmti9zgfww5t6</v>
       </c>
       <c r="B1933" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Madya/_x000d_
@@ -74005,7 +74005,7 @@
     </row>
     <row r="1934" xml:space="preserve">
       <c r="A1934" t="str">
-        <v>Kmti9yukdkbj4</v>
+        <v>Kmti9zgfwyfcf</v>
       </c>
       <c r="B1934" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -74044,7 +74044,7 @@
     </row>
     <row r="1935" xml:space="preserve">
       <c r="A1935" t="str">
-        <v>Kmti9yukdhcmi</v>
+        <v>Kmti9zgfw2bzn</v>
       </c>
       <c r="B1935" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -74159,7 +74159,7 @@
     </row>
     <row r="1938">
       <c r="A1938" t="str">
-        <v>Kmti9yukdjz19</v>
+        <v>Kmti9zgfwe6jk</v>
       </c>
       <c r="B1938" t="str">
         <v>Penata Layanan Operasional</v>
@@ -74197,7 +74197,7 @@
     </row>
     <row r="1939">
       <c r="A1939" t="str">
-        <v>Kmti9yukdazvu</v>
+        <v>Kmti9zgfwnr3v</v>
       </c>
       <c r="B1939" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -74235,7 +74235,7 @@
     </row>
     <row r="1940">
       <c r="A1940" t="str">
-        <v>Kmti9yukdh97d</v>
+        <v>Kmti9zgfw1j05</v>
       </c>
       <c r="B1940" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -74273,7 +74273,7 @@
     </row>
     <row r="1941">
       <c r="A1941" t="str">
-        <v>Kmti9yukdg6wa</v>
+        <v>Kmti9zgfw5rbq</v>
       </c>
       <c r="B1941" t="str">
         <v>Penata Keprotokolan*</v>
@@ -74387,7 +74387,7 @@
     </row>
     <row r="1944">
       <c r="A1944" t="str">
-        <v>Kmti9yukdmczk</v>
+        <v>Kmti9zgfwfb0h</v>
       </c>
       <c r="B1944" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -74425,7 +74425,7 @@
     </row>
     <row r="1945">
       <c r="A1945" t="str">
-        <v>Kmti9yukdud7o</v>
+        <v>Kmti9zgfw1aqi</v>
       </c>
       <c r="B1945" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -74463,7 +74463,7 @@
     </row>
     <row r="1946">
       <c r="A1946" t="str">
-        <v>Kmti9yukdukpv</v>
+        <v>Kmti9zgfwxvsl</v>
       </c>
       <c r="B1946" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -74539,7 +74539,7 @@
     </row>
     <row r="1948">
       <c r="A1948" t="str">
-        <v>Kmti9yukdglp5</v>
+        <v>Kmti9zgfwixeo</v>
       </c>
       <c r="B1948" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -74577,7 +74577,7 @@
     </row>
     <row r="1949">
       <c r="A1949" t="str">
-        <v>Kmti9yukdsspg</v>
+        <v>Kmti9zgfwztsm</v>
       </c>
       <c r="B1949" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -74615,7 +74615,7 @@
     </row>
     <row r="1950">
       <c r="A1950" t="str">
-        <v>Kmti9yukd6krl</v>
+        <v>Kmti9zgfwjky0</v>
       </c>
       <c r="B1950" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -74653,7 +74653,7 @@
     </row>
     <row r="1951" xml:space="preserve">
       <c r="A1951" t="str">
-        <v>Kmti9yukdn376</v>
+        <v>Kmti9zgfwql8b</v>
       </c>
       <c r="B1951" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -74692,7 +74692,7 @@
     </row>
     <row r="1952" xml:space="preserve">
       <c r="A1952" t="str">
-        <v>Kmti9yukd3to2</v>
+        <v>Kmti9zgfwb0ad</v>
       </c>
       <c r="B1952" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -74731,7 +74731,7 @@
     </row>
     <row r="1953" xml:space="preserve">
       <c r="A1953" t="str">
-        <v>Kmti9yukd3rqh</v>
+        <v>Kmti9zgfwr31d</v>
       </c>
       <c r="B1953" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -74770,7 +74770,7 @@
     </row>
     <row r="1954" xml:space="preserve">
       <c r="A1954" t="str">
-        <v>Kmti9yukdtyvp</v>
+        <v>Kmti9zgfwr8in</v>
       </c>
       <c r="B1954" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -74809,7 +74809,7 @@
     </row>
     <row r="1955" xml:space="preserve">
       <c r="A1955" t="str">
-        <v>Kmti9yukdfyug</v>
+        <v>Kmti9zgfwtaz2</v>
       </c>
       <c r="B1955" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Madya/_x000d_
@@ -74848,7 +74848,7 @@
     </row>
     <row r="1956" xml:space="preserve">
       <c r="A1956" t="str">
-        <v>Kmti9yukdx29h</v>
+        <v>Kmti9zgfwqbyo</v>
       </c>
       <c r="B1956" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -74887,7 +74887,7 @@
     </row>
     <row r="1957" xml:space="preserve">
       <c r="A1957" t="str">
-        <v>Kmti9yukdur84</v>
+        <v>Kmti9zgfw8hv9</v>
       </c>
       <c r="B1957" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -75002,7 +75002,7 @@
     </row>
     <row r="1960">
       <c r="A1960" t="str">
-        <v>Kmti9yukdk10e</v>
+        <v>Kmti9zgfwct15</v>
       </c>
       <c r="B1960" t="str">
         <v>Penata Layanan Operasional</v>
@@ -75040,7 +75040,7 @@
     </row>
     <row r="1961">
       <c r="A1961" t="str">
-        <v>Kmti9yukdhon4</v>
+        <v>Kmti9zgfwa9hm</v>
       </c>
       <c r="B1961" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75078,7 +75078,7 @@
     </row>
     <row r="1962">
       <c r="A1962" t="str">
-        <v>Kmti9yukd8ppu</v>
+        <v>Kmti9zgfwlm30</v>
       </c>
       <c r="B1962" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75116,7 +75116,7 @@
     </row>
     <row r="1963">
       <c r="A1963" t="str">
-        <v>Kmti9yukdkow8</v>
+        <v>Kmti9zgfwqbvg</v>
       </c>
       <c r="B1963" t="str">
         <v>Penata Keprotokolan*</v>
@@ -75230,7 +75230,7 @@
     </row>
     <row r="1966">
       <c r="A1966" t="str">
-        <v>Kmti9yukd71if</v>
+        <v>Kmti9zgfws9sa</v>
       </c>
       <c r="B1966" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -75268,7 +75268,7 @@
     </row>
     <row r="1967">
       <c r="A1967" t="str">
-        <v>Kmti9yukdtm84</v>
+        <v>Kmti9zgfwash5</v>
       </c>
       <c r="B1967" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75306,7 +75306,7 @@
     </row>
     <row r="1968">
       <c r="A1968" t="str">
-        <v>Kmti9yukdrwem</v>
+        <v>Kmti9zgfwquo0</v>
       </c>
       <c r="B1968" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75382,7 +75382,7 @@
     </row>
     <row r="1970">
       <c r="A1970" t="str">
-        <v>Kmti9yukdsx8a</v>
+        <v>Kmti9zgfwup3i</v>
       </c>
       <c r="B1970" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -75420,7 +75420,7 @@
     </row>
     <row r="1971">
       <c r="A1971" t="str">
-        <v>Kmti9yukd51cd</v>
+        <v>Kmti9zgfwef5s</v>
       </c>
       <c r="B1971" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75458,7 +75458,7 @@
     </row>
     <row r="1972">
       <c r="A1972" t="str">
-        <v>Kmti9yukdt5l0</v>
+        <v>Kmti9zgfwwtwu</v>
       </c>
       <c r="B1972" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75496,7 +75496,7 @@
     </row>
     <row r="1973" xml:space="preserve">
       <c r="A1973" t="str">
-        <v>Kmti9yukd6r7m</v>
+        <v>Kmti9zgfw75iy</v>
       </c>
       <c r="B1973" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -75535,7 +75535,7 @@
     </row>
     <row r="1974" xml:space="preserve">
       <c r="A1974" t="str">
-        <v>Kmti9yukdrxp3</v>
+        <v>Kmti9zgfwt3u7</v>
       </c>
       <c r="B1974" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -75574,7 +75574,7 @@
     </row>
     <row r="1975" xml:space="preserve">
       <c r="A1975" t="str">
-        <v>Kmti9yukdxxjr</v>
+        <v>Kmti9zgfwetaa</v>
       </c>
       <c r="B1975" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -75613,7 +75613,7 @@
     </row>
     <row r="1976" xml:space="preserve">
       <c r="A1976" t="str">
-        <v>Kmti9yukdgykc</v>
+        <v>Kmti9zgfwckqd</v>
       </c>
       <c r="B1976" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -75728,7 +75728,7 @@
     </row>
     <row r="1979">
       <c r="A1979" t="str">
-        <v>Kmti9yukd7yaj</v>
+        <v>Kmti9zgfwvci0</v>
       </c>
       <c r="B1979" t="str">
         <v>Penata Layanan Operasional</v>
@@ -75766,7 +75766,7 @@
     </row>
     <row r="1980">
       <c r="A1980" t="str">
-        <v>Kmti9yukd94ft</v>
+        <v>Kmti9zgfw7psj</v>
       </c>
       <c r="B1980" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75804,7 +75804,7 @@
     </row>
     <row r="1981">
       <c r="A1981" t="str">
-        <v>Kmti9yukdqgq2</v>
+        <v>Kmti9zgfw0gqv</v>
       </c>
       <c r="B1981" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75842,7 +75842,7 @@
     </row>
     <row r="1982">
       <c r="A1982" t="str">
-        <v>Kmti9yukda4jh</v>
+        <v>Kmti9zgfw1kr2</v>
       </c>
       <c r="B1982" t="str">
         <v>Penata Keprotokolan*</v>
@@ -75956,7 +75956,7 @@
     </row>
     <row r="1985">
       <c r="A1985" t="str">
-        <v>Kmti9yukdop5p</v>
+        <v>Kmti9zgfwryyh</v>
       </c>
       <c r="B1985" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -75994,7 +75994,7 @@
     </row>
     <row r="1986">
       <c r="A1986" t="str">
-        <v>Kmti9yukdn0ij</v>
+        <v>Kmti9zgfwff1h</v>
       </c>
       <c r="B1986" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76032,7 +76032,7 @@
     </row>
     <row r="1987">
       <c r="A1987" t="str">
-        <v>Kmti9yukdj1tf</v>
+        <v>Kmti9zgfw6v3w</v>
       </c>
       <c r="B1987" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76108,7 +76108,7 @@
     </row>
     <row r="1989">
       <c r="A1989" t="str">
-        <v>Kmti9yukd6dm0</v>
+        <v>Kmti9zgfw9zoj</v>
       </c>
       <c r="B1989" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -76146,7 +76146,7 @@
     </row>
     <row r="1990">
       <c r="A1990" t="str">
-        <v>Kmti9yukdpi0w</v>
+        <v>Kmti9zgfwyso0</v>
       </c>
       <c r="B1990" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76184,7 +76184,7 @@
     </row>
     <row r="1991">
       <c r="A1991" t="str">
-        <v>Kmti9yukdkhs9</v>
+        <v>Kmti9zgfwugsv</v>
       </c>
       <c r="B1991" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76222,7 +76222,7 @@
     </row>
     <row r="1992" xml:space="preserve">
       <c r="A1992" t="str">
-        <v>Kmti9yukdyo8h</v>
+        <v>Kmti9zgfw6fhy</v>
       </c>
       <c r="B1992" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -76261,7 +76261,7 @@
     </row>
     <row r="1993" xml:space="preserve">
       <c r="A1993" t="str">
-        <v>Kmti9yukd1jwm</v>
+        <v>Kmti9zgfwexxz</v>
       </c>
       <c r="B1993" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -76300,7 +76300,7 @@
     </row>
     <row r="1994" xml:space="preserve">
       <c r="A1994" t="str">
-        <v>Kmti9yukdsz3n</v>
+        <v>Kmti9zgfwx8ig</v>
       </c>
       <c r="B1994" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -76339,7 +76339,7 @@
     </row>
     <row r="1995" xml:space="preserve">
       <c r="A1995" t="str">
-        <v>Kmti9yukevvbo</v>
+        <v>Kmti9zgfwt7iw</v>
       </c>
       <c r="B1995" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -76454,7 +76454,7 @@
     </row>
     <row r="1998">
       <c r="A1998" t="str">
-        <v>Kmti9yuken0ok</v>
+        <v>Kmti9zgfw4cxt</v>
       </c>
       <c r="B1998" t="str">
         <v>Penata Layanan Operasional</v>
@@ -76492,7 +76492,7 @@
     </row>
     <row r="1999">
       <c r="A1999" t="str">
-        <v>Kmti9yukewwcg</v>
+        <v>Kmti9zgfwxx46</v>
       </c>
       <c r="B1999" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76530,7 +76530,7 @@
     </row>
     <row r="2000">
       <c r="A2000" t="str">
-        <v>Kmti9yuke55ge</v>
+        <v>Kmti9zgfwdx4b</v>
       </c>
       <c r="B2000" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76568,7 +76568,7 @@
     </row>
     <row r="2001">
       <c r="A2001" t="str">
-        <v>Kmti9yukeeapn</v>
+        <v>Kmti9zgfwuima</v>
       </c>
       <c r="B2001" t="str">
         <v>Penata Keprotokolan*</v>
@@ -76682,7 +76682,7 @@
     </row>
     <row r="2004">
       <c r="A2004" t="str">
-        <v>Kmti9yukev16f</v>
+        <v>Kmti9zgfwtjyt</v>
       </c>
       <c r="B2004" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -76720,7 +76720,7 @@
     </row>
     <row r="2005">
       <c r="A2005" t="str">
-        <v>Kmti9yuke203w</v>
+        <v>Kmti9zgfx25jb</v>
       </c>
       <c r="B2005" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76758,7 +76758,7 @@
     </row>
     <row r="2006">
       <c r="A2006" t="str">
-        <v>Kmti9yuke9miy</v>
+        <v>Kmti9zgfxvr5x</v>
       </c>
       <c r="B2006" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76834,7 +76834,7 @@
     </row>
     <row r="2008">
       <c r="A2008" t="str">
-        <v>Kmti9yukenr18</v>
+        <v>Kmti9zgfx60nq</v>
       </c>
       <c r="B2008" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -76872,7 +76872,7 @@
     </row>
     <row r="2009">
       <c r="A2009" t="str">
-        <v>Kmti9yukextx7</v>
+        <v>Kmti9zgfx5fvs</v>
       </c>
       <c r="B2009" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76910,7 +76910,7 @@
     </row>
     <row r="2010">
       <c r="A2010" t="str">
-        <v>Kmti9yukecz84</v>
+        <v>Kmti9zgfx8g5q</v>
       </c>
       <c r="B2010" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76948,7 +76948,7 @@
     </row>
     <row r="2011" xml:space="preserve">
       <c r="A2011" t="str">
-        <v>Kmti9yuke757d</v>
+        <v>Kmti9zgfxshjn</v>
       </c>
       <c r="B2011" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -76987,7 +76987,7 @@
     </row>
     <row r="2012" xml:space="preserve">
       <c r="A2012" t="str">
-        <v>Kmti9yukeqj8g</v>
+        <v>Kmti9zgfxrkcb</v>
       </c>
       <c r="B2012" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -77026,7 +77026,7 @@
     </row>
     <row r="2013" xml:space="preserve">
       <c r="A2013" t="str">
-        <v>Kmti9yukehzdz</v>
+        <v>Kmti9zgfx1osk</v>
       </c>
       <c r="B2013" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -77065,7 +77065,7 @@
     </row>
     <row r="2014" xml:space="preserve">
       <c r="A2014" t="str">
-        <v>Kmti9yuke192p</v>
+        <v>Kmti9zgfx01sb</v>
       </c>
       <c r="B2014" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -77180,7 +77180,7 @@
     </row>
     <row r="2017">
       <c r="A2017" t="str">
-        <v>Kmti9yukexnyw</v>
+        <v>Kmti9zgfxxidv</v>
       </c>
       <c r="B2017" t="str">
         <v>Penata Layanan Operasional</v>
@@ -77218,7 +77218,7 @@
     </row>
     <row r="2018">
       <c r="A2018" t="str">
-        <v>Kmti9yuke6wi6</v>
+        <v>Kmti9zgfxnyrh</v>
       </c>
       <c r="B2018" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -77256,7 +77256,7 @@
     </row>
     <row r="2019">
       <c r="A2019" t="str">
-        <v>Kmti9yukez3al</v>
+        <v>Kmti9zgfxvb34</v>
       </c>
       <c r="B2019" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -77294,7 +77294,7 @@
     </row>
     <row r="2020">
       <c r="A2020" t="str">
-        <v>Kmti9yukeol57</v>
+        <v>Kmti9zgfxoj9b</v>
       </c>
       <c r="B2020" t="str">
         <v>Penata Keprotokolan*</v>
@@ -77408,7 +77408,7 @@
     </row>
     <row r="2023">
       <c r="A2023" t="str">
-        <v>Kmti9yukegoow</v>
+        <v>Kmti9zgfxkbvv</v>
       </c>
       <c r="B2023" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -77446,7 +77446,7 @@
     </row>
     <row r="2024">
       <c r="A2024" t="str">
-        <v>Kmti9yukekino</v>
+        <v>Kmti9zgfxhm06</v>
       </c>
       <c r="B2024" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -77484,7 +77484,7 @@
     </row>
     <row r="2025">
       <c r="A2025" t="str">
-        <v>Kmti9yuke7wyt</v>
+        <v>Kmti9zgfx63dk</v>
       </c>
       <c r="B2025" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -77560,7 +77560,7 @@
     </row>
     <row r="2027">
       <c r="A2027" t="str">
-        <v>Kmti9yukeiueo</v>
+        <v>Kmti9zgfxupom</v>
       </c>
       <c r="B2027" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -77598,7 +77598,7 @@
     </row>
     <row r="2028">
       <c r="A2028" t="str">
-        <v>Kmti9yukexcfr</v>
+        <v>Kmti9zgfxovu8</v>
       </c>
       <c r="B2028" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -77636,7 +77636,7 @@
     </row>
     <row r="2029">
       <c r="A2029" t="str">
-        <v>Kmti9yukentw8</v>
+        <v>Kmti9zgfxwy6o</v>
       </c>
       <c r="B2029" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -77674,7 +77674,7 @@
     </row>
     <row r="2030" xml:space="preserve">
       <c r="A2030" t="str">
-        <v>Kmti9yukef2w2</v>
+        <v>Kmti9zgfxflrx</v>
       </c>
       <c r="B2030" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -77713,7 +77713,7 @@
     </row>
     <row r="2031" xml:space="preserve">
       <c r="A2031" t="str">
-        <v>Kmti9yuke32zg</v>
+        <v>Kmti9zgfxc1b3</v>
       </c>
       <c r="B2031" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -77752,7 +77752,7 @@
     </row>
     <row r="2032" xml:space="preserve">
       <c r="A2032" t="str">
-        <v>Kmti9yukehiz7</v>
+        <v>Kmti9zgfxt41q</v>
       </c>
       <c r="B2032" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -77791,7 +77791,7 @@
     </row>
     <row r="2033" xml:space="preserve">
       <c r="A2033" t="str">
-        <v>Kmti9yukejo44</v>
+        <v>Kmti9zgfxiwy8</v>
       </c>
       <c r="B2033" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -77830,7 +77830,7 @@
     </row>
     <row r="2034">
       <c r="A2034" t="str">
-        <v>Kmti9yukexfff</v>
+        <v>Kmti9zgfxmdk5</v>
       </c>
       <c r="B2034" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Muda</v>
@@ -77868,7 +77868,7 @@
     </row>
     <row r="2035">
       <c r="A2035" t="str">
-        <v>Kmti9yukepndc</v>
+        <v>Kmti9zgfxvt2x</v>
       </c>
       <c r="B2035" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Pertama</v>
@@ -77944,7 +77944,7 @@
     </row>
     <row r="2037" xml:space="preserve">
       <c r="A2037" t="str">
-        <v>Kmti9yukeaxlh</v>
+        <v>Kmti9zgfxcf89</v>
       </c>
       <c r="B2037" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_

</xml_diff>

<commit_message>
Perbarui struktur organisasi (2026-09-01T06:18:27.421Z)
</commit_message>
<xml_diff>
--- a/data/struktur-organisasi.xlsx
+++ b/data/struktur-organisasi.xlsx
@@ -63909,7 +63909,7 @@
     </row>
     <row r="1669">
       <c r="A1669" t="str">
-        <v>Kmti9zgfv26p3</v>
+        <v>Kmtia02g5jawg</v>
       </c>
       <c r="B1669" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -63947,7 +63947,7 @@
     </row>
     <row r="1670">
       <c r="A1670" t="str">
-        <v>Kmti9zgfvwyrb</v>
+        <v>Kmtia02g5naro</v>
       </c>
       <c r="B1670" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -63985,7 +63985,7 @@
     </row>
     <row r="1671">
       <c r="A1671" t="str">
-        <v>Kmti9zgfvtx00</v>
+        <v>Kmtia02g5i9oq</v>
       </c>
       <c r="B1671" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -64023,7 +64023,7 @@
     </row>
     <row r="1672">
       <c r="A1672" t="str">
-        <v>Kmti9zgfv4cbb</v>
+        <v>Kmtia02g5tdaw</v>
       </c>
       <c r="B1672" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -64061,7 +64061,7 @@
     </row>
     <row r="1673">
       <c r="A1673" t="str">
-        <v>Kmti9zgfv0cd5</v>
+        <v>Kmtia02g5n2em</v>
       </c>
       <c r="B1673" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -64099,7 +64099,7 @@
     </row>
     <row r="1674">
       <c r="A1674" t="str">
-        <v>Kmti9zgfv45ja</v>
+        <v>Kmtia02g5dqvc</v>
       </c>
       <c r="B1674" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64137,7 +64137,7 @@
     </row>
     <row r="1675">
       <c r="A1675" t="str">
-        <v>Kmti9zgfv5dbr</v>
+        <v>Kmtia02g58etg</v>
       </c>
       <c r="B1675" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64175,7 +64175,7 @@
     </row>
     <row r="1676">
       <c r="A1676" t="str">
-        <v>Kmti9zgfvpxse</v>
+        <v>Kmtia02g5p8rj</v>
       </c>
       <c r="B1676" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -64251,7 +64251,7 @@
     </row>
     <row r="1678">
       <c r="A1678" t="str">
-        <v>Kmti9zgfvuuv7</v>
+        <v>Kmtia02g5b6su</v>
       </c>
       <c r="B1678" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -64289,7 +64289,7 @@
     </row>
     <row r="1679">
       <c r="A1679" t="str">
-        <v>Kmti9zgfvlrdk</v>
+        <v>Kmtia02g5fh5r</v>
       </c>
       <c r="B1679" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -64327,7 +64327,7 @@
     </row>
     <row r="1680">
       <c r="A1680" t="str">
-        <v>Kmti9zgfvbsli</v>
+        <v>Kmtia02g5kbtf</v>
       </c>
       <c r="B1680" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -64365,7 +64365,7 @@
     </row>
     <row r="1681">
       <c r="A1681" t="str">
-        <v>Kmti9zgfv70po</v>
+        <v>Kmtia02g51e7e</v>
       </c>
       <c r="B1681" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -64403,7 +64403,7 @@
     </row>
     <row r="1682">
       <c r="A1682" t="str">
-        <v>Kmti9zgfveogu</v>
+        <v>Kmtia02g5377n</v>
       </c>
       <c r="B1682" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -64441,7 +64441,7 @@
     </row>
     <row r="1683">
       <c r="A1683" t="str">
-        <v>Kmti9zgfvmgxf</v>
+        <v>Kmtia02g5j4jj</v>
       </c>
       <c r="B1683" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64479,7 +64479,7 @@
     </row>
     <row r="1684">
       <c r="A1684" t="str">
-        <v>Kmti9zgfvknli</v>
+        <v>Kmtia02g5kjjt</v>
       </c>
       <c r="B1684" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64517,7 +64517,7 @@
     </row>
     <row r="1685">
       <c r="A1685" t="str">
-        <v>Kmti9zgfvprvh</v>
+        <v>Kmtia02g5qh5e</v>
       </c>
       <c r="B1685" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -64593,7 +64593,7 @@
     </row>
     <row r="1687">
       <c r="A1687" t="str">
-        <v>Kmti9zgfvbb3w</v>
+        <v>Kmtia02g5dfjp</v>
       </c>
       <c r="B1687" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -64631,7 +64631,7 @@
     </row>
     <row r="1688">
       <c r="A1688" t="str">
-        <v>Kmti9zgfvdowe</v>
+        <v>Kmtia02g5dmi3</v>
       </c>
       <c r="B1688" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -64669,7 +64669,7 @@
     </row>
     <row r="1689">
       <c r="A1689" t="str">
-        <v>Kmti9zgfvapml</v>
+        <v>Kmtia02g5h0s5</v>
       </c>
       <c r="B1689" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -64707,7 +64707,7 @@
     </row>
     <row r="1690">
       <c r="A1690" t="str">
-        <v>Kmti9zgfv6noy</v>
+        <v>Kmtia02g5fbah</v>
       </c>
       <c r="B1690" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -64745,7 +64745,7 @@
     </row>
     <row r="1691">
       <c r="A1691" t="str">
-        <v>Kmti9zgfvsrt3</v>
+        <v>Kmtia02g5kh36</v>
       </c>
       <c r="B1691" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -64783,7 +64783,7 @@
     </row>
     <row r="1692">
       <c r="A1692" t="str">
-        <v>Kmti9zgfv7snw</v>
+        <v>Kmtia02g5xi3y</v>
       </c>
       <c r="B1692" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64821,7 +64821,7 @@
     </row>
     <row r="1693">
       <c r="A1693" t="str">
-        <v>Kmti9zgfvijxf</v>
+        <v>Kmtia02g5nhoc</v>
       </c>
       <c r="B1693" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64859,7 +64859,7 @@
     </row>
     <row r="1694">
       <c r="A1694" t="str">
-        <v>Kmti9zgfvq82j</v>
+        <v>Kmtia02g54eq6</v>
       </c>
       <c r="B1694" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -64897,7 +64897,7 @@
     </row>
     <row r="1695">
       <c r="A1695" t="str">
-        <v>Kmti9zgfvy2bj</v>
+        <v>Kmtia02g5vltc</v>
       </c>
       <c r="B1695" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64935,7 +64935,7 @@
     </row>
     <row r="1696">
       <c r="A1696" t="str">
-        <v>Kmti9zgfv3xh5</v>
+        <v>Kmtia02g505c3</v>
       </c>
       <c r="B1696" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64973,7 +64973,7 @@
     </row>
     <row r="1697">
       <c r="A1697" t="str">
-        <v>Kmti9zgfv676s</v>
+        <v>Kmtia02g5vo6a</v>
       </c>
       <c r="B1697" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -65087,7 +65087,7 @@
     </row>
     <row r="1700">
       <c r="A1700" t="str">
-        <v>Kmti9zgfv4f31</v>
+        <v>Kmtia02g555dj</v>
       </c>
       <c r="B1700" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -65125,7 +65125,7 @@
     </row>
     <row r="1701">
       <c r="A1701" t="str">
-        <v>Kmti9zgfvaki2</v>
+        <v>Kmtia02g5gq2n</v>
       </c>
       <c r="B1701" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -65163,7 +65163,7 @@
     </row>
     <row r="1702">
       <c r="A1702" t="str">
-        <v>Kmti9zgfvljfh</v>
+        <v>Kmtia02g56jm2</v>
       </c>
       <c r="B1702" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -65201,7 +65201,7 @@
     </row>
     <row r="1703">
       <c r="A1703" t="str">
-        <v>Kmti9zgfvbm7i</v>
+        <v>Kmtia02g5ys50</v>
       </c>
       <c r="B1703" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -65239,7 +65239,7 @@
     </row>
     <row r="1704">
       <c r="A1704" t="str">
-        <v>Kmti9zgfvw9hy</v>
+        <v>Kmtia02g59s2o</v>
       </c>
       <c r="B1704" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -65277,7 +65277,7 @@
     </row>
     <row r="1705">
       <c r="A1705" t="str">
-        <v>Kmti9zgfv2qcb</v>
+        <v>Kmtia02g5ezsf</v>
       </c>
       <c r="B1705" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -65315,7 +65315,7 @@
     </row>
     <row r="1706">
       <c r="A1706" t="str">
-        <v>Kmti9zgfvd8mh</v>
+        <v>Kmtia02g54416</v>
       </c>
       <c r="B1706" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -65353,7 +65353,7 @@
     </row>
     <row r="1707">
       <c r="A1707" t="str">
-        <v>Kmti9zgfvc9si</v>
+        <v>Kmtia02g5m43x</v>
       </c>
       <c r="B1707" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -65391,7 +65391,7 @@
     </row>
     <row r="1708">
       <c r="A1708" t="str">
-        <v>Kmti9zgfvawm4</v>
+        <v>Kmtia02g58zdp</v>
       </c>
       <c r="B1708" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -65429,7 +65429,7 @@
     </row>
     <row r="1709">
       <c r="A1709" t="str">
-        <v>Kmti9zgfvu4kv</v>
+        <v>Kmtia02g5um0d</v>
       </c>
       <c r="B1709" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -65505,7 +65505,7 @@
     </row>
     <row r="1711">
       <c r="A1711" t="str">
-        <v>Kmti9zgfvn91l</v>
+        <v>Kmtia02g5dtlp</v>
       </c>
       <c r="B1711" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -65543,7 +65543,7 @@
     </row>
     <row r="1712">
       <c r="A1712" t="str">
-        <v>Kmti9zgfvy7ll</v>
+        <v>Kmtia02g5ug8c</v>
       </c>
       <c r="B1712" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -65581,7 +65581,7 @@
     </row>
     <row r="1713">
       <c r="A1713" t="str">
-        <v>Kmti9zgfv3bkw</v>
+        <v>Kmtia02g5azkf</v>
       </c>
       <c r="B1713" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -65619,7 +65619,7 @@
     </row>
     <row r="1714">
       <c r="A1714" t="str">
-        <v>Kmti9zgfvk58c</v>
+        <v>Kmtia02g5a723</v>
       </c>
       <c r="B1714" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -65657,7 +65657,7 @@
     </row>
     <row r="1715">
       <c r="A1715" t="str">
-        <v>Kmti9zgfvg5e1</v>
+        <v>Kmtia02g5570l</v>
       </c>
       <c r="B1715" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -65695,7 +65695,7 @@
     </row>
     <row r="1716">
       <c r="A1716" t="str">
-        <v>Kmti9zgfvk469</v>
+        <v>Kmtia02g5474m</v>
       </c>
       <c r="B1716" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -65733,7 +65733,7 @@
     </row>
     <row r="1717">
       <c r="A1717" t="str">
-        <v>Kmti9zgfwkwkh</v>
+        <v>Kmtia02g535lj</v>
       </c>
       <c r="B1717" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -65771,7 +65771,7 @@
     </row>
     <row r="1718">
       <c r="A1718" t="str">
-        <v>Kmti9zgfwsx0u</v>
+        <v>Kmtia02g58dyt</v>
       </c>
       <c r="B1718" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -65847,7 +65847,7 @@
     </row>
     <row r="1720">
       <c r="A1720" t="str">
-        <v>Kmti9zgfwr6bz</v>
+        <v>Kmtia02g5g8of</v>
       </c>
       <c r="B1720" t="str">
         <v>Penata Layanan Operasional</v>
@@ -65885,7 +65885,7 @@
     </row>
     <row r="1721">
       <c r="A1721" t="str">
-        <v>Kmti9zgfwgsxa</v>
+        <v>Kmtia02g57dow</v>
       </c>
       <c r="B1721" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -65923,7 +65923,7 @@
     </row>
     <row r="1722">
       <c r="A1722" t="str">
-        <v>Kmti9zgfw4dul</v>
+        <v>Kmtia02g5v18i</v>
       </c>
       <c r="B1722" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -65961,7 +65961,7 @@
     </row>
     <row r="1723">
       <c r="A1723" t="str">
-        <v>Kmti9zgfwowkd</v>
+        <v>Kmtia02g52jmt</v>
       </c>
       <c r="B1723" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -65999,7 +65999,7 @@
     </row>
     <row r="1724">
       <c r="A1724" t="str">
-        <v>Kmti9zgfwsb26</v>
+        <v>Kmtia02g5ews8</v>
       </c>
       <c r="B1724" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -66037,7 +66037,7 @@
     </row>
     <row r="1725">
       <c r="A1725" t="str">
-        <v>Kmti9zgfwaza4</v>
+        <v>Kmtia02g5cesx</v>
       </c>
       <c r="B1725" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -66075,7 +66075,7 @@
     </row>
     <row r="1726">
       <c r="A1726" t="str">
-        <v>Kmti9zgfwure0</v>
+        <v>Kmtia02g5n8zw</v>
       </c>
       <c r="B1726" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -66113,7 +66113,7 @@
     </row>
     <row r="1727">
       <c r="A1727" t="str">
-        <v>Kmti9zgfwsb5n</v>
+        <v>Kmtia02g552t4</v>
       </c>
       <c r="B1727" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -66189,7 +66189,7 @@
     </row>
     <row r="1729">
       <c r="A1729" t="str">
-        <v>Kmti9zgfw36rk</v>
+        <v>Kmtia02g504v6</v>
       </c>
       <c r="B1729" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -66227,7 +66227,7 @@
     </row>
     <row r="1730">
       <c r="A1730" t="str">
-        <v>Kmti9zgfw3xp6</v>
+        <v>Kmtia02g5brv4</v>
       </c>
       <c r="B1730" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -66265,7 +66265,7 @@
     </row>
     <row r="1731">
       <c r="A1731" t="str">
-        <v>Kmti9zgfwfvik</v>
+        <v>Kmtia02g5gq6m</v>
       </c>
       <c r="B1731" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -66303,7 +66303,7 @@
     </row>
     <row r="1732">
       <c r="A1732" t="str">
-        <v>Kmti9zgfw4593</v>
+        <v>Kmtia02g5v3hn</v>
       </c>
       <c r="B1732" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -66341,7 +66341,7 @@
     </row>
     <row r="1733">
       <c r="A1733" t="str">
-        <v>Kmti9zgfw4kki</v>
+        <v>Kmtia02g5sieb</v>
       </c>
       <c r="B1733" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -66379,7 +66379,7 @@
     </row>
     <row r="1734">
       <c r="A1734" t="str">
-        <v>Kmti9zgfw72q9</v>
+        <v>Kmtia02g5lvtj</v>
       </c>
       <c r="B1734" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -66417,7 +66417,7 @@
     </row>
     <row r="1735">
       <c r="A1735" t="str">
-        <v>Kmti9zgfw0hmg</v>
+        <v>Kmtia02g5r2ur</v>
       </c>
       <c r="B1735" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -66455,7 +66455,7 @@
     </row>
     <row r="1736">
       <c r="A1736" t="str">
-        <v>Kmti9zgfw9jf7</v>
+        <v>Kmtia02g5oaqr</v>
       </c>
       <c r="B1736" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -66493,7 +66493,7 @@
     </row>
     <row r="1737">
       <c r="A1737" t="str">
-        <v>Kmti9zgfw4y3j</v>
+        <v>Kmtia02g5n333</v>
       </c>
       <c r="B1737" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -66531,7 +66531,7 @@
     </row>
     <row r="1738">
       <c r="A1738" t="str">
-        <v>Kmti9zgfwto78</v>
+        <v>Kmtia02g57e65</v>
       </c>
       <c r="B1738" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -66569,7 +66569,7 @@
     </row>
     <row r="1739">
       <c r="A1739" t="str">
-        <v>Kmti9zgfw6xgk</v>
+        <v>Kmtia02g5c10j</v>
       </c>
       <c r="B1739" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -66607,7 +66607,7 @@
     </row>
     <row r="1740">
       <c r="A1740" t="str">
-        <v>Kmti9zgfw57jm</v>
+        <v>Kmtia02g57618</v>
       </c>
       <c r="B1740" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -66645,7 +66645,7 @@
     </row>
     <row r="1741">
       <c r="A1741" t="str">
-        <v>Kmti9zgfwlksp</v>
+        <v>Kmtia02g5bfnx</v>
       </c>
       <c r="B1741" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -66683,7 +66683,7 @@
     </row>
     <row r="1742">
       <c r="A1742" t="str">
-        <v>Kmti9zgfwiets</v>
+        <v>Kmtia02g5og4z</v>
       </c>
       <c r="B1742" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -66721,7 +66721,7 @@
     </row>
     <row r="1743">
       <c r="A1743" t="str">
-        <v>Kmti9zgfwmd71</v>
+        <v>Kmtia02g57n1z</v>
       </c>
       <c r="B1743" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -66835,7 +66835,7 @@
     </row>
     <row r="1746">
       <c r="A1746" t="str">
-        <v>Kmti9zgfwph3s</v>
+        <v>Kmtia02g5uor5</v>
       </c>
       <c r="B1746" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -66873,7 +66873,7 @@
     </row>
     <row r="1747">
       <c r="A1747" t="str">
-        <v>Kmti9zgfwkppc</v>
+        <v>Kmtia02g5kucy</v>
       </c>
       <c r="B1747" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -66911,7 +66911,7 @@
     </row>
     <row r="1748">
       <c r="A1748" t="str">
-        <v>Kmti9zgfw0cxv</v>
+        <v>Kmtia02g5quiy</v>
       </c>
       <c r="B1748" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -66949,7 +66949,7 @@
     </row>
     <row r="1749" xml:space="preserve">
       <c r="A1749" t="str">
-        <v>Kmti9zgfw6ykh</v>
+        <v>Kmtia02g5rqqv</v>
       </c>
       <c r="B1749" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -66988,7 +66988,7 @@
     </row>
     <row r="1750">
       <c r="A1750" t="str">
-        <v>Kmti9zgfwrkt3</v>
+        <v>Kmtia02g5y05f</v>
       </c>
       <c r="B1750" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -67064,7 +67064,7 @@
     </row>
     <row r="1752">
       <c r="A1752" t="str">
-        <v>Kmti9zgfw2txy</v>
+        <v>Kmtia02g5mc4x</v>
       </c>
       <c r="B1752" t="str">
         <v>Penata Layanan Operasional</v>
@@ -67102,7 +67102,7 @@
     </row>
     <row r="1753">
       <c r="A1753" t="str">
-        <v>Kmti9zgfw3olu</v>
+        <v>Kmtia02g5ooyp</v>
       </c>
       <c r="B1753" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -67140,7 +67140,7 @@
     </row>
     <row r="1754">
       <c r="A1754" t="str">
-        <v>Kmti9zgfwyrgw</v>
+        <v>Kmtia02g5f59f</v>
       </c>
       <c r="B1754" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -67178,7 +67178,7 @@
     </row>
     <row r="1755" xml:space="preserve">
       <c r="A1755" t="str">
-        <v>Kmti9zgfw5xjt</v>
+        <v>Kmtia02g5ie9e</v>
       </c>
       <c r="B1755" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -67217,7 +67217,7 @@
     </row>
     <row r="1756" xml:space="preserve">
       <c r="A1756" t="str">
-        <v>Kmti9zgfwukt5</v>
+        <v>Kmtia02g50k5a</v>
       </c>
       <c r="B1756" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -67256,7 +67256,7 @@
     </row>
     <row r="1757">
       <c r="A1757" t="str">
-        <v>Kmti9zgfwffgf</v>
+        <v>Kmtia02g5qac8</v>
       </c>
       <c r="B1757" t="str">
         <v>Pranata Keuangan APBN Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -67294,7 +67294,7 @@
     </row>
     <row r="1758" xml:space="preserve">
       <c r="A1758" t="str">
-        <v>Kmti9zgfwfrt0</v>
+        <v>Kmtia02g5hnhr</v>
       </c>
       <c r="B1758" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Mahir/_x000d_
@@ -67333,7 +67333,7 @@
     </row>
     <row r="1759" xml:space="preserve">
       <c r="A1759" t="str">
-        <v>Kmti9zgfwqx35</v>
+        <v>Kmtia02g5ow1a</v>
       </c>
       <c r="B1759" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Terampil/_x000d_
@@ -67410,7 +67410,7 @@
     </row>
     <row r="1761">
       <c r="A1761" t="str">
-        <v>Kmti9zgfwp79t</v>
+        <v>Kmtia02g504rl</v>
       </c>
       <c r="B1761" t="str">
         <v>Penata Layanan Operasional</v>
@@ -67448,7 +67448,7 @@
     </row>
     <row r="1762">
       <c r="A1762" t="str">
-        <v>Kmti9zgfw5w0d</v>
+        <v>Kmtia02g5z7ob</v>
       </c>
       <c r="B1762" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -67486,7 +67486,7 @@
     </row>
     <row r="1763">
       <c r="A1763" t="str">
-        <v>Kmti9zgfwwc7b</v>
+        <v>Kmtia02g56yb1</v>
       </c>
       <c r="B1763" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -67524,7 +67524,7 @@
     </row>
     <row r="1764" xml:space="preserve">
       <c r="A1764" t="str">
-        <v>Kmti9zgfwgmis</v>
+        <v>Kmtia02g5l8u6</v>
       </c>
       <c r="B1764" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -67563,7 +67563,7 @@
     </row>
     <row r="1765" xml:space="preserve">
       <c r="A1765" t="str">
-        <v>Kmti9zgfwqfcn</v>
+        <v>Kmtia02g5y7sd</v>
       </c>
       <c r="B1765" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -67602,7 +67602,7 @@
     </row>
     <row r="1766">
       <c r="A1766" t="str">
-        <v>Kmti9zgfw8fwd</v>
+        <v>Kmtia02g5iaic</v>
       </c>
       <c r="B1766" t="str">
         <v>Pranata Keuangan APBN Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -67640,7 +67640,7 @@
     </row>
     <row r="1767" xml:space="preserve">
       <c r="A1767" t="str">
-        <v>Kmti9zgfw3a03</v>
+        <v>Kmtia02g59bdb</v>
       </c>
       <c r="B1767" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Mahir/_x000d_
@@ -67679,7 +67679,7 @@
     </row>
     <row r="1768" xml:space="preserve">
       <c r="A1768" t="str">
-        <v>Kmti9zgfwnd9w</v>
+        <v>Kmtia02g5jhar</v>
       </c>
       <c r="B1768" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Terampil/_x000d_
@@ -67718,7 +67718,7 @@
     </row>
     <row r="1769">
       <c r="A1769" t="str">
-        <v>Kmti9zgfwg7p6</v>
+        <v>Kmtia02g5otlq</v>
       </c>
       <c r="B1769" t="str">
         <v>Analis Anggaran Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -67756,7 +67756,7 @@
     </row>
     <row r="1770">
       <c r="A1770" t="str">
-        <v>Kmti9zgfwlxww</v>
+        <v>Kmtia02g50c5p</v>
       </c>
       <c r="B1770" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -67794,7 +67794,7 @@
     </row>
     <row r="1771">
       <c r="A1771" t="str">
-        <v>Kmti9zgfweso7</v>
+        <v>Kmtia02g5fxu8</v>
       </c>
       <c r="B1771" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Madya/Pengawas Keuangan Negara Ahli Madya</v>
@@ -67832,7 +67832,7 @@
     </row>
     <row r="1772">
       <c r="A1772" t="str">
-        <v>Kmti9zgfwya1b</v>
+        <v>Kmtia02g51840</v>
       </c>
       <c r="B1772" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Muda/Pengawas Keuangan Negara Ahli Ahli Muda</v>
@@ -67870,7 +67870,7 @@
     </row>
     <row r="1773">
       <c r="A1773" t="str">
-        <v>Kmti9zgfwol0w</v>
+        <v>Kmtia02g54482</v>
       </c>
       <c r="B1773" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Pertama/Pengawas Keuangan Negara Ahli Pertama</v>
@@ -67908,7 +67908,7 @@
     </row>
     <row r="1774">
       <c r="A1774" t="str">
-        <v>Kmti9zgfw4mzw</v>
+        <v>Kmtia02g5x7dm</v>
       </c>
       <c r="B1774" t="str">
         <v>Pranata Keuangan APBN Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -67946,7 +67946,7 @@
     </row>
     <row r="1775">
       <c r="A1775" t="str">
-        <v>Kmti9zgfwb5sn</v>
+        <v>Kmtia02g56c0k</v>
       </c>
       <c r="B1775" t="str">
         <v>Pranata Keuangan APBN Mahir/Pengawas Keuangan Negara Mahir</v>
@@ -67984,7 +67984,7 @@
     </row>
     <row r="1776">
       <c r="A1776" t="str">
-        <v>Kmti9zgfw42g7</v>
+        <v>Kmtia02g57l4j</v>
       </c>
       <c r="B1776" t="str">
         <v>Pranata Keuangan APBN Terampil/Pengawas Keuangan Negara Terampil</v>
@@ -68098,7 +68098,7 @@
     </row>
     <row r="1779">
       <c r="A1779" t="str">
-        <v>Kmti9zgfwgvaq</v>
+        <v>Kmtia02g5ijsg</v>
       </c>
       <c r="B1779" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68136,7 +68136,7 @@
     </row>
     <row r="1780">
       <c r="A1780" t="str">
-        <v>Kmti9zgfw117s</v>
+        <v>Kmtia02g5q6zy</v>
       </c>
       <c r="B1780" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -68174,7 +68174,7 @@
     </row>
     <row r="1781">
       <c r="A1781" t="str">
-        <v>Kmti9zgfwc6hl</v>
+        <v>Kmtia02g51nq2</v>
       </c>
       <c r="B1781" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -68250,7 +68250,7 @@
     </row>
     <row r="1783">
       <c r="A1783" t="str">
-        <v>Kmti9zgfwprkg</v>
+        <v>Kmtia02g5mcdz</v>
       </c>
       <c r="B1783" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68288,7 +68288,7 @@
     </row>
     <row r="1784">
       <c r="A1784" t="str">
-        <v>Kmti9zgfwlhys</v>
+        <v>Kmtia02g57aq0</v>
       </c>
       <c r="B1784" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -68326,7 +68326,7 @@
     </row>
     <row r="1785">
       <c r="A1785" t="str">
-        <v>Kmti9zgfwkuna</v>
+        <v>Kmtia02g548bq</v>
       </c>
       <c r="B1785" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -68364,7 +68364,7 @@
     </row>
     <row r="1786">
       <c r="A1786" t="str">
-        <v>Kmti9zgfwluh2</v>
+        <v>Kmtia02g5em6c</v>
       </c>
       <c r="B1786" t="str">
         <v>Penata Keprotokolan*</v>
@@ -68402,7 +68402,7 @@
     </row>
     <row r="1787">
       <c r="A1787" t="str">
-        <v>Kmti9zgfwg7ii</v>
+        <v>Kmtia02g5wbt0</v>
       </c>
       <c r="B1787" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -68440,7 +68440,7 @@
     </row>
     <row r="1788">
       <c r="A1788" t="str">
-        <v>Kmti9zgfwzqqc</v>
+        <v>Kmtia02g5tsuz</v>
       </c>
       <c r="B1788" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -68478,7 +68478,7 @@
     </row>
     <row r="1789">
       <c r="A1789" t="str">
-        <v>Kmti9zgfwg8vo</v>
+        <v>Kmtia02g5zee5</v>
       </c>
       <c r="B1789" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -68516,7 +68516,7 @@
     </row>
     <row r="1790">
       <c r="A1790" t="str">
-        <v>Kmti9zgfw6kia</v>
+        <v>Kmtia02g5bzk7</v>
       </c>
       <c r="B1790" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -68592,7 +68592,7 @@
     </row>
     <row r="1792">
       <c r="A1792" t="str">
-        <v>Kmti9zgfwvs7f</v>
+        <v>Kmtia02g5q7o3</v>
       </c>
       <c r="B1792" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68630,7 +68630,7 @@
     </row>
     <row r="1793">
       <c r="A1793" t="str">
-        <v>Kmti9zgfwinbd</v>
+        <v>Kmtia02g5t885</v>
       </c>
       <c r="B1793" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -68668,7 +68668,7 @@
     </row>
     <row r="1794">
       <c r="A1794" t="str">
-        <v>Kmti9zgfwi2a5</v>
+        <v>Kmtia02g541cu</v>
       </c>
       <c r="B1794" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -68706,7 +68706,7 @@
     </row>
     <row r="1795">
       <c r="A1795" t="str">
-        <v>Kmti9zgfw1s7e</v>
+        <v>Kmtia02g57jxa</v>
       </c>
       <c r="B1795" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -68744,7 +68744,7 @@
     </row>
     <row r="1796">
       <c r="A1796" t="str">
-        <v>Kmti9zgfwtdxj</v>
+        <v>Kmtia02g5wphh</v>
       </c>
       <c r="B1796" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -68782,7 +68782,7 @@
     </row>
     <row r="1797">
       <c r="A1797" t="str">
-        <v>Kmti9zgfw2ch2</v>
+        <v>Kmtia02g5f8fz</v>
       </c>
       <c r="B1797" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -68820,7 +68820,7 @@
     </row>
     <row r="1798">
       <c r="A1798" t="str">
-        <v>Kmti9zgfwp942</v>
+        <v>Kmtia02g5hyc0</v>
       </c>
       <c r="B1798" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -68858,7 +68858,7 @@
     </row>
     <row r="1799">
       <c r="A1799" t="str">
-        <v>Kmti9zgfw2ttx</v>
+        <v>Kmtia02g5lelq</v>
       </c>
       <c r="B1799" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -68934,7 +68934,7 @@
     </row>
     <row r="1801">
       <c r="A1801" t="str">
-        <v>Kmti9zgfw74gb</v>
+        <v>Kmtia02g5i80r</v>
       </c>
       <c r="B1801" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68972,7 +68972,7 @@
     </row>
     <row r="1802">
       <c r="A1802" t="str">
-        <v>Kmti9zgfwbjjg</v>
+        <v>Kmtia02g5mz8o</v>
       </c>
       <c r="B1802" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -69010,7 +69010,7 @@
     </row>
     <row r="1803">
       <c r="A1803" t="str">
-        <v>Kmti9zgfwrqwo</v>
+        <v>Kmtia02g59ck3</v>
       </c>
       <c r="B1803" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -69048,7 +69048,7 @@
     </row>
     <row r="1804">
       <c r="A1804" t="str">
-        <v>Kmti9zgfwhexu</v>
+        <v>Kmtia02g5851z</v>
       </c>
       <c r="B1804" t="str">
         <v>Penata Keprotokolan*</v>
@@ -69086,7 +69086,7 @@
     </row>
     <row r="1805">
       <c r="A1805" t="str">
-        <v>Kmti9zgfwdna0</v>
+        <v>Kmtia02g528yh</v>
       </c>
       <c r="B1805" t="str">
         <v>Arsiparis Ahli Muda</v>
@@ -69124,7 +69124,7 @@
     </row>
     <row r="1806">
       <c r="A1806" t="str">
-        <v>Kmti9zgfwxez5</v>
+        <v>Kmtia02g5g3cc</v>
       </c>
       <c r="B1806" t="str">
         <v>Arsiparis Ahli Pertama</v>
@@ -69162,7 +69162,7 @@
     </row>
     <row r="1807">
       <c r="A1807" t="str">
-        <v>Kmti9zgfwy5z6</v>
+        <v>Kmtia02g5qi08</v>
       </c>
       <c r="B1807" t="str">
         <v>Arsiparis Penyelia</v>
@@ -69200,7 +69200,7 @@
     </row>
     <row r="1808">
       <c r="A1808" t="str">
-        <v>Kmti9zgfw5cy1</v>
+        <v>Kmtia02g5tf66</v>
       </c>
       <c r="B1808" t="str">
         <v>Arsiparis Mahir</v>
@@ -69238,7 +69238,7 @@
     </row>
     <row r="1809">
       <c r="A1809" t="str">
-        <v>Kmti9zgfweff0</v>
+        <v>Kmtia02g5en5p</v>
       </c>
       <c r="B1809" t="str">
         <v>Arsiparis Terampil</v>
@@ -69276,7 +69276,7 @@
     </row>
     <row r="1810">
       <c r="A1810" t="str">
-        <v>Kmti9zgfwfxcr</v>
+        <v>Kmtia02g54v75</v>
       </c>
       <c r="B1810" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -69314,7 +69314,7 @@
     </row>
     <row r="1811">
       <c r="A1811" t="str">
-        <v>Kmti9zgfwj2pm</v>
+        <v>Kmtia02g59puy</v>
       </c>
       <c r="B1811" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -69352,7 +69352,7 @@
     </row>
     <row r="1812">
       <c r="A1812" t="str">
-        <v>Kmti9zgfwe8ra</v>
+        <v>Kmtia02g5y4cv</v>
       </c>
       <c r="B1812" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -69390,7 +69390,7 @@
     </row>
     <row r="1813">
       <c r="A1813" t="str">
-        <v>Kmti9zgfwaj0c</v>
+        <v>Kmtia02g5vd0v</v>
       </c>
       <c r="B1813" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -69428,7 +69428,7 @@
     </row>
     <row r="1814">
       <c r="A1814" t="str">
-        <v>Kmti9zgfwvo49</v>
+        <v>Kmtia02g5u2cs</v>
       </c>
       <c r="B1814" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -69542,7 +69542,7 @@
     </row>
     <row r="1817">
       <c r="A1817" t="str">
-        <v>Kmti9zgfwjqwo</v>
+        <v>Kmtia02g5fwmp</v>
       </c>
       <c r="B1817" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -69580,7 +69580,7 @@
     </row>
     <row r="1818">
       <c r="A1818" t="str">
-        <v>Kmti9zgfwem78</v>
+        <v>Kmtia02g5mhs7</v>
       </c>
       <c r="B1818" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -69618,7 +69618,7 @@
     </row>
     <row r="1819">
       <c r="A1819" t="str">
-        <v>Kmti9zgfw48hj</v>
+        <v>Kmtia02g58hq9</v>
       </c>
       <c r="B1819" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -69656,7 +69656,7 @@
     </row>
     <row r="1820">
       <c r="A1820" t="str">
-        <v>Kmti9zgfwyiy6</v>
+        <v>Kmtia02g5ucy1</v>
       </c>
       <c r="B1820" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -69694,7 +69694,7 @@
     </row>
     <row r="1821">
       <c r="A1821" t="str">
-        <v>Kmti9zgfw4rmo</v>
+        <v>Kmtia02g57urv</v>
       </c>
       <c r="B1821" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -69732,7 +69732,7 @@
     </row>
     <row r="1822">
       <c r="A1822" t="str">
-        <v>Kmti9zgfwsdmd</v>
+        <v>Kmtia02g570vk</v>
       </c>
       <c r="B1822" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -69808,7 +69808,7 @@
     </row>
     <row r="1824">
       <c r="A1824" t="str">
-        <v>Kmti9zgfwhaic</v>
+        <v>Kmtia02g5dgnc</v>
       </c>
       <c r="B1824" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -69846,7 +69846,7 @@
     </row>
     <row r="1825">
       <c r="A1825" t="str">
-        <v>Kmti9zgfwz66l</v>
+        <v>Kmtia02g51x9j</v>
       </c>
       <c r="B1825" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -69884,7 +69884,7 @@
     </row>
     <row r="1826">
       <c r="A1826" t="str">
-        <v>Kmti9zgfw2y2o</v>
+        <v>Kmtia02g58aiv</v>
       </c>
       <c r="B1826" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -69922,7 +69922,7 @@
     </row>
     <row r="1827">
       <c r="A1827" t="str">
-        <v>Kmti9zgfwldzg</v>
+        <v>Kmtia02g5094l</v>
       </c>
       <c r="B1827" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -69960,7 +69960,7 @@
     </row>
     <row r="1828">
       <c r="A1828" t="str">
-        <v>Kmti9zgfwln2m</v>
+        <v>Kmtia02g5d1t4</v>
       </c>
       <c r="B1828" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -69998,7 +69998,7 @@
     </row>
     <row r="1829">
       <c r="A1829" t="str">
-        <v>Kmti9zgfw4fjz</v>
+        <v>Kmtia02g57duk</v>
       </c>
       <c r="B1829" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -70036,7 +70036,7 @@
     </row>
     <row r="1830">
       <c r="A1830" t="str">
-        <v>Kmti9zgfwrcj7</v>
+        <v>Kmtia02g5awdb</v>
       </c>
       <c r="B1830" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -70112,7 +70112,7 @@
     </row>
     <row r="1832">
       <c r="A1832" t="str">
-        <v>Kmti9zgfwwsyh</v>
+        <v>Kmtia02g506h5</v>
       </c>
       <c r="B1832" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -70150,7 +70150,7 @@
     </row>
     <row r="1833">
       <c r="A1833" t="str">
-        <v>Kmti9zgfwtkvi</v>
+        <v>Kmtia02g5tgav</v>
       </c>
       <c r="B1833" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -70188,7 +70188,7 @@
     </row>
     <row r="1834">
       <c r="A1834" t="str">
-        <v>Kmti9zgfwv418</v>
+        <v>Kmtia02g53yk1</v>
       </c>
       <c r="B1834" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -70226,7 +70226,7 @@
     </row>
     <row r="1835">
       <c r="A1835" t="str">
-        <v>Kmti9zgfw5nyi</v>
+        <v>Kmtia02g5bnta</v>
       </c>
       <c r="B1835" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -70264,7 +70264,7 @@
     </row>
     <row r="1836">
       <c r="A1836" t="str">
-        <v>Kmti9zgfw36v4</v>
+        <v>Kmtia02g50mv0</v>
       </c>
       <c r="B1836" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -70302,7 +70302,7 @@
     </row>
     <row r="1837">
       <c r="A1837" t="str">
-        <v>Kmti9zgfwrhj9</v>
+        <v>Kmtia02g5en1j</v>
       </c>
       <c r="B1837" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -70340,7 +70340,7 @@
     </row>
     <row r="1838">
       <c r="A1838" t="str">
-        <v>Kmti9zgfw9p5y</v>
+        <v>Kmtia02g5wgv9</v>
       </c>
       <c r="B1838" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -70378,7 +70378,7 @@
     </row>
     <row r="1839">
       <c r="A1839" t="str">
-        <v>Kmti9zgfw7yh8</v>
+        <v>Kmtia02g52l3u</v>
       </c>
       <c r="B1839" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -70416,7 +70416,7 @@
     </row>
     <row r="1840">
       <c r="A1840" t="str">
-        <v>Kmti9zgfwytqd</v>
+        <v>Kmtia02g5sr20</v>
       </c>
       <c r="B1840" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -70454,7 +70454,7 @@
     </row>
     <row r="1841">
       <c r="A1841" t="str">
-        <v>Kmti9zgfwidk1</v>
+        <v>Kmtia02g59eyb</v>
       </c>
       <c r="B1841" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -70492,7 +70492,7 @@
     </row>
     <row r="1842">
       <c r="A1842" t="str">
-        <v>Kmti9zgfw5qi3</v>
+        <v>Kmtia02g5y8fb</v>
       </c>
       <c r="B1842" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -70568,7 +70568,7 @@
     </row>
     <row r="1844">
       <c r="A1844" t="str">
-        <v>Kmti9zgfw7bm4</v>
+        <v>Kmtia02g5mx3q</v>
       </c>
       <c r="B1844" t="str">
         <v>Penata Layanan Operasional</v>
@@ -70606,7 +70606,7 @@
     </row>
     <row r="1845">
       <c r="A1845" t="str">
-        <v>Kmti9zgfwsvbt</v>
+        <v>Kmtia02g5gv4c</v>
       </c>
       <c r="B1845" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -70644,7 +70644,7 @@
     </row>
     <row r="1846">
       <c r="A1846" t="str">
-        <v>Kmti9zgfwg9f7</v>
+        <v>Kmtia02g5mlx1</v>
       </c>
       <c r="B1846" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -70682,7 +70682,7 @@
     </row>
     <row r="1847">
       <c r="A1847" t="str">
-        <v>Kmti9zgfwwt6t</v>
+        <v>Kmtia02g52bdq</v>
       </c>
       <c r="B1847" t="str">
         <v>Pranata Humas Ahli Muda</v>
@@ -70720,7 +70720,7 @@
     </row>
     <row r="1848">
       <c r="A1848" t="str">
-        <v>Kmti9zgfwv7iq</v>
+        <v>Kmtia02g5seaj</v>
       </c>
       <c r="B1848" t="str">
         <v>Pranata Humas Ahli Pertama</v>
@@ -70758,7 +70758,7 @@
     </row>
     <row r="1849">
       <c r="A1849" t="str">
-        <v>Kmti9zgfwdkza</v>
+        <v>Kmtia02g5blr7</v>
       </c>
       <c r="B1849" t="str">
         <v>Pranata Humas Penyelia</v>
@@ -70796,7 +70796,7 @@
     </row>
     <row r="1850">
       <c r="A1850" t="str">
-        <v>Kmti9zgfwko74</v>
+        <v>Kmtia02g5p73l</v>
       </c>
       <c r="B1850" t="str">
         <v>Pranata Humas Mahir</v>
@@ -70834,7 +70834,7 @@
     </row>
     <row r="1851">
       <c r="A1851" t="str">
-        <v>Kmti9zgfwifm5</v>
+        <v>Kmtia02g5zppp</v>
       </c>
       <c r="B1851" t="str">
         <v>Pranata Humas Terampil</v>
@@ -70872,7 +70872,7 @@
     </row>
     <row r="1852">
       <c r="A1852" t="str">
-        <v>Kmti9zgfw8us7</v>
+        <v>Kmtia02g5evqm</v>
       </c>
       <c r="B1852" t="str">
         <v>Pustakawan Ahli Muda</v>
@@ -70910,7 +70910,7 @@
     </row>
     <row r="1853">
       <c r="A1853" t="str">
-        <v>Kmti9zgfwbumm</v>
+        <v>Kmtia02g5sk81</v>
       </c>
       <c r="B1853" t="str">
         <v>Pustakawan Ahli Pertama</v>
@@ -70948,7 +70948,7 @@
     </row>
     <row r="1854">
       <c r="A1854" t="str">
-        <v>Kmti9zgfw2iij</v>
+        <v>Kmtia02g5847t</v>
       </c>
       <c r="B1854" t="str">
         <v>Pustakawan Penyelia</v>
@@ -70986,7 +70986,7 @@
     </row>
     <row r="1855">
       <c r="A1855" t="str">
-        <v>Kmti9zgfwyyps</v>
+        <v>Kmtia02g5esxu</v>
       </c>
       <c r="B1855" t="str">
         <v>Pustakawan Mahir</v>
@@ -71024,7 +71024,7 @@
     </row>
     <row r="1856">
       <c r="A1856" t="str">
-        <v>Kmti9zgfwjo3x</v>
+        <v>Kmtia02g5xv9d</v>
       </c>
       <c r="B1856" t="str">
         <v>Pustakawan Terampil</v>
@@ -71138,7 +71138,7 @@
     </row>
     <row r="1859">
       <c r="A1859" t="str">
-        <v>Kmti9zgfw0xyq</v>
+        <v>Kmtia02g5751t</v>
       </c>
       <c r="B1859" t="str">
         <v>Penata Layanan Operasional</v>
@@ -71176,7 +71176,7 @@
     </row>
     <row r="1860">
       <c r="A1860" t="str">
-        <v>Kmti9zgfwe6ho</v>
+        <v>Kmtia02g5n6is</v>
       </c>
       <c r="B1860" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71214,7 +71214,7 @@
     </row>
     <row r="1861">
       <c r="A1861" t="str">
-        <v>Kmti9zgfwfgw6</v>
+        <v>Kmtia02g5jo1h</v>
       </c>
       <c r="B1861" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71252,7 +71252,7 @@
     </row>
     <row r="1862">
       <c r="A1862" t="str">
-        <v>Kmti9zgfwla25</v>
+        <v>Kmtia02g5fhzw</v>
       </c>
       <c r="B1862" t="str">
         <v>Penata Keprotokolan*</v>
@@ -71366,7 +71366,7 @@
     </row>
     <row r="1865">
       <c r="A1865" t="str">
-        <v>Kmti9zgfw2nin</v>
+        <v>Kmtia02g52apj</v>
       </c>
       <c r="B1865" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -71404,7 +71404,7 @@
     </row>
     <row r="1866">
       <c r="A1866" t="str">
-        <v>Kmti9zgfw7zit</v>
+        <v>Kmtia02g51nt1</v>
       </c>
       <c r="B1866" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71442,7 +71442,7 @@
     </row>
     <row r="1867">
       <c r="A1867" t="str">
-        <v>Kmti9zgfwii39</v>
+        <v>Kmtia02g543v3</v>
       </c>
       <c r="B1867" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71518,7 +71518,7 @@
     </row>
     <row r="1869">
       <c r="A1869" t="str">
-        <v>Kmti9zgfwzuwq</v>
+        <v>Kmtia02g5ufdv</v>
       </c>
       <c r="B1869" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -71556,7 +71556,7 @@
     </row>
     <row r="1870">
       <c r="A1870" t="str">
-        <v>Kmti9zgfwlnqc</v>
+        <v>Kmtia02g5h0pq</v>
       </c>
       <c r="B1870" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71594,7 +71594,7 @@
     </row>
     <row r="1871">
       <c r="A1871" t="str">
-        <v>Kmti9zgfwp5sv</v>
+        <v>Kmtia02g52i5g</v>
       </c>
       <c r="B1871" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71632,7 +71632,7 @@
     </row>
     <row r="1872" xml:space="preserve">
       <c r="A1872" t="str">
-        <v>Kmti9zgfw0ds4</v>
+        <v>Kmtia02g5arra</v>
       </c>
       <c r="B1872" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -71671,7 +71671,7 @@
     </row>
     <row r="1873" xml:space="preserve">
       <c r="A1873" t="str">
-        <v>Kmti9zgfwa6fc</v>
+        <v>Kmtia02g5vqpj</v>
       </c>
       <c r="B1873" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -71710,7 +71710,7 @@
     </row>
     <row r="1874" xml:space="preserve">
       <c r="A1874" t="str">
-        <v>Kmti9zgfwajv1</v>
+        <v>Kmtia02g5dw28</v>
       </c>
       <c r="B1874" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -71749,7 +71749,7 @@
     </row>
     <row r="1875" xml:space="preserve">
       <c r="A1875" t="str">
-        <v>Kmti9zgfwc10z</v>
+        <v>Kmtia02g50kef</v>
       </c>
       <c r="B1875" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -71864,7 +71864,7 @@
     </row>
     <row r="1878">
       <c r="A1878" t="str">
-        <v>Kmti9zgfwygzd</v>
+        <v>Kmtia02g5xkth</v>
       </c>
       <c r="B1878" t="str">
         <v>Penata Layanan Operasional</v>
@@ -71902,7 +71902,7 @@
     </row>
     <row r="1879">
       <c r="A1879" t="str">
-        <v>Kmti9zgfwoltt</v>
+        <v>Kmtia02g5w1p4</v>
       </c>
       <c r="B1879" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71940,7 +71940,7 @@
     </row>
     <row r="1880">
       <c r="A1880" t="str">
-        <v>Kmti9zgfwqkai</v>
+        <v>Kmtia02g5emrb</v>
       </c>
       <c r="B1880" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71978,7 +71978,7 @@
     </row>
     <row r="1881">
       <c r="A1881" t="str">
-        <v>Kmti9zgfwypfl</v>
+        <v>Kmtia02g5jwg2</v>
       </c>
       <c r="B1881" t="str">
         <v>Penata Keprotokolan*</v>
@@ -72092,7 +72092,7 @@
     </row>
     <row r="1884">
       <c r="A1884" t="str">
-        <v>Kmti9zgfwhczd</v>
+        <v>Kmtia02g5rr92</v>
       </c>
       <c r="B1884" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -72130,7 +72130,7 @@
     </row>
     <row r="1885">
       <c r="A1885" t="str">
-        <v>Kmti9zgfw7qoi</v>
+        <v>Kmtia02g5z6a2</v>
       </c>
       <c r="B1885" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72168,7 +72168,7 @@
     </row>
     <row r="1886">
       <c r="A1886" t="str">
-        <v>Kmti9zgfwb0ne</v>
+        <v>Kmtia02g5c1v6</v>
       </c>
       <c r="B1886" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72244,7 +72244,7 @@
     </row>
     <row r="1888">
       <c r="A1888" t="str">
-        <v>Kmti9zgfwonwb</v>
+        <v>Kmtia02g5yd27</v>
       </c>
       <c r="B1888" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -72282,7 +72282,7 @@
     </row>
     <row r="1889">
       <c r="A1889" t="str">
-        <v>Kmti9zgfwmcx1</v>
+        <v>Kmtia02g5sdjj</v>
       </c>
       <c r="B1889" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72320,7 +72320,7 @@
     </row>
     <row r="1890">
       <c r="A1890" t="str">
-        <v>Kmti9zgfwvgey</v>
+        <v>Kmtia02g5rlp6</v>
       </c>
       <c r="B1890" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72358,7 +72358,7 @@
     </row>
     <row r="1891" xml:space="preserve">
       <c r="A1891" t="str">
-        <v>Kmti9zgfwhsjl</v>
+        <v>Kmtia02g5gw3m</v>
       </c>
       <c r="B1891" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -72397,7 +72397,7 @@
     </row>
     <row r="1892" xml:space="preserve">
       <c r="A1892" t="str">
-        <v>Kmti9zgfwz45u</v>
+        <v>Kmtia02g5ycyf</v>
       </c>
       <c r="B1892" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -72436,7 +72436,7 @@
     </row>
     <row r="1893" xml:space="preserve">
       <c r="A1893" t="str">
-        <v>Kmti9zgfwkdjf</v>
+        <v>Kmtia02g5xp44</v>
       </c>
       <c r="B1893" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -72475,7 +72475,7 @@
     </row>
     <row r="1894" xml:space="preserve">
       <c r="A1894" t="str">
-        <v>Kmti9zgfwqky1</v>
+        <v>Kmtia02g5po7x</v>
       </c>
       <c r="B1894" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -72590,7 +72590,7 @@
     </row>
     <row r="1897">
       <c r="A1897" t="str">
-        <v>Kmti9zgfwdg9m</v>
+        <v>Kmtia02g5jnvm</v>
       </c>
       <c r="B1897" t="str">
         <v>Penata Layanan Operasional</v>
@@ -72628,7 +72628,7 @@
     </row>
     <row r="1898">
       <c r="A1898" t="str">
-        <v>Kmti9zgfw93o7</v>
+        <v>Kmtia02g5tu8l</v>
       </c>
       <c r="B1898" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72666,7 +72666,7 @@
     </row>
     <row r="1899">
       <c r="A1899" t="str">
-        <v>Kmti9zgfw3rvs</v>
+        <v>Kmtia02g59zte</v>
       </c>
       <c r="B1899" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72704,7 +72704,7 @@
     </row>
     <row r="1900">
       <c r="A1900" t="str">
-        <v>Kmti9zgfwaiyz</v>
+        <v>Kmtia02g54rf9</v>
       </c>
       <c r="B1900" t="str">
         <v>Penata Keprotokolan*</v>
@@ -72818,7 +72818,7 @@
     </row>
     <row r="1903">
       <c r="A1903" t="str">
-        <v>Kmti9zgfwqae2</v>
+        <v>Kmtia02g5eucu</v>
       </c>
       <c r="B1903" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -72856,7 +72856,7 @@
     </row>
     <row r="1904">
       <c r="A1904" t="str">
-        <v>Kmti9zgfwd4z6</v>
+        <v>Kmtia02g5xv40</v>
       </c>
       <c r="B1904" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72894,7 +72894,7 @@
     </row>
     <row r="1905">
       <c r="A1905" t="str">
-        <v>Kmti9zgfw2ujl</v>
+        <v>Kmtia02g5tio4</v>
       </c>
       <c r="B1905" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72970,7 +72970,7 @@
     </row>
     <row r="1907">
       <c r="A1907" t="str">
-        <v>Kmti9zgfw9m04</v>
+        <v>Kmtia02g52b6t</v>
       </c>
       <c r="B1907" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -73008,7 +73008,7 @@
     </row>
     <row r="1908">
       <c r="A1908" t="str">
-        <v>Kmti9zgfwx768</v>
+        <v>Kmtia02g5xi3c</v>
       </c>
       <c r="B1908" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73046,7 +73046,7 @@
     </row>
     <row r="1909">
       <c r="A1909" t="str">
-        <v>Kmti9zgfwvkwj</v>
+        <v>Kmtia02g5ju1t</v>
       </c>
       <c r="B1909" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73084,7 +73084,7 @@
     </row>
     <row r="1910" xml:space="preserve">
       <c r="A1910" t="str">
-        <v>Kmti9zgfw6b8v</v>
+        <v>Kmtia02g5j8e4</v>
       </c>
       <c r="B1910" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -73123,7 +73123,7 @@
     </row>
     <row r="1911" xml:space="preserve">
       <c r="A1911" t="str">
-        <v>Kmti9zgfwsy1c</v>
+        <v>Kmtia02g5lo7f</v>
       </c>
       <c r="B1911" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -73162,7 +73162,7 @@
     </row>
     <row r="1912" xml:space="preserve">
       <c r="A1912" t="str">
-        <v>Kmti9zgfw5kvp</v>
+        <v>Kmtia02g54w5v</v>
       </c>
       <c r="B1912" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -73201,7 +73201,7 @@
     </row>
     <row r="1913" xml:space="preserve">
       <c r="A1913" t="str">
-        <v>Kmti9zgfwz84e</v>
+        <v>Kmtia02g5tsmj</v>
       </c>
       <c r="B1913" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -73316,7 +73316,7 @@
     </row>
     <row r="1916">
       <c r="A1916" t="str">
-        <v>Kmti9zgfwbw3m</v>
+        <v>Kmtia02g67x9r</v>
       </c>
       <c r="B1916" t="str">
         <v>Penata Layanan Operasional</v>
@@ -73354,7 +73354,7 @@
     </row>
     <row r="1917">
       <c r="A1917" t="str">
-        <v>Kmti9zgfwkfny</v>
+        <v>Kmtia02g6l4mu</v>
       </c>
       <c r="B1917" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73392,7 +73392,7 @@
     </row>
     <row r="1918">
       <c r="A1918" t="str">
-        <v>Kmti9zgfwcyo6</v>
+        <v>Kmtia02g6fhzw</v>
       </c>
       <c r="B1918" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73430,7 +73430,7 @@
     </row>
     <row r="1919">
       <c r="A1919" t="str">
-        <v>Kmti9zgfw0tnz</v>
+        <v>Kmtia02g6xz2g</v>
       </c>
       <c r="B1919" t="str">
         <v>Penata Keprotokolan*</v>
@@ -73544,7 +73544,7 @@
     </row>
     <row r="1922">
       <c r="A1922" t="str">
-        <v>Kmti9zgfwltys</v>
+        <v>Kmtia02g6mfnb</v>
       </c>
       <c r="B1922" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -73582,7 +73582,7 @@
     </row>
     <row r="1923">
       <c r="A1923" t="str">
-        <v>Kmti9zgfwlv3o</v>
+        <v>Kmtia02g6sda7</v>
       </c>
       <c r="B1923" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73620,7 +73620,7 @@
     </row>
     <row r="1924">
       <c r="A1924" t="str">
-        <v>Kmti9zgfwjioh</v>
+        <v>Kmtia02g6m9u1</v>
       </c>
       <c r="B1924" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73696,7 +73696,7 @@
     </row>
     <row r="1926">
       <c r="A1926" t="str">
-        <v>Kmti9zgfw06pe</v>
+        <v>Kmtia02g6uvuq</v>
       </c>
       <c r="B1926" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -73734,7 +73734,7 @@
     </row>
     <row r="1927">
       <c r="A1927" t="str">
-        <v>Kmti9zgfwuj6q</v>
+        <v>Kmtia02g65myt</v>
       </c>
       <c r="B1927" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73772,7 +73772,7 @@
     </row>
     <row r="1928">
       <c r="A1928" t="str">
-        <v>Kmti9zgfw033o</v>
+        <v>Kmtia02g6oiwu</v>
       </c>
       <c r="B1928" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73810,7 +73810,7 @@
     </row>
     <row r="1929" xml:space="preserve">
       <c r="A1929" t="str">
-        <v>Kmti9zgfwjjey</v>
+        <v>Kmtia02g6s09i</v>
       </c>
       <c r="B1929" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -73849,7 +73849,7 @@
     </row>
     <row r="1930" xml:space="preserve">
       <c r="A1930" t="str">
-        <v>Kmti9zgfwnnpn</v>
+        <v>Kmtia02g6x36c</v>
       </c>
       <c r="B1930" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -73888,7 +73888,7 @@
     </row>
     <row r="1931" xml:space="preserve">
       <c r="A1931" t="str">
-        <v>Kmti9zgfw6gap</v>
+        <v>Kmtia02g6x3zw</v>
       </c>
       <c r="B1931" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -73927,7 +73927,7 @@
     </row>
     <row r="1932" xml:space="preserve">
       <c r="A1932" t="str">
-        <v>Kmti9zgfwoabt</v>
+        <v>Kmtia02g6iuxz</v>
       </c>
       <c r="B1932" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -73966,7 +73966,7 @@
     </row>
     <row r="1933" xml:space="preserve">
       <c r="A1933" t="str">
-        <v>Kmti9zgfww5t6</v>
+        <v>Kmtia02g6rzrv</v>
       </c>
       <c r="B1933" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Madya/_x000d_
@@ -74005,7 +74005,7 @@
     </row>
     <row r="1934" xml:space="preserve">
       <c r="A1934" t="str">
-        <v>Kmti9zgfwyfcf</v>
+        <v>Kmtia02g68m2x</v>
       </c>
       <c r="B1934" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -74044,7 +74044,7 @@
     </row>
     <row r="1935" xml:space="preserve">
       <c r="A1935" t="str">
-        <v>Kmti9zgfw2bzn</v>
+        <v>Kmtia02g6b66o</v>
       </c>
       <c r="B1935" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -74159,7 +74159,7 @@
     </row>
     <row r="1938">
       <c r="A1938" t="str">
-        <v>Kmti9zgfwe6jk</v>
+        <v>Kmtia02g6ix1r</v>
       </c>
       <c r="B1938" t="str">
         <v>Penata Layanan Operasional</v>
@@ -74197,7 +74197,7 @@
     </row>
     <row r="1939">
       <c r="A1939" t="str">
-        <v>Kmti9zgfwnr3v</v>
+        <v>Kmtia02g6bevy</v>
       </c>
       <c r="B1939" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -74235,7 +74235,7 @@
     </row>
     <row r="1940">
       <c r="A1940" t="str">
-        <v>Kmti9zgfw1j05</v>
+        <v>Kmtia02g6gfob</v>
       </c>
       <c r="B1940" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -74273,7 +74273,7 @@
     </row>
     <row r="1941">
       <c r="A1941" t="str">
-        <v>Kmti9zgfw5rbq</v>
+        <v>Kmtia02g69792</v>
       </c>
       <c r="B1941" t="str">
         <v>Penata Keprotokolan*</v>
@@ -74387,7 +74387,7 @@
     </row>
     <row r="1944">
       <c r="A1944" t="str">
-        <v>Kmti9zgfwfb0h</v>
+        <v>Kmtia02g634r5</v>
       </c>
       <c r="B1944" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -74425,7 +74425,7 @@
     </row>
     <row r="1945">
       <c r="A1945" t="str">
-        <v>Kmti9zgfw1aqi</v>
+        <v>Kmtia02g69to5</v>
       </c>
       <c r="B1945" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -74463,7 +74463,7 @@
     </row>
     <row r="1946">
       <c r="A1946" t="str">
-        <v>Kmti9zgfwxvsl</v>
+        <v>Kmtia02g6j9iw</v>
       </c>
       <c r="B1946" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -74539,7 +74539,7 @@
     </row>
     <row r="1948">
       <c r="A1948" t="str">
-        <v>Kmti9zgfwixeo</v>
+        <v>Kmtia02g6yxsa</v>
       </c>
       <c r="B1948" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -74577,7 +74577,7 @@
     </row>
     <row r="1949">
       <c r="A1949" t="str">
-        <v>Kmti9zgfwztsm</v>
+        <v>Kmtia02g6c24a</v>
       </c>
       <c r="B1949" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -74615,7 +74615,7 @@
     </row>
     <row r="1950">
       <c r="A1950" t="str">
-        <v>Kmti9zgfwjky0</v>
+        <v>Kmtia02g6uyjx</v>
       </c>
       <c r="B1950" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -74653,7 +74653,7 @@
     </row>
     <row r="1951" xml:space="preserve">
       <c r="A1951" t="str">
-        <v>Kmti9zgfwql8b</v>
+        <v>Kmtia02g60w4t</v>
       </c>
       <c r="B1951" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -74692,7 +74692,7 @@
     </row>
     <row r="1952" xml:space="preserve">
       <c r="A1952" t="str">
-        <v>Kmti9zgfwb0ad</v>
+        <v>Kmtia02g6jo7p</v>
       </c>
       <c r="B1952" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -74731,7 +74731,7 @@
     </row>
     <row r="1953" xml:space="preserve">
       <c r="A1953" t="str">
-        <v>Kmti9zgfwr31d</v>
+        <v>Kmtia02g6zxp9</v>
       </c>
       <c r="B1953" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -74770,7 +74770,7 @@
     </row>
     <row r="1954" xml:space="preserve">
       <c r="A1954" t="str">
-        <v>Kmti9zgfwr8in</v>
+        <v>Kmtia02g64hhx</v>
       </c>
       <c r="B1954" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -74809,7 +74809,7 @@
     </row>
     <row r="1955" xml:space="preserve">
       <c r="A1955" t="str">
-        <v>Kmti9zgfwtaz2</v>
+        <v>Kmtia02g6vv0j</v>
       </c>
       <c r="B1955" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Madya/_x000d_
@@ -74848,7 +74848,7 @@
     </row>
     <row r="1956" xml:space="preserve">
       <c r="A1956" t="str">
-        <v>Kmti9zgfwqbyo</v>
+        <v>Kmtia02g6i9p7</v>
       </c>
       <c r="B1956" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -74887,7 +74887,7 @@
     </row>
     <row r="1957" xml:space="preserve">
       <c r="A1957" t="str">
-        <v>Kmti9zgfw8hv9</v>
+        <v>Kmtia02g6t9dv</v>
       </c>
       <c r="B1957" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -75002,7 +75002,7 @@
     </row>
     <row r="1960">
       <c r="A1960" t="str">
-        <v>Kmti9zgfwct15</v>
+        <v>Kmtia02g6fz4z</v>
       </c>
       <c r="B1960" t="str">
         <v>Penata Layanan Operasional</v>
@@ -75040,7 +75040,7 @@
     </row>
     <row r="1961">
       <c r="A1961" t="str">
-        <v>Kmti9zgfwa9hm</v>
+        <v>Kmtia02g66nrd</v>
       </c>
       <c r="B1961" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75078,7 +75078,7 @@
     </row>
     <row r="1962">
       <c r="A1962" t="str">
-        <v>Kmti9zgfwlm30</v>
+        <v>Kmtia02g6jop0</v>
       </c>
       <c r="B1962" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75116,7 +75116,7 @@
     </row>
     <row r="1963">
       <c r="A1963" t="str">
-        <v>Kmti9zgfwqbvg</v>
+        <v>Kmtia02g6klnl</v>
       </c>
       <c r="B1963" t="str">
         <v>Penata Keprotokolan*</v>
@@ -75230,7 +75230,7 @@
     </row>
     <row r="1966">
       <c r="A1966" t="str">
-        <v>Kmti9zgfws9sa</v>
+        <v>Kmtia02g6ov06</v>
       </c>
       <c r="B1966" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -75268,7 +75268,7 @@
     </row>
     <row r="1967">
       <c r="A1967" t="str">
-        <v>Kmti9zgfwash5</v>
+        <v>Kmtia02g6yv4s</v>
       </c>
       <c r="B1967" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75306,7 +75306,7 @@
     </row>
     <row r="1968">
       <c r="A1968" t="str">
-        <v>Kmti9zgfwquo0</v>
+        <v>Kmtia02g6kky4</v>
       </c>
       <c r="B1968" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75382,7 +75382,7 @@
     </row>
     <row r="1970">
       <c r="A1970" t="str">
-        <v>Kmti9zgfwup3i</v>
+        <v>Kmtia02g6cqkx</v>
       </c>
       <c r="B1970" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -75420,7 +75420,7 @@
     </row>
     <row r="1971">
       <c r="A1971" t="str">
-        <v>Kmti9zgfwef5s</v>
+        <v>Kmtia02g6q0vj</v>
       </c>
       <c r="B1971" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75458,7 +75458,7 @@
     </row>
     <row r="1972">
       <c r="A1972" t="str">
-        <v>Kmti9zgfwwtwu</v>
+        <v>Kmtia02g6mn3p</v>
       </c>
       <c r="B1972" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75496,7 +75496,7 @@
     </row>
     <row r="1973" xml:space="preserve">
       <c r="A1973" t="str">
-        <v>Kmti9zgfw75iy</v>
+        <v>Kmtia02g6gtj3</v>
       </c>
       <c r="B1973" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -75535,7 +75535,7 @@
     </row>
     <row r="1974" xml:space="preserve">
       <c r="A1974" t="str">
-        <v>Kmti9zgfwt3u7</v>
+        <v>Kmtia02g61exi</v>
       </c>
       <c r="B1974" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -75574,7 +75574,7 @@
     </row>
     <row r="1975" xml:space="preserve">
       <c r="A1975" t="str">
-        <v>Kmti9zgfwetaa</v>
+        <v>Kmtia02g6dxfe</v>
       </c>
       <c r="B1975" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -75613,7 +75613,7 @@
     </row>
     <row r="1976" xml:space="preserve">
       <c r="A1976" t="str">
-        <v>Kmti9zgfwckqd</v>
+        <v>Kmtia02g6ubih</v>
       </c>
       <c r="B1976" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -75728,7 +75728,7 @@
     </row>
     <row r="1979">
       <c r="A1979" t="str">
-        <v>Kmti9zgfwvci0</v>
+        <v>Kmtia02g6t1vj</v>
       </c>
       <c r="B1979" t="str">
         <v>Penata Layanan Operasional</v>
@@ -75766,7 +75766,7 @@
     </row>
     <row r="1980">
       <c r="A1980" t="str">
-        <v>Kmti9zgfw7psj</v>
+        <v>Kmtia02g6vjq0</v>
       </c>
       <c r="B1980" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75804,7 +75804,7 @@
     </row>
     <row r="1981">
       <c r="A1981" t="str">
-        <v>Kmti9zgfw0gqv</v>
+        <v>Kmtia02g6o1h4</v>
       </c>
       <c r="B1981" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75842,7 +75842,7 @@
     </row>
     <row r="1982">
       <c r="A1982" t="str">
-        <v>Kmti9zgfw1kr2</v>
+        <v>Kmtia02g6ufxj</v>
       </c>
       <c r="B1982" t="str">
         <v>Penata Keprotokolan*</v>
@@ -75956,7 +75956,7 @@
     </row>
     <row r="1985">
       <c r="A1985" t="str">
-        <v>Kmti9zgfwryyh</v>
+        <v>Kmtia02g6eqwo</v>
       </c>
       <c r="B1985" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -75994,7 +75994,7 @@
     </row>
     <row r="1986">
       <c r="A1986" t="str">
-        <v>Kmti9zgfwff1h</v>
+        <v>Kmtia02g656ap</v>
       </c>
       <c r="B1986" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76032,7 +76032,7 @@
     </row>
     <row r="1987">
       <c r="A1987" t="str">
-        <v>Kmti9zgfw6v3w</v>
+        <v>Kmtia02g62ruv</v>
       </c>
       <c r="B1987" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76108,7 +76108,7 @@
     </row>
     <row r="1989">
       <c r="A1989" t="str">
-        <v>Kmti9zgfw9zoj</v>
+        <v>Kmtia02g6f242</v>
       </c>
       <c r="B1989" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -76146,7 +76146,7 @@
     </row>
     <row r="1990">
       <c r="A1990" t="str">
-        <v>Kmti9zgfwyso0</v>
+        <v>Kmtia02g6bh6y</v>
       </c>
       <c r="B1990" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76184,7 +76184,7 @@
     </row>
     <row r="1991">
       <c r="A1991" t="str">
-        <v>Kmti9zgfwugsv</v>
+        <v>Kmtia02g6tcdt</v>
       </c>
       <c r="B1991" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76222,7 +76222,7 @@
     </row>
     <row r="1992" xml:space="preserve">
       <c r="A1992" t="str">
-        <v>Kmti9zgfw6fhy</v>
+        <v>Kmtia02g6qn01</v>
       </c>
       <c r="B1992" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -76261,7 +76261,7 @@
     </row>
     <row r="1993" xml:space="preserve">
       <c r="A1993" t="str">
-        <v>Kmti9zgfwexxz</v>
+        <v>Kmtia02g690ph</v>
       </c>
       <c r="B1993" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -76300,7 +76300,7 @@
     </row>
     <row r="1994" xml:space="preserve">
       <c r="A1994" t="str">
-        <v>Kmti9zgfwx8ig</v>
+        <v>Kmtia02g63qre</v>
       </c>
       <c r="B1994" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -76339,7 +76339,7 @@
     </row>
     <row r="1995" xml:space="preserve">
       <c r="A1995" t="str">
-        <v>Kmti9zgfwt7iw</v>
+        <v>Kmtia02g69f8a</v>
       </c>
       <c r="B1995" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -76454,7 +76454,7 @@
     </row>
     <row r="1998">
       <c r="A1998" t="str">
-        <v>Kmti9zgfw4cxt</v>
+        <v>Kmtia02g66bb0</v>
       </c>
       <c r="B1998" t="str">
         <v>Penata Layanan Operasional</v>
@@ -76492,7 +76492,7 @@
     </row>
     <row r="1999">
       <c r="A1999" t="str">
-        <v>Kmti9zgfwxx46</v>
+        <v>Kmtia02g6cgaj</v>
       </c>
       <c r="B1999" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76530,7 +76530,7 @@
     </row>
     <row r="2000">
       <c r="A2000" t="str">
-        <v>Kmti9zgfwdx4b</v>
+        <v>Kmtia02g6wnsc</v>
       </c>
       <c r="B2000" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76568,7 +76568,7 @@
     </row>
     <row r="2001">
       <c r="A2001" t="str">
-        <v>Kmti9zgfwuima</v>
+        <v>Kmtia02g6wqz2</v>
       </c>
       <c r="B2001" t="str">
         <v>Penata Keprotokolan*</v>
@@ -76682,7 +76682,7 @@
     </row>
     <row r="2004">
       <c r="A2004" t="str">
-        <v>Kmti9zgfwtjyt</v>
+        <v>Kmtia02g6vn1p</v>
       </c>
       <c r="B2004" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -76720,7 +76720,7 @@
     </row>
     <row r="2005">
       <c r="A2005" t="str">
-        <v>Kmti9zgfx25jb</v>
+        <v>Kmtia02g6lyqk</v>
       </c>
       <c r="B2005" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76758,7 +76758,7 @@
     </row>
     <row r="2006">
       <c r="A2006" t="str">
-        <v>Kmti9zgfxvr5x</v>
+        <v>Kmtia02g67sbl</v>
       </c>
       <c r="B2006" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76834,7 +76834,7 @@
     </row>
     <row r="2008">
       <c r="A2008" t="str">
-        <v>Kmti9zgfx60nq</v>
+        <v>Kmtia02g6wg95</v>
       </c>
       <c r="B2008" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -76872,7 +76872,7 @@
     </row>
     <row r="2009">
       <c r="A2009" t="str">
-        <v>Kmti9zgfx5fvs</v>
+        <v>Kmtia02g6tyo0</v>
       </c>
       <c r="B2009" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76910,7 +76910,7 @@
     </row>
     <row r="2010">
       <c r="A2010" t="str">
-        <v>Kmti9zgfx8g5q</v>
+        <v>Kmtia02g6j3y3</v>
       </c>
       <c r="B2010" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76948,7 +76948,7 @@
     </row>
     <row r="2011" xml:space="preserve">
       <c r="A2011" t="str">
-        <v>Kmti9zgfxshjn</v>
+        <v>Kmtia02g6ftgs</v>
       </c>
       <c r="B2011" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -76987,7 +76987,7 @@
     </row>
     <row r="2012" xml:space="preserve">
       <c r="A2012" t="str">
-        <v>Kmti9zgfxrkcb</v>
+        <v>Kmtia02g6iwfs</v>
       </c>
       <c r="B2012" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -77026,7 +77026,7 @@
     </row>
     <row r="2013" xml:space="preserve">
       <c r="A2013" t="str">
-        <v>Kmti9zgfx1osk</v>
+        <v>Kmtia02g6ij3d</v>
       </c>
       <c r="B2013" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -77065,7 +77065,7 @@
     </row>
     <row r="2014" xml:space="preserve">
       <c r="A2014" t="str">
-        <v>Kmti9zgfx01sb</v>
+        <v>Kmtia02g61wcy</v>
       </c>
       <c r="B2014" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -77180,7 +77180,7 @@
     </row>
     <row r="2017">
       <c r="A2017" t="str">
-        <v>Kmti9zgfxxidv</v>
+        <v>Kmtia02g6jmi4</v>
       </c>
       <c r="B2017" t="str">
         <v>Penata Layanan Operasional</v>
@@ -77218,7 +77218,7 @@
     </row>
     <row r="2018">
       <c r="A2018" t="str">
-        <v>Kmti9zgfxnyrh</v>
+        <v>Kmtia02g6ivzc</v>
       </c>
       <c r="B2018" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -77256,7 +77256,7 @@
     </row>
     <row r="2019">
       <c r="A2019" t="str">
-        <v>Kmti9zgfxvb34</v>
+        <v>Kmtia02g65mjt</v>
       </c>
       <c r="B2019" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -77294,7 +77294,7 @@
     </row>
     <row r="2020">
       <c r="A2020" t="str">
-        <v>Kmti9zgfxoj9b</v>
+        <v>Kmtia02g6f6p9</v>
       </c>
       <c r="B2020" t="str">
         <v>Penata Keprotokolan*</v>
@@ -77408,7 +77408,7 @@
     </row>
     <row r="2023">
       <c r="A2023" t="str">
-        <v>Kmti9zgfxkbvv</v>
+        <v>Kmtia02g65q8m</v>
       </c>
       <c r="B2023" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -77446,7 +77446,7 @@
     </row>
     <row r="2024">
       <c r="A2024" t="str">
-        <v>Kmti9zgfxhm06</v>
+        <v>Kmtia02g62e4f</v>
       </c>
       <c r="B2024" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -77484,7 +77484,7 @@
     </row>
     <row r="2025">
       <c r="A2025" t="str">
-        <v>Kmti9zgfx63dk</v>
+        <v>Kmtia02g6azc8</v>
       </c>
       <c r="B2025" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -77560,7 +77560,7 @@
     </row>
     <row r="2027">
       <c r="A2027" t="str">
-        <v>Kmti9zgfxupom</v>
+        <v>Kmtia02g6w5gk</v>
       </c>
       <c r="B2027" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -77598,7 +77598,7 @@
     </row>
     <row r="2028">
       <c r="A2028" t="str">
-        <v>Kmti9zgfxovu8</v>
+        <v>Kmtia02g6on0i</v>
       </c>
       <c r="B2028" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -77636,7 +77636,7 @@
     </row>
     <row r="2029">
       <c r="A2029" t="str">
-        <v>Kmti9zgfxwy6o</v>
+        <v>Kmtia02g6f17q</v>
       </c>
       <c r="B2029" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -77674,7 +77674,7 @@
     </row>
     <row r="2030" xml:space="preserve">
       <c r="A2030" t="str">
-        <v>Kmti9zgfxflrx</v>
+        <v>Kmtia02g6202h</v>
       </c>
       <c r="B2030" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -77713,7 +77713,7 @@
     </row>
     <row r="2031" xml:space="preserve">
       <c r="A2031" t="str">
-        <v>Kmti9zgfxc1b3</v>
+        <v>Kmtia02g6cj3j</v>
       </c>
       <c r="B2031" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -77752,7 +77752,7 @@
     </row>
     <row r="2032" xml:space="preserve">
       <c r="A2032" t="str">
-        <v>Kmti9zgfxt41q</v>
+        <v>Kmtia02g6cz8d</v>
       </c>
       <c r="B2032" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -77791,7 +77791,7 @@
     </row>
     <row r="2033" xml:space="preserve">
       <c r="A2033" t="str">
-        <v>Kmti9zgfxiwy8</v>
+        <v>Kmtia02g6wjtm</v>
       </c>
       <c r="B2033" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -77830,7 +77830,7 @@
     </row>
     <row r="2034">
       <c r="A2034" t="str">
-        <v>Kmti9zgfxmdk5</v>
+        <v>Kmtia02g68p82</v>
       </c>
       <c r="B2034" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Muda</v>
@@ -77868,7 +77868,7 @@
     </row>
     <row r="2035">
       <c r="A2035" t="str">
-        <v>Kmti9zgfxvt2x</v>
+        <v>Kmtia02g6mn0u</v>
       </c>
       <c r="B2035" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Pertama</v>
@@ -77944,7 +77944,7 @@
     </row>
     <row r="2037" xml:space="preserve">
       <c r="A2037" t="str">
-        <v>Kmti9zgfxcf89</v>
+        <v>Kmtia02g6u0rs</v>
       </c>
       <c r="B2037" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_

</xml_diff>

<commit_message>
Perbarui struktur organisasi (2026-09-01T06:18:50.517Z)
</commit_message>
<xml_diff>
--- a/data/struktur-organisasi.xlsx
+++ b/data/struktur-organisasi.xlsx
@@ -63909,7 +63909,7 @@
     </row>
     <row r="1669">
       <c r="A1669" t="str">
-        <v>Kmtia02g5jawg</v>
+        <v>Kmti9zgfv26p3</v>
       </c>
       <c r="B1669" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -63947,7 +63947,7 @@
     </row>
     <row r="1670">
       <c r="A1670" t="str">
-        <v>Kmtia02g5naro</v>
+        <v>Kmti9zgfvwyrb</v>
       </c>
       <c r="B1670" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -63985,7 +63985,7 @@
     </row>
     <row r="1671">
       <c r="A1671" t="str">
-        <v>Kmtia02g5i9oq</v>
+        <v>Kmti9zgfvtx00</v>
       </c>
       <c r="B1671" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -64023,7 +64023,7 @@
     </row>
     <row r="1672">
       <c r="A1672" t="str">
-        <v>Kmtia02g5tdaw</v>
+        <v>Kmti9zgfv4cbb</v>
       </c>
       <c r="B1672" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -64061,7 +64061,7 @@
     </row>
     <row r="1673">
       <c r="A1673" t="str">
-        <v>Kmtia02g5n2em</v>
+        <v>Kmti9zgfv0cd5</v>
       </c>
       <c r="B1673" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -64099,7 +64099,7 @@
     </row>
     <row r="1674">
       <c r="A1674" t="str">
-        <v>Kmtia02g5dqvc</v>
+        <v>Kmti9zgfv45ja</v>
       </c>
       <c r="B1674" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64137,7 +64137,7 @@
     </row>
     <row r="1675">
       <c r="A1675" t="str">
-        <v>Kmtia02g58etg</v>
+        <v>Kmti9zgfv5dbr</v>
       </c>
       <c r="B1675" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64175,7 +64175,7 @@
     </row>
     <row r="1676">
       <c r="A1676" t="str">
-        <v>Kmtia02g5p8rj</v>
+        <v>Kmti9zgfvpxse</v>
       </c>
       <c r="B1676" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -64251,7 +64251,7 @@
     </row>
     <row r="1678">
       <c r="A1678" t="str">
-        <v>Kmtia02g5b6su</v>
+        <v>Kmti9zgfvuuv7</v>
       </c>
       <c r="B1678" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -64289,7 +64289,7 @@
     </row>
     <row r="1679">
       <c r="A1679" t="str">
-        <v>Kmtia02g5fh5r</v>
+        <v>Kmti9zgfvlrdk</v>
       </c>
       <c r="B1679" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -64327,7 +64327,7 @@
     </row>
     <row r="1680">
       <c r="A1680" t="str">
-        <v>Kmtia02g5kbtf</v>
+        <v>Kmti9zgfvbsli</v>
       </c>
       <c r="B1680" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -64365,7 +64365,7 @@
     </row>
     <row r="1681">
       <c r="A1681" t="str">
-        <v>Kmtia02g51e7e</v>
+        <v>Kmti9zgfv70po</v>
       </c>
       <c r="B1681" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -64403,7 +64403,7 @@
     </row>
     <row r="1682">
       <c r="A1682" t="str">
-        <v>Kmtia02g5377n</v>
+        <v>Kmti9zgfveogu</v>
       </c>
       <c r="B1682" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -64441,7 +64441,7 @@
     </row>
     <row r="1683">
       <c r="A1683" t="str">
-        <v>Kmtia02g5j4jj</v>
+        <v>Kmti9zgfvmgxf</v>
       </c>
       <c r="B1683" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64479,7 +64479,7 @@
     </row>
     <row r="1684">
       <c r="A1684" t="str">
-        <v>Kmtia02g5kjjt</v>
+        <v>Kmti9zgfvknli</v>
       </c>
       <c r="B1684" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64517,7 +64517,7 @@
     </row>
     <row r="1685">
       <c r="A1685" t="str">
-        <v>Kmtia02g5qh5e</v>
+        <v>Kmti9zgfvprvh</v>
       </c>
       <c r="B1685" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -64593,7 +64593,7 @@
     </row>
     <row r="1687">
       <c r="A1687" t="str">
-        <v>Kmtia02g5dfjp</v>
+        <v>Kmti9zgfvbb3w</v>
       </c>
       <c r="B1687" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -64631,7 +64631,7 @@
     </row>
     <row r="1688">
       <c r="A1688" t="str">
-        <v>Kmtia02g5dmi3</v>
+        <v>Kmti9zgfvdowe</v>
       </c>
       <c r="B1688" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -64669,7 +64669,7 @@
     </row>
     <row r="1689">
       <c r="A1689" t="str">
-        <v>Kmtia02g5h0s5</v>
+        <v>Kmti9zgfvapml</v>
       </c>
       <c r="B1689" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -64707,7 +64707,7 @@
     </row>
     <row r="1690">
       <c r="A1690" t="str">
-        <v>Kmtia02g5fbah</v>
+        <v>Kmti9zgfv6noy</v>
       </c>
       <c r="B1690" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -64745,7 +64745,7 @@
     </row>
     <row r="1691">
       <c r="A1691" t="str">
-        <v>Kmtia02g5kh36</v>
+        <v>Kmti9zgfvsrt3</v>
       </c>
       <c r="B1691" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -64783,7 +64783,7 @@
     </row>
     <row r="1692">
       <c r="A1692" t="str">
-        <v>Kmtia02g5xi3y</v>
+        <v>Kmti9zgfv7snw</v>
       </c>
       <c r="B1692" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64821,7 +64821,7 @@
     </row>
     <row r="1693">
       <c r="A1693" t="str">
-        <v>Kmtia02g5nhoc</v>
+        <v>Kmti9zgfvijxf</v>
       </c>
       <c r="B1693" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64859,7 +64859,7 @@
     </row>
     <row r="1694">
       <c r="A1694" t="str">
-        <v>Kmtia02g54eq6</v>
+        <v>Kmti9zgfvq82j</v>
       </c>
       <c r="B1694" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -64897,7 +64897,7 @@
     </row>
     <row r="1695">
       <c r="A1695" t="str">
-        <v>Kmtia02g5vltc</v>
+        <v>Kmti9zgfvy2bj</v>
       </c>
       <c r="B1695" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -64935,7 +64935,7 @@
     </row>
     <row r="1696">
       <c r="A1696" t="str">
-        <v>Kmtia02g505c3</v>
+        <v>Kmti9zgfv3xh5</v>
       </c>
       <c r="B1696" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -64973,7 +64973,7 @@
     </row>
     <row r="1697">
       <c r="A1697" t="str">
-        <v>Kmtia02g5vo6a</v>
+        <v>Kmti9zgfv676s</v>
       </c>
       <c r="B1697" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -65087,7 +65087,7 @@
     </row>
     <row r="1700">
       <c r="A1700" t="str">
-        <v>Kmtia02g555dj</v>
+        <v>Kmti9zgfv4f31</v>
       </c>
       <c r="B1700" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -65125,7 +65125,7 @@
     </row>
     <row r="1701">
       <c r="A1701" t="str">
-        <v>Kmtia02g5gq2n</v>
+        <v>Kmti9zgfvaki2</v>
       </c>
       <c r="B1701" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -65163,7 +65163,7 @@
     </row>
     <row r="1702">
       <c r="A1702" t="str">
-        <v>Kmtia02g56jm2</v>
+        <v>Kmti9zgfvljfh</v>
       </c>
       <c r="B1702" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -65201,7 +65201,7 @@
     </row>
     <row r="1703">
       <c r="A1703" t="str">
-        <v>Kmtia02g5ys50</v>
+        <v>Kmti9zgfvbm7i</v>
       </c>
       <c r="B1703" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -65239,7 +65239,7 @@
     </row>
     <row r="1704">
       <c r="A1704" t="str">
-        <v>Kmtia02g59s2o</v>
+        <v>Kmti9zgfvw9hy</v>
       </c>
       <c r="B1704" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -65277,7 +65277,7 @@
     </row>
     <row r="1705">
       <c r="A1705" t="str">
-        <v>Kmtia02g5ezsf</v>
+        <v>Kmti9zgfv2qcb</v>
       </c>
       <c r="B1705" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -65315,7 +65315,7 @@
     </row>
     <row r="1706">
       <c r="A1706" t="str">
-        <v>Kmtia02g54416</v>
+        <v>Kmti9zgfvd8mh</v>
       </c>
       <c r="B1706" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -65353,7 +65353,7 @@
     </row>
     <row r="1707">
       <c r="A1707" t="str">
-        <v>Kmtia02g5m43x</v>
+        <v>Kmti9zgfvc9si</v>
       </c>
       <c r="B1707" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -65391,7 +65391,7 @@
     </row>
     <row r="1708">
       <c r="A1708" t="str">
-        <v>Kmtia02g58zdp</v>
+        <v>Kmti9zgfvawm4</v>
       </c>
       <c r="B1708" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -65429,7 +65429,7 @@
     </row>
     <row r="1709">
       <c r="A1709" t="str">
-        <v>Kmtia02g5um0d</v>
+        <v>Kmti9zgfvu4kv</v>
       </c>
       <c r="B1709" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -65505,7 +65505,7 @@
     </row>
     <row r="1711">
       <c r="A1711" t="str">
-        <v>Kmtia02g5dtlp</v>
+        <v>Kmti9zgfvn91l</v>
       </c>
       <c r="B1711" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -65543,7 +65543,7 @@
     </row>
     <row r="1712">
       <c r="A1712" t="str">
-        <v>Kmtia02g5ug8c</v>
+        <v>Kmti9zgfvy7ll</v>
       </c>
       <c r="B1712" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -65581,7 +65581,7 @@
     </row>
     <row r="1713">
       <c r="A1713" t="str">
-        <v>Kmtia02g5azkf</v>
+        <v>Kmti9zgfv3bkw</v>
       </c>
       <c r="B1713" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -65619,7 +65619,7 @@
     </row>
     <row r="1714">
       <c r="A1714" t="str">
-        <v>Kmtia02g5a723</v>
+        <v>Kmti9zgfvk58c</v>
       </c>
       <c r="B1714" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -65657,7 +65657,7 @@
     </row>
     <row r="1715">
       <c r="A1715" t="str">
-        <v>Kmtia02g5570l</v>
+        <v>Kmti9zgfvg5e1</v>
       </c>
       <c r="B1715" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -65695,7 +65695,7 @@
     </row>
     <row r="1716">
       <c r="A1716" t="str">
-        <v>Kmtia02g5474m</v>
+        <v>Kmti9zgfvk469</v>
       </c>
       <c r="B1716" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -65733,7 +65733,7 @@
     </row>
     <row r="1717">
       <c r="A1717" t="str">
-        <v>Kmtia02g535lj</v>
+        <v>Kmti9zgfwkwkh</v>
       </c>
       <c r="B1717" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -65771,7 +65771,7 @@
     </row>
     <row r="1718">
       <c r="A1718" t="str">
-        <v>Kmtia02g58dyt</v>
+        <v>Kmti9zgfwsx0u</v>
       </c>
       <c r="B1718" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -65847,7 +65847,7 @@
     </row>
     <row r="1720">
       <c r="A1720" t="str">
-        <v>Kmtia02g5g8of</v>
+        <v>Kmti9zgfwr6bz</v>
       </c>
       <c r="B1720" t="str">
         <v>Penata Layanan Operasional</v>
@@ -65885,7 +65885,7 @@
     </row>
     <row r="1721">
       <c r="A1721" t="str">
-        <v>Kmtia02g57dow</v>
+        <v>Kmti9zgfwgsxa</v>
       </c>
       <c r="B1721" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -65923,7 +65923,7 @@
     </row>
     <row r="1722">
       <c r="A1722" t="str">
-        <v>Kmtia02g5v18i</v>
+        <v>Kmti9zgfw4dul</v>
       </c>
       <c r="B1722" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -65961,7 +65961,7 @@
     </row>
     <row r="1723">
       <c r="A1723" t="str">
-        <v>Kmtia02g52jmt</v>
+        <v>Kmti9zgfwowkd</v>
       </c>
       <c r="B1723" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -65999,7 +65999,7 @@
     </row>
     <row r="1724">
       <c r="A1724" t="str">
-        <v>Kmtia02g5ews8</v>
+        <v>Kmti9zgfwsb26</v>
       </c>
       <c r="B1724" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -66037,7 +66037,7 @@
     </row>
     <row r="1725">
       <c r="A1725" t="str">
-        <v>Kmtia02g5cesx</v>
+        <v>Kmti9zgfwaza4</v>
       </c>
       <c r="B1725" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -66075,7 +66075,7 @@
     </row>
     <row r="1726">
       <c r="A1726" t="str">
-        <v>Kmtia02g5n8zw</v>
+        <v>Kmti9zgfwure0</v>
       </c>
       <c r="B1726" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -66113,7 +66113,7 @@
     </row>
     <row r="1727">
       <c r="A1727" t="str">
-        <v>Kmtia02g552t4</v>
+        <v>Kmti9zgfwsb5n</v>
       </c>
       <c r="B1727" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -66189,7 +66189,7 @@
     </row>
     <row r="1729">
       <c r="A1729" t="str">
-        <v>Kmtia02g504v6</v>
+        <v>Kmti9zgfw36rk</v>
       </c>
       <c r="B1729" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -66227,7 +66227,7 @@
     </row>
     <row r="1730">
       <c r="A1730" t="str">
-        <v>Kmtia02g5brv4</v>
+        <v>Kmti9zgfw3xp6</v>
       </c>
       <c r="B1730" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -66265,7 +66265,7 @@
     </row>
     <row r="1731">
       <c r="A1731" t="str">
-        <v>Kmtia02g5gq6m</v>
+        <v>Kmti9zgfwfvik</v>
       </c>
       <c r="B1731" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -66303,7 +66303,7 @@
     </row>
     <row r="1732">
       <c r="A1732" t="str">
-        <v>Kmtia02g5v3hn</v>
+        <v>Kmti9zgfw4593</v>
       </c>
       <c r="B1732" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -66341,7 +66341,7 @@
     </row>
     <row r="1733">
       <c r="A1733" t="str">
-        <v>Kmtia02g5sieb</v>
+        <v>Kmti9zgfw4kki</v>
       </c>
       <c r="B1733" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -66379,7 +66379,7 @@
     </row>
     <row r="1734">
       <c r="A1734" t="str">
-        <v>Kmtia02g5lvtj</v>
+        <v>Kmti9zgfw72q9</v>
       </c>
       <c r="B1734" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -66417,7 +66417,7 @@
     </row>
     <row r="1735">
       <c r="A1735" t="str">
-        <v>Kmtia02g5r2ur</v>
+        <v>Kmti9zgfw0hmg</v>
       </c>
       <c r="B1735" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -66455,7 +66455,7 @@
     </row>
     <row r="1736">
       <c r="A1736" t="str">
-        <v>Kmtia02g5oaqr</v>
+        <v>Kmti9zgfw9jf7</v>
       </c>
       <c r="B1736" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -66493,7 +66493,7 @@
     </row>
     <row r="1737">
       <c r="A1737" t="str">
-        <v>Kmtia02g5n333</v>
+        <v>Kmti9zgfw4y3j</v>
       </c>
       <c r="B1737" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -66531,7 +66531,7 @@
     </row>
     <row r="1738">
       <c r="A1738" t="str">
-        <v>Kmtia02g57e65</v>
+        <v>Kmti9zgfwto78</v>
       </c>
       <c r="B1738" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -66569,7 +66569,7 @@
     </row>
     <row r="1739">
       <c r="A1739" t="str">
-        <v>Kmtia02g5c10j</v>
+        <v>Kmti9zgfw6xgk</v>
       </c>
       <c r="B1739" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -66607,7 +66607,7 @@
     </row>
     <row r="1740">
       <c r="A1740" t="str">
-        <v>Kmtia02g57618</v>
+        <v>Kmti9zgfw57jm</v>
       </c>
       <c r="B1740" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -66645,7 +66645,7 @@
     </row>
     <row r="1741">
       <c r="A1741" t="str">
-        <v>Kmtia02g5bfnx</v>
+        <v>Kmti9zgfwlksp</v>
       </c>
       <c r="B1741" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -66683,7 +66683,7 @@
     </row>
     <row r="1742">
       <c r="A1742" t="str">
-        <v>Kmtia02g5og4z</v>
+        <v>Kmti9zgfwiets</v>
       </c>
       <c r="B1742" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -66721,7 +66721,7 @@
     </row>
     <row r="1743">
       <c r="A1743" t="str">
-        <v>Kmtia02g57n1z</v>
+        <v>Kmti9zgfwmd71</v>
       </c>
       <c r="B1743" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -66835,7 +66835,7 @@
     </row>
     <row r="1746">
       <c r="A1746" t="str">
-        <v>Kmtia02g5uor5</v>
+        <v>Kmti9zgfwph3s</v>
       </c>
       <c r="B1746" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -66873,7 +66873,7 @@
     </row>
     <row r="1747">
       <c r="A1747" t="str">
-        <v>Kmtia02g5kucy</v>
+        <v>Kmti9zgfwkppc</v>
       </c>
       <c r="B1747" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -66911,7 +66911,7 @@
     </row>
     <row r="1748">
       <c r="A1748" t="str">
-        <v>Kmtia02g5quiy</v>
+        <v>Kmti9zgfw0cxv</v>
       </c>
       <c r="B1748" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -66949,7 +66949,7 @@
     </row>
     <row r="1749" xml:space="preserve">
       <c r="A1749" t="str">
-        <v>Kmtia02g5rqqv</v>
+        <v>Kmti9zgfw6ykh</v>
       </c>
       <c r="B1749" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -66988,7 +66988,7 @@
     </row>
     <row r="1750">
       <c r="A1750" t="str">
-        <v>Kmtia02g5y05f</v>
+        <v>Kmti9zgfwrkt3</v>
       </c>
       <c r="B1750" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -67064,7 +67064,7 @@
     </row>
     <row r="1752">
       <c r="A1752" t="str">
-        <v>Kmtia02g5mc4x</v>
+        <v>Kmti9zgfw2txy</v>
       </c>
       <c r="B1752" t="str">
         <v>Penata Layanan Operasional</v>
@@ -67102,7 +67102,7 @@
     </row>
     <row r="1753">
       <c r="A1753" t="str">
-        <v>Kmtia02g5ooyp</v>
+        <v>Kmti9zgfw3olu</v>
       </c>
       <c r="B1753" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -67140,7 +67140,7 @@
     </row>
     <row r="1754">
       <c r="A1754" t="str">
-        <v>Kmtia02g5f59f</v>
+        <v>Kmti9zgfwyrgw</v>
       </c>
       <c r="B1754" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -67178,7 +67178,7 @@
     </row>
     <row r="1755" xml:space="preserve">
       <c r="A1755" t="str">
-        <v>Kmtia02g5ie9e</v>
+        <v>Kmti9zgfw5xjt</v>
       </c>
       <c r="B1755" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -67217,7 +67217,7 @@
     </row>
     <row r="1756" xml:space="preserve">
       <c r="A1756" t="str">
-        <v>Kmtia02g50k5a</v>
+        <v>Kmti9zgfwukt5</v>
       </c>
       <c r="B1756" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -67256,7 +67256,7 @@
     </row>
     <row r="1757">
       <c r="A1757" t="str">
-        <v>Kmtia02g5qac8</v>
+        <v>Kmti9zgfwffgf</v>
       </c>
       <c r="B1757" t="str">
         <v>Pranata Keuangan APBN Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -67294,7 +67294,7 @@
     </row>
     <row r="1758" xml:space="preserve">
       <c r="A1758" t="str">
-        <v>Kmtia02g5hnhr</v>
+        <v>Kmti9zgfwfrt0</v>
       </c>
       <c r="B1758" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Mahir/_x000d_
@@ -67333,7 +67333,7 @@
     </row>
     <row r="1759" xml:space="preserve">
       <c r="A1759" t="str">
-        <v>Kmtia02g5ow1a</v>
+        <v>Kmti9zgfwqx35</v>
       </c>
       <c r="B1759" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Terampil/_x000d_
@@ -67410,7 +67410,7 @@
     </row>
     <row r="1761">
       <c r="A1761" t="str">
-        <v>Kmtia02g504rl</v>
+        <v>Kmti9zgfwp79t</v>
       </c>
       <c r="B1761" t="str">
         <v>Penata Layanan Operasional</v>
@@ -67448,7 +67448,7 @@
     </row>
     <row r="1762">
       <c r="A1762" t="str">
-        <v>Kmtia02g5z7ob</v>
+        <v>Kmti9zgfw5w0d</v>
       </c>
       <c r="B1762" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -67486,7 +67486,7 @@
     </row>
     <row r="1763">
       <c r="A1763" t="str">
-        <v>Kmtia02g56yb1</v>
+        <v>Kmti9zgfwwc7b</v>
       </c>
       <c r="B1763" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -67524,7 +67524,7 @@
     </row>
     <row r="1764" xml:space="preserve">
       <c r="A1764" t="str">
-        <v>Kmtia02g5l8u6</v>
+        <v>Kmti9zgfwgmis</v>
       </c>
       <c r="B1764" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -67563,7 +67563,7 @@
     </row>
     <row r="1765" xml:space="preserve">
       <c r="A1765" t="str">
-        <v>Kmtia02g5y7sd</v>
+        <v>Kmti9zgfwqfcn</v>
       </c>
       <c r="B1765" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -67602,7 +67602,7 @@
     </row>
     <row r="1766">
       <c r="A1766" t="str">
-        <v>Kmtia02g5iaic</v>
+        <v>Kmti9zgfw8fwd</v>
       </c>
       <c r="B1766" t="str">
         <v>Pranata Keuangan APBN Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -67640,7 +67640,7 @@
     </row>
     <row r="1767" xml:space="preserve">
       <c r="A1767" t="str">
-        <v>Kmtia02g59bdb</v>
+        <v>Kmti9zgfw3a03</v>
       </c>
       <c r="B1767" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Mahir/_x000d_
@@ -67679,7 +67679,7 @@
     </row>
     <row r="1768" xml:space="preserve">
       <c r="A1768" t="str">
-        <v>Kmtia02g5jhar</v>
+        <v>Kmti9zgfwnd9w</v>
       </c>
       <c r="B1768" t="str" xml:space="preserve">
         <v xml:space="preserve">Pranata Keuangan APBN Terampil/_x000d_
@@ -67718,7 +67718,7 @@
     </row>
     <row r="1769">
       <c r="A1769" t="str">
-        <v>Kmtia02g5otlq</v>
+        <v>Kmti9zgfwg7p6</v>
       </c>
       <c r="B1769" t="str">
         <v>Analis Anggaran Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -67756,7 +67756,7 @@
     </row>
     <row r="1770">
       <c r="A1770" t="str">
-        <v>Kmtia02g50c5p</v>
+        <v>Kmti9zgfwlxww</v>
       </c>
       <c r="B1770" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -67794,7 +67794,7 @@
     </row>
     <row r="1771">
       <c r="A1771" t="str">
-        <v>Kmtia02g5fxu8</v>
+        <v>Kmti9zgfweso7</v>
       </c>
       <c r="B1771" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Madya/Pengawas Keuangan Negara Ahli Madya</v>
@@ -67832,7 +67832,7 @@
     </row>
     <row r="1772">
       <c r="A1772" t="str">
-        <v>Kmtia02g51840</v>
+        <v>Kmti9zgfwya1b</v>
       </c>
       <c r="B1772" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Muda/Pengawas Keuangan Negara Ahli Ahli Muda</v>
@@ -67870,7 +67870,7 @@
     </row>
     <row r="1773">
       <c r="A1773" t="str">
-        <v>Kmtia02g54482</v>
+        <v>Kmti9zgfwol0w</v>
       </c>
       <c r="B1773" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Pertama/Pengawas Keuangan Negara Ahli Pertama</v>
@@ -67908,7 +67908,7 @@
     </row>
     <row r="1774">
       <c r="A1774" t="str">
-        <v>Kmtia02g5x7dm</v>
+        <v>Kmti9zgfw4mzw</v>
       </c>
       <c r="B1774" t="str">
         <v>Pranata Keuangan APBN Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -67946,7 +67946,7 @@
     </row>
     <row r="1775">
       <c r="A1775" t="str">
-        <v>Kmtia02g56c0k</v>
+        <v>Kmti9zgfwb5sn</v>
       </c>
       <c r="B1775" t="str">
         <v>Pranata Keuangan APBN Mahir/Pengawas Keuangan Negara Mahir</v>
@@ -67984,7 +67984,7 @@
     </row>
     <row r="1776">
       <c r="A1776" t="str">
-        <v>Kmtia02g57l4j</v>
+        <v>Kmti9zgfw42g7</v>
       </c>
       <c r="B1776" t="str">
         <v>Pranata Keuangan APBN Terampil/Pengawas Keuangan Negara Terampil</v>
@@ -68098,7 +68098,7 @@
     </row>
     <row r="1779">
       <c r="A1779" t="str">
-        <v>Kmtia02g5ijsg</v>
+        <v>Kmti9zgfwgvaq</v>
       </c>
       <c r="B1779" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68136,7 +68136,7 @@
     </row>
     <row r="1780">
       <c r="A1780" t="str">
-        <v>Kmtia02g5q6zy</v>
+        <v>Kmti9zgfw117s</v>
       </c>
       <c r="B1780" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -68174,7 +68174,7 @@
     </row>
     <row r="1781">
       <c r="A1781" t="str">
-        <v>Kmtia02g51nq2</v>
+        <v>Kmti9zgfwc6hl</v>
       </c>
       <c r="B1781" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -68250,7 +68250,7 @@
     </row>
     <row r="1783">
       <c r="A1783" t="str">
-        <v>Kmtia02g5mcdz</v>
+        <v>Kmti9zgfwprkg</v>
       </c>
       <c r="B1783" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68288,7 +68288,7 @@
     </row>
     <row r="1784">
       <c r="A1784" t="str">
-        <v>Kmtia02g57aq0</v>
+        <v>Kmti9zgfwlhys</v>
       </c>
       <c r="B1784" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -68326,7 +68326,7 @@
     </row>
     <row r="1785">
       <c r="A1785" t="str">
-        <v>Kmtia02g548bq</v>
+        <v>Kmti9zgfwkuna</v>
       </c>
       <c r="B1785" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -68364,7 +68364,7 @@
     </row>
     <row r="1786">
       <c r="A1786" t="str">
-        <v>Kmtia02g5em6c</v>
+        <v>Kmti9zgfwluh2</v>
       </c>
       <c r="B1786" t="str">
         <v>Penata Keprotokolan*</v>
@@ -68402,7 +68402,7 @@
     </row>
     <row r="1787">
       <c r="A1787" t="str">
-        <v>Kmtia02g5wbt0</v>
+        <v>Kmti9zgfwg7ii</v>
       </c>
       <c r="B1787" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -68440,7 +68440,7 @@
     </row>
     <row r="1788">
       <c r="A1788" t="str">
-        <v>Kmtia02g5tsuz</v>
+        <v>Kmti9zgfwzqqc</v>
       </c>
       <c r="B1788" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -68478,7 +68478,7 @@
     </row>
     <row r="1789">
       <c r="A1789" t="str">
-        <v>Kmtia02g5zee5</v>
+        <v>Kmti9zgfwg8vo</v>
       </c>
       <c r="B1789" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -68516,7 +68516,7 @@
     </row>
     <row r="1790">
       <c r="A1790" t="str">
-        <v>Kmtia02g5bzk7</v>
+        <v>Kmti9zgfw6kia</v>
       </c>
       <c r="B1790" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -68592,7 +68592,7 @@
     </row>
     <row r="1792">
       <c r="A1792" t="str">
-        <v>Kmtia02g5q7o3</v>
+        <v>Kmti9zgfwvs7f</v>
       </c>
       <c r="B1792" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68630,7 +68630,7 @@
     </row>
     <row r="1793">
       <c r="A1793" t="str">
-        <v>Kmtia02g5t885</v>
+        <v>Kmti9zgfwinbd</v>
       </c>
       <c r="B1793" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -68668,7 +68668,7 @@
     </row>
     <row r="1794">
       <c r="A1794" t="str">
-        <v>Kmtia02g541cu</v>
+        <v>Kmti9zgfwi2a5</v>
       </c>
       <c r="B1794" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -68706,7 +68706,7 @@
     </row>
     <row r="1795">
       <c r="A1795" t="str">
-        <v>Kmtia02g57jxa</v>
+        <v>Kmti9zgfw1s7e</v>
       </c>
       <c r="B1795" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -68744,7 +68744,7 @@
     </row>
     <row r="1796">
       <c r="A1796" t="str">
-        <v>Kmtia02g5wphh</v>
+        <v>Kmti9zgfwtdxj</v>
       </c>
       <c r="B1796" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -68782,7 +68782,7 @@
     </row>
     <row r="1797">
       <c r="A1797" t="str">
-        <v>Kmtia02g5f8fz</v>
+        <v>Kmti9zgfw2ch2</v>
       </c>
       <c r="B1797" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -68820,7 +68820,7 @@
     </row>
     <row r="1798">
       <c r="A1798" t="str">
-        <v>Kmtia02g5hyc0</v>
+        <v>Kmti9zgfwp942</v>
       </c>
       <c r="B1798" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -68858,7 +68858,7 @@
     </row>
     <row r="1799">
       <c r="A1799" t="str">
-        <v>Kmtia02g5lelq</v>
+        <v>Kmti9zgfw2ttx</v>
       </c>
       <c r="B1799" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -68934,7 +68934,7 @@
     </row>
     <row r="1801">
       <c r="A1801" t="str">
-        <v>Kmtia02g5i80r</v>
+        <v>Kmti9zgfw74gb</v>
       </c>
       <c r="B1801" t="str">
         <v>Penata Layanan Operasional</v>
@@ -68972,7 +68972,7 @@
     </row>
     <row r="1802">
       <c r="A1802" t="str">
-        <v>Kmtia02g5mz8o</v>
+        <v>Kmti9zgfwbjjg</v>
       </c>
       <c r="B1802" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -69010,7 +69010,7 @@
     </row>
     <row r="1803">
       <c r="A1803" t="str">
-        <v>Kmtia02g59ck3</v>
+        <v>Kmti9zgfwrqwo</v>
       </c>
       <c r="B1803" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -69048,7 +69048,7 @@
     </row>
     <row r="1804">
       <c r="A1804" t="str">
-        <v>Kmtia02g5851z</v>
+        <v>Kmti9zgfwhexu</v>
       </c>
       <c r="B1804" t="str">
         <v>Penata Keprotokolan*</v>
@@ -69086,7 +69086,7 @@
     </row>
     <row r="1805">
       <c r="A1805" t="str">
-        <v>Kmtia02g528yh</v>
+        <v>Kmti9zgfwdna0</v>
       </c>
       <c r="B1805" t="str">
         <v>Arsiparis Ahli Muda</v>
@@ -69124,7 +69124,7 @@
     </row>
     <row r="1806">
       <c r="A1806" t="str">
-        <v>Kmtia02g5g3cc</v>
+        <v>Kmti9zgfwxez5</v>
       </c>
       <c r="B1806" t="str">
         <v>Arsiparis Ahli Pertama</v>
@@ -69162,7 +69162,7 @@
     </row>
     <row r="1807">
       <c r="A1807" t="str">
-        <v>Kmtia02g5qi08</v>
+        <v>Kmti9zgfwy5z6</v>
       </c>
       <c r="B1807" t="str">
         <v>Arsiparis Penyelia</v>
@@ -69200,7 +69200,7 @@
     </row>
     <row r="1808">
       <c r="A1808" t="str">
-        <v>Kmtia02g5tf66</v>
+        <v>Kmti9zgfw5cy1</v>
       </c>
       <c r="B1808" t="str">
         <v>Arsiparis Mahir</v>
@@ -69238,7 +69238,7 @@
     </row>
     <row r="1809">
       <c r="A1809" t="str">
-        <v>Kmtia02g5en5p</v>
+        <v>Kmti9zgfweff0</v>
       </c>
       <c r="B1809" t="str">
         <v>Arsiparis Terampil</v>
@@ -69276,7 +69276,7 @@
     </row>
     <row r="1810">
       <c r="A1810" t="str">
-        <v>Kmtia02g54v75</v>
+        <v>Kmti9zgfwfxcr</v>
       </c>
       <c r="B1810" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -69314,7 +69314,7 @@
     </row>
     <row r="1811">
       <c r="A1811" t="str">
-        <v>Kmtia02g59puy</v>
+        <v>Kmti9zgfwj2pm</v>
       </c>
       <c r="B1811" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -69352,7 +69352,7 @@
     </row>
     <row r="1812">
       <c r="A1812" t="str">
-        <v>Kmtia02g5y4cv</v>
+        <v>Kmti9zgfwe8ra</v>
       </c>
       <c r="B1812" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -69390,7 +69390,7 @@
     </row>
     <row r="1813">
       <c r="A1813" t="str">
-        <v>Kmtia02g5vd0v</v>
+        <v>Kmti9zgfwaj0c</v>
       </c>
       <c r="B1813" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -69428,7 +69428,7 @@
     </row>
     <row r="1814">
       <c r="A1814" t="str">
-        <v>Kmtia02g5u2cs</v>
+        <v>Kmti9zgfwvo49</v>
       </c>
       <c r="B1814" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -69542,7 +69542,7 @@
     </row>
     <row r="1817">
       <c r="A1817" t="str">
-        <v>Kmtia02g5fwmp</v>
+        <v>Kmti9zgfwjqwo</v>
       </c>
       <c r="B1817" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -69580,7 +69580,7 @@
     </row>
     <row r="1818">
       <c r="A1818" t="str">
-        <v>Kmtia02g5mhs7</v>
+        <v>Kmti9zgfwem78</v>
       </c>
       <c r="B1818" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -69618,7 +69618,7 @@
     </row>
     <row r="1819">
       <c r="A1819" t="str">
-        <v>Kmtia02g58hq9</v>
+        <v>Kmti9zgfw48hj</v>
       </c>
       <c r="B1819" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -69656,7 +69656,7 @@
     </row>
     <row r="1820">
       <c r="A1820" t="str">
-        <v>Kmtia02g5ucy1</v>
+        <v>Kmti9zgfwyiy6</v>
       </c>
       <c r="B1820" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -69694,7 +69694,7 @@
     </row>
     <row r="1821">
       <c r="A1821" t="str">
-        <v>Kmtia02g57urv</v>
+        <v>Kmti9zgfw4rmo</v>
       </c>
       <c r="B1821" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -69732,7 +69732,7 @@
     </row>
     <row r="1822">
       <c r="A1822" t="str">
-        <v>Kmtia02g570vk</v>
+        <v>Kmti9zgfwsdmd</v>
       </c>
       <c r="B1822" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -69808,7 +69808,7 @@
     </row>
     <row r="1824">
       <c r="A1824" t="str">
-        <v>Kmtia02g5dgnc</v>
+        <v>Kmti9zgfwhaic</v>
       </c>
       <c r="B1824" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -69846,7 +69846,7 @@
     </row>
     <row r="1825">
       <c r="A1825" t="str">
-        <v>Kmtia02g51x9j</v>
+        <v>Kmti9zgfwz66l</v>
       </c>
       <c r="B1825" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -69884,7 +69884,7 @@
     </row>
     <row r="1826">
       <c r="A1826" t="str">
-        <v>Kmtia02g58aiv</v>
+        <v>Kmti9zgfw2y2o</v>
       </c>
       <c r="B1826" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -69922,7 +69922,7 @@
     </row>
     <row r="1827">
       <c r="A1827" t="str">
-        <v>Kmtia02g5094l</v>
+        <v>Kmti9zgfwldzg</v>
       </c>
       <c r="B1827" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -69960,7 +69960,7 @@
     </row>
     <row r="1828">
       <c r="A1828" t="str">
-        <v>Kmtia02g5d1t4</v>
+        <v>Kmti9zgfwln2m</v>
       </c>
       <c r="B1828" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -69998,7 +69998,7 @@
     </row>
     <row r="1829">
       <c r="A1829" t="str">
-        <v>Kmtia02g57duk</v>
+        <v>Kmti9zgfw4fjz</v>
       </c>
       <c r="B1829" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -70036,7 +70036,7 @@
     </row>
     <row r="1830">
       <c r="A1830" t="str">
-        <v>Kmtia02g5awdb</v>
+        <v>Kmti9zgfwrcj7</v>
       </c>
       <c r="B1830" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -70112,7 +70112,7 @@
     </row>
     <row r="1832">
       <c r="A1832" t="str">
-        <v>Kmtia02g506h5</v>
+        <v>Kmti9zgfwwsyh</v>
       </c>
       <c r="B1832" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -70150,7 +70150,7 @@
     </row>
     <row r="1833">
       <c r="A1833" t="str">
-        <v>Kmtia02g5tgav</v>
+        <v>Kmti9zgfwtkvi</v>
       </c>
       <c r="B1833" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -70188,7 +70188,7 @@
     </row>
     <row r="1834">
       <c r="A1834" t="str">
-        <v>Kmtia02g53yk1</v>
+        <v>Kmti9zgfwv418</v>
       </c>
       <c r="B1834" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -70226,7 +70226,7 @@
     </row>
     <row r="1835">
       <c r="A1835" t="str">
-        <v>Kmtia02g5bnta</v>
+        <v>Kmti9zgfw5nyi</v>
       </c>
       <c r="B1835" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -70264,7 +70264,7 @@
     </row>
     <row r="1836">
       <c r="A1836" t="str">
-        <v>Kmtia02g50mv0</v>
+        <v>Kmti9zgfw36v4</v>
       </c>
       <c r="B1836" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -70302,7 +70302,7 @@
     </row>
     <row r="1837">
       <c r="A1837" t="str">
-        <v>Kmtia02g5en1j</v>
+        <v>Kmti9zgfwrhj9</v>
       </c>
       <c r="B1837" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -70340,7 +70340,7 @@
     </row>
     <row r="1838">
       <c r="A1838" t="str">
-        <v>Kmtia02g5wgv9</v>
+        <v>Kmti9zgfw9p5y</v>
       </c>
       <c r="B1838" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -70378,7 +70378,7 @@
     </row>
     <row r="1839">
       <c r="A1839" t="str">
-        <v>Kmtia02g52l3u</v>
+        <v>Kmti9zgfw7yh8</v>
       </c>
       <c r="B1839" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -70416,7 +70416,7 @@
     </row>
     <row r="1840">
       <c r="A1840" t="str">
-        <v>Kmtia02g5sr20</v>
+        <v>Kmti9zgfwytqd</v>
       </c>
       <c r="B1840" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -70454,7 +70454,7 @@
     </row>
     <row r="1841">
       <c r="A1841" t="str">
-        <v>Kmtia02g59eyb</v>
+        <v>Kmti9zgfwidk1</v>
       </c>
       <c r="B1841" t="str">
         <v xml:space="preserve">Pengawas Keuangan Negara Mahir </v>
@@ -70492,7 +70492,7 @@
     </row>
     <row r="1842">
       <c r="A1842" t="str">
-        <v>Kmtia02g5y8fb</v>
+        <v>Kmti9zgfw5qi3</v>
       </c>
       <c r="B1842" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -70568,7 +70568,7 @@
     </row>
     <row r="1844">
       <c r="A1844" t="str">
-        <v>Kmtia02g5mx3q</v>
+        <v>Kmti9zgfw7bm4</v>
       </c>
       <c r="B1844" t="str">
         <v>Penata Layanan Operasional</v>
@@ -70606,7 +70606,7 @@
     </row>
     <row r="1845">
       <c r="A1845" t="str">
-        <v>Kmtia02g5gv4c</v>
+        <v>Kmti9zgfwsvbt</v>
       </c>
       <c r="B1845" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -70644,7 +70644,7 @@
     </row>
     <row r="1846">
       <c r="A1846" t="str">
-        <v>Kmtia02g5mlx1</v>
+        <v>Kmti9zgfwg9f7</v>
       </c>
       <c r="B1846" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -70682,7 +70682,7 @@
     </row>
     <row r="1847">
       <c r="A1847" t="str">
-        <v>Kmtia02g52bdq</v>
+        <v>Kmti9zgfwwt6t</v>
       </c>
       <c r="B1847" t="str">
         <v>Pranata Humas Ahli Muda</v>
@@ -70720,7 +70720,7 @@
     </row>
     <row r="1848">
       <c r="A1848" t="str">
-        <v>Kmtia02g5seaj</v>
+        <v>Kmti9zgfwv7iq</v>
       </c>
       <c r="B1848" t="str">
         <v>Pranata Humas Ahli Pertama</v>
@@ -70758,7 +70758,7 @@
     </row>
     <row r="1849">
       <c r="A1849" t="str">
-        <v>Kmtia02g5blr7</v>
+        <v>Kmti9zgfwdkza</v>
       </c>
       <c r="B1849" t="str">
         <v>Pranata Humas Penyelia</v>
@@ -70796,7 +70796,7 @@
     </row>
     <row r="1850">
       <c r="A1850" t="str">
-        <v>Kmtia02g5p73l</v>
+        <v>Kmti9zgfwko74</v>
       </c>
       <c r="B1850" t="str">
         <v>Pranata Humas Mahir</v>
@@ -70834,7 +70834,7 @@
     </row>
     <row r="1851">
       <c r="A1851" t="str">
-        <v>Kmtia02g5zppp</v>
+        <v>Kmti9zgfwifm5</v>
       </c>
       <c r="B1851" t="str">
         <v>Pranata Humas Terampil</v>
@@ -70872,7 +70872,7 @@
     </row>
     <row r="1852">
       <c r="A1852" t="str">
-        <v>Kmtia02g5evqm</v>
+        <v>Kmti9zgfw8us7</v>
       </c>
       <c r="B1852" t="str">
         <v>Pustakawan Ahli Muda</v>
@@ -70910,7 +70910,7 @@
     </row>
     <row r="1853">
       <c r="A1853" t="str">
-        <v>Kmtia02g5sk81</v>
+        <v>Kmti9zgfwbumm</v>
       </c>
       <c r="B1853" t="str">
         <v>Pustakawan Ahli Pertama</v>
@@ -70948,7 +70948,7 @@
     </row>
     <row r="1854">
       <c r="A1854" t="str">
-        <v>Kmtia02g5847t</v>
+        <v>Kmti9zgfw2iij</v>
       </c>
       <c r="B1854" t="str">
         <v>Pustakawan Penyelia</v>
@@ -70986,7 +70986,7 @@
     </row>
     <row r="1855">
       <c r="A1855" t="str">
-        <v>Kmtia02g5esxu</v>
+        <v>Kmti9zgfwyyps</v>
       </c>
       <c r="B1855" t="str">
         <v>Pustakawan Mahir</v>
@@ -71024,7 +71024,7 @@
     </row>
     <row r="1856">
       <c r="A1856" t="str">
-        <v>Kmtia02g5xv9d</v>
+        <v>Kmti9zgfwjo3x</v>
       </c>
       <c r="B1856" t="str">
         <v>Pustakawan Terampil</v>
@@ -71138,7 +71138,7 @@
     </row>
     <row r="1859">
       <c r="A1859" t="str">
-        <v>Kmtia02g5751t</v>
+        <v>Kmti9zgfw0xyq</v>
       </c>
       <c r="B1859" t="str">
         <v>Penata Layanan Operasional</v>
@@ -71176,7 +71176,7 @@
     </row>
     <row r="1860">
       <c r="A1860" t="str">
-        <v>Kmtia02g5n6is</v>
+        <v>Kmti9zgfwe6ho</v>
       </c>
       <c r="B1860" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71214,7 +71214,7 @@
     </row>
     <row r="1861">
       <c r="A1861" t="str">
-        <v>Kmtia02g5jo1h</v>
+        <v>Kmti9zgfwfgw6</v>
       </c>
       <c r="B1861" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71252,7 +71252,7 @@
     </row>
     <row r="1862">
       <c r="A1862" t="str">
-        <v>Kmtia02g5fhzw</v>
+        <v>Kmti9zgfwla25</v>
       </c>
       <c r="B1862" t="str">
         <v>Penata Keprotokolan*</v>
@@ -71366,7 +71366,7 @@
     </row>
     <row r="1865">
       <c r="A1865" t="str">
-        <v>Kmtia02g52apj</v>
+        <v>Kmti9zgfw2nin</v>
       </c>
       <c r="B1865" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -71404,7 +71404,7 @@
     </row>
     <row r="1866">
       <c r="A1866" t="str">
-        <v>Kmtia02g51nt1</v>
+        <v>Kmti9zgfw7zit</v>
       </c>
       <c r="B1866" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71442,7 +71442,7 @@
     </row>
     <row r="1867">
       <c r="A1867" t="str">
-        <v>Kmtia02g543v3</v>
+        <v>Kmti9zgfwii39</v>
       </c>
       <c r="B1867" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71518,7 +71518,7 @@
     </row>
     <row r="1869">
       <c r="A1869" t="str">
-        <v>Kmtia02g5ufdv</v>
+        <v>Kmti9zgfwzuwq</v>
       </c>
       <c r="B1869" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -71556,7 +71556,7 @@
     </row>
     <row r="1870">
       <c r="A1870" t="str">
-        <v>Kmtia02g5h0pq</v>
+        <v>Kmti9zgfwlnqc</v>
       </c>
       <c r="B1870" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71594,7 +71594,7 @@
     </row>
     <row r="1871">
       <c r="A1871" t="str">
-        <v>Kmtia02g52i5g</v>
+        <v>Kmti9zgfwp5sv</v>
       </c>
       <c r="B1871" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71632,7 +71632,7 @@
     </row>
     <row r="1872" xml:space="preserve">
       <c r="A1872" t="str">
-        <v>Kmtia02g5arra</v>
+        <v>Kmti9zgfw0ds4</v>
       </c>
       <c r="B1872" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -71671,7 +71671,7 @@
     </row>
     <row r="1873" xml:space="preserve">
       <c r="A1873" t="str">
-        <v>Kmtia02g5vqpj</v>
+        <v>Kmti9zgfwa6fc</v>
       </c>
       <c r="B1873" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -71710,7 +71710,7 @@
     </row>
     <row r="1874" xml:space="preserve">
       <c r="A1874" t="str">
-        <v>Kmtia02g5dw28</v>
+        <v>Kmti9zgfwajv1</v>
       </c>
       <c r="B1874" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -71749,7 +71749,7 @@
     </row>
     <row r="1875" xml:space="preserve">
       <c r="A1875" t="str">
-        <v>Kmtia02g50kef</v>
+        <v>Kmti9zgfwc10z</v>
       </c>
       <c r="B1875" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -71864,7 +71864,7 @@
     </row>
     <row r="1878">
       <c r="A1878" t="str">
-        <v>Kmtia02g5xkth</v>
+        <v>Kmti9zgfwygzd</v>
       </c>
       <c r="B1878" t="str">
         <v>Penata Layanan Operasional</v>
@@ -71902,7 +71902,7 @@
     </row>
     <row r="1879">
       <c r="A1879" t="str">
-        <v>Kmtia02g5w1p4</v>
+        <v>Kmti9zgfwoltt</v>
       </c>
       <c r="B1879" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -71940,7 +71940,7 @@
     </row>
     <row r="1880">
       <c r="A1880" t="str">
-        <v>Kmtia02g5emrb</v>
+        <v>Kmti9zgfwqkai</v>
       </c>
       <c r="B1880" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -71978,7 +71978,7 @@
     </row>
     <row r="1881">
       <c r="A1881" t="str">
-        <v>Kmtia02g5jwg2</v>
+        <v>Kmti9zgfwypfl</v>
       </c>
       <c r="B1881" t="str">
         <v>Penata Keprotokolan*</v>
@@ -72092,7 +72092,7 @@
     </row>
     <row r="1884">
       <c r="A1884" t="str">
-        <v>Kmtia02g5rr92</v>
+        <v>Kmti9zgfwhczd</v>
       </c>
       <c r="B1884" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -72130,7 +72130,7 @@
     </row>
     <row r="1885">
       <c r="A1885" t="str">
-        <v>Kmtia02g5z6a2</v>
+        <v>Kmti9zgfw7qoi</v>
       </c>
       <c r="B1885" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72168,7 +72168,7 @@
     </row>
     <row r="1886">
       <c r="A1886" t="str">
-        <v>Kmtia02g5c1v6</v>
+        <v>Kmti9zgfwb0ne</v>
       </c>
       <c r="B1886" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72244,7 +72244,7 @@
     </row>
     <row r="1888">
       <c r="A1888" t="str">
-        <v>Kmtia02g5yd27</v>
+        <v>Kmti9zgfwonwb</v>
       </c>
       <c r="B1888" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -72282,7 +72282,7 @@
     </row>
     <row r="1889">
       <c r="A1889" t="str">
-        <v>Kmtia02g5sdjj</v>
+        <v>Kmti9zgfwmcx1</v>
       </c>
       <c r="B1889" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72320,7 +72320,7 @@
     </row>
     <row r="1890">
       <c r="A1890" t="str">
-        <v>Kmtia02g5rlp6</v>
+        <v>Kmti9zgfwvgey</v>
       </c>
       <c r="B1890" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72358,7 +72358,7 @@
     </row>
     <row r="1891" xml:space="preserve">
       <c r="A1891" t="str">
-        <v>Kmtia02g5gw3m</v>
+        <v>Kmti9zgfwhsjl</v>
       </c>
       <c r="B1891" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -72397,7 +72397,7 @@
     </row>
     <row r="1892" xml:space="preserve">
       <c r="A1892" t="str">
-        <v>Kmtia02g5ycyf</v>
+        <v>Kmti9zgfwz45u</v>
       </c>
       <c r="B1892" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -72436,7 +72436,7 @@
     </row>
     <row r="1893" xml:space="preserve">
       <c r="A1893" t="str">
-        <v>Kmtia02g5xp44</v>
+        <v>Kmti9zgfwkdjf</v>
       </c>
       <c r="B1893" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -72475,7 +72475,7 @@
     </row>
     <row r="1894" xml:space="preserve">
       <c r="A1894" t="str">
-        <v>Kmtia02g5po7x</v>
+        <v>Kmti9zgfwqky1</v>
       </c>
       <c r="B1894" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -72590,7 +72590,7 @@
     </row>
     <row r="1897">
       <c r="A1897" t="str">
-        <v>Kmtia02g5jnvm</v>
+        <v>Kmti9zgfwdg9m</v>
       </c>
       <c r="B1897" t="str">
         <v>Penata Layanan Operasional</v>
@@ -72628,7 +72628,7 @@
     </row>
     <row r="1898">
       <c r="A1898" t="str">
-        <v>Kmtia02g5tu8l</v>
+        <v>Kmti9zgfw93o7</v>
       </c>
       <c r="B1898" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72666,7 +72666,7 @@
     </row>
     <row r="1899">
       <c r="A1899" t="str">
-        <v>Kmtia02g59zte</v>
+        <v>Kmti9zgfw3rvs</v>
       </c>
       <c r="B1899" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72704,7 +72704,7 @@
     </row>
     <row r="1900">
       <c r="A1900" t="str">
-        <v>Kmtia02g54rf9</v>
+        <v>Kmti9zgfwaiyz</v>
       </c>
       <c r="B1900" t="str">
         <v>Penata Keprotokolan*</v>
@@ -72818,7 +72818,7 @@
     </row>
     <row r="1903">
       <c r="A1903" t="str">
-        <v>Kmtia02g5eucu</v>
+        <v>Kmti9zgfwqae2</v>
       </c>
       <c r="B1903" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -72856,7 +72856,7 @@
     </row>
     <row r="1904">
       <c r="A1904" t="str">
-        <v>Kmtia02g5xv40</v>
+        <v>Kmti9zgfwd4z6</v>
       </c>
       <c r="B1904" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -72894,7 +72894,7 @@
     </row>
     <row r="1905">
       <c r="A1905" t="str">
-        <v>Kmtia02g5tio4</v>
+        <v>Kmti9zgfw2ujl</v>
       </c>
       <c r="B1905" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -72970,7 +72970,7 @@
     </row>
     <row r="1907">
       <c r="A1907" t="str">
-        <v>Kmtia02g52b6t</v>
+        <v>Kmti9zgfw9m04</v>
       </c>
       <c r="B1907" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -73008,7 +73008,7 @@
     </row>
     <row r="1908">
       <c r="A1908" t="str">
-        <v>Kmtia02g5xi3c</v>
+        <v>Kmti9zgfwx768</v>
       </c>
       <c r="B1908" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73046,7 +73046,7 @@
     </row>
     <row r="1909">
       <c r="A1909" t="str">
-        <v>Kmtia02g5ju1t</v>
+        <v>Kmti9zgfwvkwj</v>
       </c>
       <c r="B1909" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73084,7 +73084,7 @@
     </row>
     <row r="1910" xml:space="preserve">
       <c r="A1910" t="str">
-        <v>Kmtia02g5j8e4</v>
+        <v>Kmti9zgfw6b8v</v>
       </c>
       <c r="B1910" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -73123,7 +73123,7 @@
     </row>
     <row r="1911" xml:space="preserve">
       <c r="A1911" t="str">
-        <v>Kmtia02g5lo7f</v>
+        <v>Kmti9zgfwsy1c</v>
       </c>
       <c r="B1911" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -73162,7 +73162,7 @@
     </row>
     <row r="1912" xml:space="preserve">
       <c r="A1912" t="str">
-        <v>Kmtia02g54w5v</v>
+        <v>Kmti9zgfw5kvp</v>
       </c>
       <c r="B1912" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -73201,7 +73201,7 @@
     </row>
     <row r="1913" xml:space="preserve">
       <c r="A1913" t="str">
-        <v>Kmtia02g5tsmj</v>
+        <v>Kmti9zgfwz84e</v>
       </c>
       <c r="B1913" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -73316,7 +73316,7 @@
     </row>
     <row r="1916">
       <c r="A1916" t="str">
-        <v>Kmtia02g67x9r</v>
+        <v>Kmti9zgfwbw3m</v>
       </c>
       <c r="B1916" t="str">
         <v>Penata Layanan Operasional</v>
@@ -73354,7 +73354,7 @@
     </row>
     <row r="1917">
       <c r="A1917" t="str">
-        <v>Kmtia02g6l4mu</v>
+        <v>Kmti9zgfwkfny</v>
       </c>
       <c r="B1917" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73392,7 +73392,7 @@
     </row>
     <row r="1918">
       <c r="A1918" t="str">
-        <v>Kmtia02g6fhzw</v>
+        <v>Kmti9zgfwcyo6</v>
       </c>
       <c r="B1918" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73430,7 +73430,7 @@
     </row>
     <row r="1919">
       <c r="A1919" t="str">
-        <v>Kmtia02g6xz2g</v>
+        <v>Kmti9zgfw0tnz</v>
       </c>
       <c r="B1919" t="str">
         <v>Penata Keprotokolan*</v>
@@ -73544,7 +73544,7 @@
     </row>
     <row r="1922">
       <c r="A1922" t="str">
-        <v>Kmtia02g6mfnb</v>
+        <v>Kmti9zgfwltys</v>
       </c>
       <c r="B1922" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -73582,7 +73582,7 @@
     </row>
     <row r="1923">
       <c r="A1923" t="str">
-        <v>Kmtia02g6sda7</v>
+        <v>Kmti9zgfwlv3o</v>
       </c>
       <c r="B1923" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73620,7 +73620,7 @@
     </row>
     <row r="1924">
       <c r="A1924" t="str">
-        <v>Kmtia02g6m9u1</v>
+        <v>Kmti9zgfwjioh</v>
       </c>
       <c r="B1924" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73696,7 +73696,7 @@
     </row>
     <row r="1926">
       <c r="A1926" t="str">
-        <v>Kmtia02g6uvuq</v>
+        <v>Kmti9zgfw06pe</v>
       </c>
       <c r="B1926" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -73734,7 +73734,7 @@
     </row>
     <row r="1927">
       <c r="A1927" t="str">
-        <v>Kmtia02g65myt</v>
+        <v>Kmti9zgfwuj6q</v>
       </c>
       <c r="B1927" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -73772,7 +73772,7 @@
     </row>
     <row r="1928">
       <c r="A1928" t="str">
-        <v>Kmtia02g6oiwu</v>
+        <v>Kmti9zgfw033o</v>
       </c>
       <c r="B1928" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -73810,7 +73810,7 @@
     </row>
     <row r="1929" xml:space="preserve">
       <c r="A1929" t="str">
-        <v>Kmtia02g6s09i</v>
+        <v>Kmti9zgfwjjey</v>
       </c>
       <c r="B1929" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -73849,7 +73849,7 @@
     </row>
     <row r="1930" xml:space="preserve">
       <c r="A1930" t="str">
-        <v>Kmtia02g6x36c</v>
+        <v>Kmti9zgfwnnpn</v>
       </c>
       <c r="B1930" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -73888,7 +73888,7 @@
     </row>
     <row r="1931" xml:space="preserve">
       <c r="A1931" t="str">
-        <v>Kmtia02g6x3zw</v>
+        <v>Kmti9zgfw6gap</v>
       </c>
       <c r="B1931" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -73927,7 +73927,7 @@
     </row>
     <row r="1932" xml:space="preserve">
       <c r="A1932" t="str">
-        <v>Kmtia02g6iuxz</v>
+        <v>Kmti9zgfwoabt</v>
       </c>
       <c r="B1932" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -73966,7 +73966,7 @@
     </row>
     <row r="1933" xml:space="preserve">
       <c r="A1933" t="str">
-        <v>Kmtia02g6rzrv</v>
+        <v>Kmti9zgfww5t6</v>
       </c>
       <c r="B1933" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Madya/_x000d_
@@ -74005,7 +74005,7 @@
     </row>
     <row r="1934" xml:space="preserve">
       <c r="A1934" t="str">
-        <v>Kmtia02g68m2x</v>
+        <v>Kmti9zgfwyfcf</v>
       </c>
       <c r="B1934" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -74044,7 +74044,7 @@
     </row>
     <row r="1935" xml:space="preserve">
       <c r="A1935" t="str">
-        <v>Kmtia02g6b66o</v>
+        <v>Kmti9zgfw2bzn</v>
       </c>
       <c r="B1935" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -74159,7 +74159,7 @@
     </row>
     <row r="1938">
       <c r="A1938" t="str">
-        <v>Kmtia02g6ix1r</v>
+        <v>Kmti9zgfwe6jk</v>
       </c>
       <c r="B1938" t="str">
         <v>Penata Layanan Operasional</v>
@@ -74197,7 +74197,7 @@
     </row>
     <row r="1939">
       <c r="A1939" t="str">
-        <v>Kmtia02g6bevy</v>
+        <v>Kmti9zgfwnr3v</v>
       </c>
       <c r="B1939" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -74235,7 +74235,7 @@
     </row>
     <row r="1940">
       <c r="A1940" t="str">
-        <v>Kmtia02g6gfob</v>
+        <v>Kmti9zgfw1j05</v>
       </c>
       <c r="B1940" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -74273,7 +74273,7 @@
     </row>
     <row r="1941">
       <c r="A1941" t="str">
-        <v>Kmtia02g69792</v>
+        <v>Kmti9zgfw5rbq</v>
       </c>
       <c r="B1941" t="str">
         <v>Penata Keprotokolan*</v>
@@ -74387,7 +74387,7 @@
     </row>
     <row r="1944">
       <c r="A1944" t="str">
-        <v>Kmtia02g634r5</v>
+        <v>Kmti9zgfwfb0h</v>
       </c>
       <c r="B1944" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -74425,7 +74425,7 @@
     </row>
     <row r="1945">
       <c r="A1945" t="str">
-        <v>Kmtia02g69to5</v>
+        <v>Kmti9zgfw1aqi</v>
       </c>
       <c r="B1945" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -74463,7 +74463,7 @@
     </row>
     <row r="1946">
       <c r="A1946" t="str">
-        <v>Kmtia02g6j9iw</v>
+        <v>Kmti9zgfwxvsl</v>
       </c>
       <c r="B1946" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -74539,7 +74539,7 @@
     </row>
     <row r="1948">
       <c r="A1948" t="str">
-        <v>Kmtia02g6yxsa</v>
+        <v>Kmti9zgfwixeo</v>
       </c>
       <c r="B1948" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -74577,7 +74577,7 @@
     </row>
     <row r="1949">
       <c r="A1949" t="str">
-        <v>Kmtia02g6c24a</v>
+        <v>Kmti9zgfwztsm</v>
       </c>
       <c r="B1949" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -74615,7 +74615,7 @@
     </row>
     <row r="1950">
       <c r="A1950" t="str">
-        <v>Kmtia02g6uyjx</v>
+        <v>Kmti9zgfwjky0</v>
       </c>
       <c r="B1950" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -74653,7 +74653,7 @@
     </row>
     <row r="1951" xml:space="preserve">
       <c r="A1951" t="str">
-        <v>Kmtia02g60w4t</v>
+        <v>Kmti9zgfwql8b</v>
       </c>
       <c r="B1951" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -74692,7 +74692,7 @@
     </row>
     <row r="1952" xml:space="preserve">
       <c r="A1952" t="str">
-        <v>Kmtia02g6jo7p</v>
+        <v>Kmti9zgfwb0ad</v>
       </c>
       <c r="B1952" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -74731,7 +74731,7 @@
     </row>
     <row r="1953" xml:space="preserve">
       <c r="A1953" t="str">
-        <v>Kmtia02g6zxp9</v>
+        <v>Kmti9zgfwr31d</v>
       </c>
       <c r="B1953" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -74770,7 +74770,7 @@
     </row>
     <row r="1954" xml:space="preserve">
       <c r="A1954" t="str">
-        <v>Kmtia02g64hhx</v>
+        <v>Kmti9zgfwr8in</v>
       </c>
       <c r="B1954" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -74809,7 +74809,7 @@
     </row>
     <row r="1955" xml:space="preserve">
       <c r="A1955" t="str">
-        <v>Kmtia02g6vv0j</v>
+        <v>Kmti9zgfwtaz2</v>
       </c>
       <c r="B1955" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Madya/_x000d_
@@ -74848,7 +74848,7 @@
     </row>
     <row r="1956" xml:space="preserve">
       <c r="A1956" t="str">
-        <v>Kmtia02g6i9p7</v>
+        <v>Kmti9zgfwqbyo</v>
       </c>
       <c r="B1956" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Muda/_x000d_
@@ -74887,7 +74887,7 @@
     </row>
     <row r="1957" xml:space="preserve">
       <c r="A1957" t="str">
-        <v>Kmtia02g6t9dv</v>
+        <v>Kmti9zgfw8hv9</v>
       </c>
       <c r="B1957" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Pengelolaan Keuangan APBN Ahli Pertama/_x000d_
@@ -75002,7 +75002,7 @@
     </row>
     <row r="1960">
       <c r="A1960" t="str">
-        <v>Kmtia02g6fz4z</v>
+        <v>Kmti9zgfwct15</v>
       </c>
       <c r="B1960" t="str">
         <v>Penata Layanan Operasional</v>
@@ -75040,7 +75040,7 @@
     </row>
     <row r="1961">
       <c r="A1961" t="str">
-        <v>Kmtia02g66nrd</v>
+        <v>Kmti9zgfwa9hm</v>
       </c>
       <c r="B1961" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75078,7 +75078,7 @@
     </row>
     <row r="1962">
       <c r="A1962" t="str">
-        <v>Kmtia02g6jop0</v>
+        <v>Kmti9zgfwlm30</v>
       </c>
       <c r="B1962" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75116,7 +75116,7 @@
     </row>
     <row r="1963">
       <c r="A1963" t="str">
-        <v>Kmtia02g6klnl</v>
+        <v>Kmti9zgfwqbvg</v>
       </c>
       <c r="B1963" t="str">
         <v>Penata Keprotokolan*</v>
@@ -75230,7 +75230,7 @@
     </row>
     <row r="1966">
       <c r="A1966" t="str">
-        <v>Kmtia02g6ov06</v>
+        <v>Kmti9zgfws9sa</v>
       </c>
       <c r="B1966" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -75268,7 +75268,7 @@
     </row>
     <row r="1967">
       <c r="A1967" t="str">
-        <v>Kmtia02g6yv4s</v>
+        <v>Kmti9zgfwash5</v>
       </c>
       <c r="B1967" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75306,7 +75306,7 @@
     </row>
     <row r="1968">
       <c r="A1968" t="str">
-        <v>Kmtia02g6kky4</v>
+        <v>Kmti9zgfwquo0</v>
       </c>
       <c r="B1968" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75382,7 +75382,7 @@
     </row>
     <row r="1970">
       <c r="A1970" t="str">
-        <v>Kmtia02g6cqkx</v>
+        <v>Kmti9zgfwup3i</v>
       </c>
       <c r="B1970" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -75420,7 +75420,7 @@
     </row>
     <row r="1971">
       <c r="A1971" t="str">
-        <v>Kmtia02g6q0vj</v>
+        <v>Kmti9zgfwef5s</v>
       </c>
       <c r="B1971" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75458,7 +75458,7 @@
     </row>
     <row r="1972">
       <c r="A1972" t="str">
-        <v>Kmtia02g6mn3p</v>
+        <v>Kmti9zgfwwtwu</v>
       </c>
       <c r="B1972" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75496,7 +75496,7 @@
     </row>
     <row r="1973" xml:space="preserve">
       <c r="A1973" t="str">
-        <v>Kmtia02g6gtj3</v>
+        <v>Kmti9zgfw75iy</v>
       </c>
       <c r="B1973" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -75535,7 +75535,7 @@
     </row>
     <row r="1974" xml:space="preserve">
       <c r="A1974" t="str">
-        <v>Kmtia02g61exi</v>
+        <v>Kmti9zgfwt3u7</v>
       </c>
       <c r="B1974" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -75574,7 +75574,7 @@
     </row>
     <row r="1975" xml:space="preserve">
       <c r="A1975" t="str">
-        <v>Kmtia02g6dxfe</v>
+        <v>Kmti9zgfwetaa</v>
       </c>
       <c r="B1975" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -75613,7 +75613,7 @@
     </row>
     <row r="1976" xml:space="preserve">
       <c r="A1976" t="str">
-        <v>Kmtia02g6ubih</v>
+        <v>Kmti9zgfwckqd</v>
       </c>
       <c r="B1976" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -75728,7 +75728,7 @@
     </row>
     <row r="1979">
       <c r="A1979" t="str">
-        <v>Kmtia02g6t1vj</v>
+        <v>Kmti9zgfwvci0</v>
       </c>
       <c r="B1979" t="str">
         <v>Penata Layanan Operasional</v>
@@ -75766,7 +75766,7 @@
     </row>
     <row r="1980">
       <c r="A1980" t="str">
-        <v>Kmtia02g6vjq0</v>
+        <v>Kmti9zgfw7psj</v>
       </c>
       <c r="B1980" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -75804,7 +75804,7 @@
     </row>
     <row r="1981">
       <c r="A1981" t="str">
-        <v>Kmtia02g6o1h4</v>
+        <v>Kmti9zgfw0gqv</v>
       </c>
       <c r="B1981" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -75842,7 +75842,7 @@
     </row>
     <row r="1982">
       <c r="A1982" t="str">
-        <v>Kmtia02g6ufxj</v>
+        <v>Kmti9zgfw1kr2</v>
       </c>
       <c r="B1982" t="str">
         <v>Penata Keprotokolan*</v>
@@ -75956,7 +75956,7 @@
     </row>
     <row r="1985">
       <c r="A1985" t="str">
-        <v>Kmtia02g6eqwo</v>
+        <v>Kmti9zgfwryyh</v>
       </c>
       <c r="B1985" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -75994,7 +75994,7 @@
     </row>
     <row r="1986">
       <c r="A1986" t="str">
-        <v>Kmtia02g656ap</v>
+        <v>Kmti9zgfwff1h</v>
       </c>
       <c r="B1986" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76032,7 +76032,7 @@
     </row>
     <row r="1987">
       <c r="A1987" t="str">
-        <v>Kmtia02g62ruv</v>
+        <v>Kmti9zgfw6v3w</v>
       </c>
       <c r="B1987" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76108,7 +76108,7 @@
     </row>
     <row r="1989">
       <c r="A1989" t="str">
-        <v>Kmtia02g6f242</v>
+        <v>Kmti9zgfw9zoj</v>
       </c>
       <c r="B1989" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -76146,7 +76146,7 @@
     </row>
     <row r="1990">
       <c r="A1990" t="str">
-        <v>Kmtia02g6bh6y</v>
+        <v>Kmti9zgfwyso0</v>
       </c>
       <c r="B1990" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76184,7 +76184,7 @@
     </row>
     <row r="1991">
       <c r="A1991" t="str">
-        <v>Kmtia02g6tcdt</v>
+        <v>Kmti9zgfwugsv</v>
       </c>
       <c r="B1991" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76222,7 +76222,7 @@
     </row>
     <row r="1992" xml:space="preserve">
       <c r="A1992" t="str">
-        <v>Kmtia02g6qn01</v>
+        <v>Kmti9zgfw6fhy</v>
       </c>
       <c r="B1992" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -76261,7 +76261,7 @@
     </row>
     <row r="1993" xml:space="preserve">
       <c r="A1993" t="str">
-        <v>Kmtia02g690ph</v>
+        <v>Kmti9zgfwexxz</v>
       </c>
       <c r="B1993" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -76300,7 +76300,7 @@
     </row>
     <row r="1994" xml:space="preserve">
       <c r="A1994" t="str">
-        <v>Kmtia02g63qre</v>
+        <v>Kmti9zgfwx8ig</v>
       </c>
       <c r="B1994" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -76339,7 +76339,7 @@
     </row>
     <row r="1995" xml:space="preserve">
       <c r="A1995" t="str">
-        <v>Kmtia02g69f8a</v>
+        <v>Kmti9zgfwt7iw</v>
       </c>
       <c r="B1995" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -76454,7 +76454,7 @@
     </row>
     <row r="1998">
       <c r="A1998" t="str">
-        <v>Kmtia02g66bb0</v>
+        <v>Kmti9zgfw4cxt</v>
       </c>
       <c r="B1998" t="str">
         <v>Penata Layanan Operasional</v>
@@ -76492,7 +76492,7 @@
     </row>
     <row r="1999">
       <c r="A1999" t="str">
-        <v>Kmtia02g6cgaj</v>
+        <v>Kmti9zgfwxx46</v>
       </c>
       <c r="B1999" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76530,7 +76530,7 @@
     </row>
     <row r="2000">
       <c r="A2000" t="str">
-        <v>Kmtia02g6wnsc</v>
+        <v>Kmti9zgfwdx4b</v>
       </c>
       <c r="B2000" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76568,7 +76568,7 @@
     </row>
     <row r="2001">
       <c r="A2001" t="str">
-        <v>Kmtia02g6wqz2</v>
+        <v>Kmti9zgfwuima</v>
       </c>
       <c r="B2001" t="str">
         <v>Penata Keprotokolan*</v>
@@ -76682,7 +76682,7 @@
     </row>
     <row r="2004">
       <c r="A2004" t="str">
-        <v>Kmtia02g6vn1p</v>
+        <v>Kmti9zgfwtjyt</v>
       </c>
       <c r="B2004" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -76720,7 +76720,7 @@
     </row>
     <row r="2005">
       <c r="A2005" t="str">
-        <v>Kmtia02g6lyqk</v>
+        <v>Kmti9zgfx25jb</v>
       </c>
       <c r="B2005" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76758,7 +76758,7 @@
     </row>
     <row r="2006">
       <c r="A2006" t="str">
-        <v>Kmtia02g67sbl</v>
+        <v>Kmti9zgfxvr5x</v>
       </c>
       <c r="B2006" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76834,7 +76834,7 @@
     </row>
     <row r="2008">
       <c r="A2008" t="str">
-        <v>Kmtia02g6wg95</v>
+        <v>Kmti9zgfx60nq</v>
       </c>
       <c r="B2008" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -76872,7 +76872,7 @@
     </row>
     <row r="2009">
       <c r="A2009" t="str">
-        <v>Kmtia02g6tyo0</v>
+        <v>Kmti9zgfx5fvs</v>
       </c>
       <c r="B2009" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -76910,7 +76910,7 @@
     </row>
     <row r="2010">
       <c r="A2010" t="str">
-        <v>Kmtia02g6j3y3</v>
+        <v>Kmti9zgfx8g5q</v>
       </c>
       <c r="B2010" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -76948,7 +76948,7 @@
     </row>
     <row r="2011" xml:space="preserve">
       <c r="A2011" t="str">
-        <v>Kmtia02g6ftgs</v>
+        <v>Kmti9zgfxshjn</v>
       </c>
       <c r="B2011" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -76987,7 +76987,7 @@
     </row>
     <row r="2012" xml:space="preserve">
       <c r="A2012" t="str">
-        <v>Kmtia02g6iwfs</v>
+        <v>Kmti9zgfxrkcb</v>
       </c>
       <c r="B2012" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -77026,7 +77026,7 @@
     </row>
     <row r="2013" xml:space="preserve">
       <c r="A2013" t="str">
-        <v>Kmtia02g6ij3d</v>
+        <v>Kmti9zgfx1osk</v>
       </c>
       <c r="B2013" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -77065,7 +77065,7 @@
     </row>
     <row r="2014" xml:space="preserve">
       <c r="A2014" t="str">
-        <v>Kmtia02g61wcy</v>
+        <v>Kmti9zgfx01sb</v>
       </c>
       <c r="B2014" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -77180,7 +77180,7 @@
     </row>
     <row r="2017">
       <c r="A2017" t="str">
-        <v>Kmtia02g6jmi4</v>
+        <v>Kmti9zgfxxidv</v>
       </c>
       <c r="B2017" t="str">
         <v>Penata Layanan Operasional</v>
@@ -77218,7 +77218,7 @@
     </row>
     <row r="2018">
       <c r="A2018" t="str">
-        <v>Kmtia02g6ivzc</v>
+        <v>Kmti9zgfxnyrh</v>
       </c>
       <c r="B2018" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -77256,7 +77256,7 @@
     </row>
     <row r="2019">
       <c r="A2019" t="str">
-        <v>Kmtia02g65mjt</v>
+        <v>Kmti9zgfxvb34</v>
       </c>
       <c r="B2019" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -77294,7 +77294,7 @@
     </row>
     <row r="2020">
       <c r="A2020" t="str">
-        <v>Kmtia02g6f6p9</v>
+        <v>Kmti9zgfxoj9b</v>
       </c>
       <c r="B2020" t="str">
         <v>Penata Keprotokolan*</v>
@@ -77408,7 +77408,7 @@
     </row>
     <row r="2023">
       <c r="A2023" t="str">
-        <v>Kmtia02g65q8m</v>
+        <v>Kmti9zgfxkbvv</v>
       </c>
       <c r="B2023" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -77446,7 +77446,7 @@
     </row>
     <row r="2024">
       <c r="A2024" t="str">
-        <v>Kmtia02g62e4f</v>
+        <v>Kmti9zgfxhm06</v>
       </c>
       <c r="B2024" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -77484,7 +77484,7 @@
     </row>
     <row r="2025">
       <c r="A2025" t="str">
-        <v>Kmtia02g6azc8</v>
+        <v>Kmti9zgfx63dk</v>
       </c>
       <c r="B2025" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -77560,7 +77560,7 @@
     </row>
     <row r="2027">
       <c r="A2027" t="str">
-        <v>Kmtia02g6w5gk</v>
+        <v>Kmti9zgfxupom</v>
       </c>
       <c r="B2027" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -77598,7 +77598,7 @@
     </row>
     <row r="2028">
       <c r="A2028" t="str">
-        <v>Kmtia02g6on0i</v>
+        <v>Kmti9zgfxovu8</v>
       </c>
       <c r="B2028" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -77636,7 +77636,7 @@
     </row>
     <row r="2029">
       <c r="A2029" t="str">
-        <v>Kmtia02g6f17q</v>
+        <v>Kmti9zgfxwy6o</v>
       </c>
       <c r="B2029" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -77674,7 +77674,7 @@
     </row>
     <row r="2030" xml:space="preserve">
       <c r="A2030" t="str">
-        <v>Kmtia02g6202h</v>
+        <v>Kmti9zgfxflrx</v>
       </c>
       <c r="B2030" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_
@@ -77713,7 +77713,7 @@
     </row>
     <row r="2031" xml:space="preserve">
       <c r="A2031" t="str">
-        <v>Kmtia02g6cj3j</v>
+        <v>Kmti9zgfxc1b3</v>
       </c>
       <c r="B2031" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Madya/_x000d_
@@ -77752,7 +77752,7 @@
     </row>
     <row r="2032" xml:space="preserve">
       <c r="A2032" t="str">
-        <v>Kmtia02g6cz8d</v>
+        <v>Kmti9zgfxt41q</v>
       </c>
       <c r="B2032" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Muda/_x000d_
@@ -77791,7 +77791,7 @@
     </row>
     <row r="2033" xml:space="preserve">
       <c r="A2033" t="str">
-        <v>Kmtia02g6wjtm</v>
+        <v>Kmti9zgfxiwy8</v>
       </c>
       <c r="B2033" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Pertama/_x000d_
@@ -77830,7 +77830,7 @@
     </row>
     <row r="2034">
       <c r="A2034" t="str">
-        <v>Kmtia02g68p82</v>
+        <v>Kmti9zgfxmdk5</v>
       </c>
       <c r="B2034" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Muda</v>
@@ -77868,7 +77868,7 @@
     </row>
     <row r="2035">
       <c r="A2035" t="str">
-        <v>Kmtia02g6mn0u</v>
+        <v>Kmti9zgfxvt2x</v>
       </c>
       <c r="B2035" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Pertama</v>
@@ -77944,7 +77944,7 @@
     </row>
     <row r="2037" xml:space="preserve">
       <c r="A2037" t="str">
-        <v>Kmtia02g6u0rs</v>
+        <v>Kmti9zgfxcf89</v>
       </c>
       <c r="B2037" t="str" xml:space="preserve">
         <v xml:space="preserve">Analis Anggaran Ahli Utama/_x000d_

</xml_diff>